<commit_message>
Moved location of scc
</commit_message>
<xml_diff>
--- a/LOC tracking outputs/code_metrics.xlsx
+++ b/LOC tracking outputs/code_metrics.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -865,6 +865,56 @@
         <v>10739</v>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2024-11-25</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>40224</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" t="n">
+        <v>2643</v>
+      </c>
+      <c r="G18" t="n">
+        <v>10739</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2024-11-25</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>40224</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" t="n">
+        <v>2643</v>
+      </c>
+      <c r="G19" t="n">
+        <v>10739</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
SCC moved from linux
</commit_message>
<xml_diff>
--- a/LOC tracking outputs/code_metrics.xlsx
+++ b/LOC tracking outputs/code_metrics.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -615,6 +615,56 @@
         <v>6</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2024-11-26</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>828</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>780</v>
+      </c>
+      <c r="G8" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2024-11-26</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>828</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="n">
+        <v>780</v>
+      </c>
+      <c r="G9" t="n">
+        <v>48</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fixed data directory issues and fixed code counter
</commit_message>
<xml_diff>
--- a/LOC tracking outputs/code_metrics.xlsx
+++ b/LOC tracking outputs/code_metrics.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -665,6 +665,31 @@
         <v>48</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2024-11-26</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>866</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>860</v>
+      </c>
+      <c r="G10" t="n">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fully working code counter using the counter extension
</commit_message>
<xml_diff>
--- a/LOC tracking outputs/code_metrics.xlsx
+++ b/LOC tracking outputs/code_metrics.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,11 +468,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2024-11-25</t>
+          <t>2024-12-12</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>701</v>
+        <v>8606</v>
       </c>
       <c r="C2" t="n">
         <v>0</v>
@@ -484,20 +484,20 @@
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>695</v>
+        <v>2605</v>
       </c>
       <c r="G2" t="n">
-        <v>6</v>
+        <v>6001</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2024-11-25</t>
+          <t>2024-12-12 10:10:11</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>701</v>
+        <v>8606</v>
       </c>
       <c r="C3" t="n">
         <v>0</v>
@@ -509,20 +509,20 @@
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>695</v>
+        <v>2605</v>
       </c>
       <c r="G3" t="n">
-        <v>6</v>
+        <v>6001</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2024-11-25</t>
+          <t>2024-12-12 10:10:11</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>701</v>
+        <v>8606</v>
       </c>
       <c r="C4" t="n">
         <v>0</v>
@@ -534,20 +534,20 @@
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>695</v>
+        <v>2605</v>
       </c>
       <c r="G4" t="n">
-        <v>6</v>
+        <v>6001</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2024-11-25</t>
+          <t>2024-12-12 10:10:11</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>701</v>
+        <v>8606</v>
       </c>
       <c r="C5" t="n">
         <v>0</v>
@@ -559,20 +559,20 @@
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>695</v>
+        <v>2605</v>
       </c>
       <c r="G5" t="n">
-        <v>6</v>
+        <v>6001</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2024-11-25</t>
+          <t>2024-12-12 10:10:11</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>731</v>
+        <v>8606</v>
       </c>
       <c r="C6" t="n">
         <v>0</v>
@@ -584,20 +584,20 @@
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>725</v>
+        <v>2605</v>
       </c>
       <c r="G6" t="n">
-        <v>6</v>
+        <v>6001</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2024-11-25</t>
+          <t>2024-12-12 10:10:11</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>783</v>
+        <v>8606</v>
       </c>
       <c r="C7" t="n">
         <v>0</v>
@@ -609,20 +609,20 @@
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>777</v>
+        <v>2605</v>
       </c>
       <c r="G7" t="n">
-        <v>6</v>
+        <v>6001</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2024-11-26</t>
+          <t>2024-12-12 10:10:11</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>828</v>
+        <v>8606</v>
       </c>
       <c r="C8" t="n">
         <v>0</v>
@@ -634,20 +634,20 @@
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>780</v>
+        <v>2605</v>
       </c>
       <c r="G8" t="n">
-        <v>48</v>
+        <v>6001</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2024-11-26</t>
+          <t>2024-12-12 10:10:11</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>828</v>
+        <v>8606</v>
       </c>
       <c r="C9" t="n">
         <v>0</v>
@@ -659,20 +659,20 @@
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>780</v>
+        <v>2605</v>
       </c>
       <c r="G9" t="n">
-        <v>48</v>
+        <v>6001</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2024-11-26</t>
+          <t>2024-12-12 10:10:11</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>866</v>
+        <v>8606</v>
       </c>
       <c r="C10" t="n">
         <v>0</v>
@@ -684,16 +684,16 @@
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>860</v>
+        <v>2605</v>
       </c>
       <c r="G10" t="n">
-        <v>6</v>
+        <v>6001</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2024-12-12</t>
+          <t>2024-12-12 10:10:11</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -718,7 +718,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2024-12-12</t>
+          <t>2024-12-12 10:10:11</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -743,7 +743,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2024-12-12</t>
+          <t>2024-12-12 10:10:11</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -768,7 +768,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2024-12-12</t>
+          <t>2024-12-12 10:10:11</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -793,7 +793,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2024-12-12</t>
+          <t>2024-12-12 10:10:11</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -818,7 +818,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2024-12-12</t>
+          <t>2024-12-12 10:10:11</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -843,7 +843,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2024-12-12</t>
+          <t>2024-12-12 10:10:11</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -868,7 +868,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2024-12-12</t>
+          <t>2024-12-12 10:10:11</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -893,7 +893,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2024-12-12</t>
+          <t>2024-12-12 10:10:11</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -918,7 +918,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2024-12-12</t>
+          <t>2024-12-12 10:10:11</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -937,6 +937,706 @@
         <v>2605</v>
       </c>
       <c r="G20" t="n">
+        <v>6001</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2024-12-12 10:10:11</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>8606</v>
+      </c>
+      <c r="C21" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" t="n">
+        <v>2605</v>
+      </c>
+      <c r="G21" t="n">
+        <v>6001</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2024-12-12 10:59:33</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>8606</v>
+      </c>
+      <c r="C22" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" t="n">
+        <v>2605</v>
+      </c>
+      <c r="G22" t="n">
+        <v>6001</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2024-12-12 10:59:37</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>8606</v>
+      </c>
+      <c r="C23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" t="n">
+        <v>2605</v>
+      </c>
+      <c r="G23" t="n">
+        <v>6001</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2024-12-12 10:59:41</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>8606</v>
+      </c>
+      <c r="C24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" t="n">
+        <v>2605</v>
+      </c>
+      <c r="G24" t="n">
+        <v>6001</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2024-12-12 10:10:11</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>8606</v>
+      </c>
+      <c r="C25" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" t="n">
+        <v>2605</v>
+      </c>
+      <c r="G25" t="n">
+        <v>6001</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2024-12-12 10:59:33</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>8606</v>
+      </c>
+      <c r="C26" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" t="n">
+        <v>2605</v>
+      </c>
+      <c r="G26" t="n">
+        <v>6001</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2024-12-12 10:59:37</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>8606</v>
+      </c>
+      <c r="C27" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" t="n">
+        <v>2605</v>
+      </c>
+      <c r="G27" t="n">
+        <v>6001</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2024-12-12 10:59:41</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>8606</v>
+      </c>
+      <c r="C28" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" t="n">
+        <v>2605</v>
+      </c>
+      <c r="G28" t="n">
+        <v>6001</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2024-12-12 10:10:11</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>8606</v>
+      </c>
+      <c r="C29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" t="n">
+        <v>2605</v>
+      </c>
+      <c r="G29" t="n">
+        <v>6001</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2024-12-12 10:59:33</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>8606</v>
+      </c>
+      <c r="C30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" t="n">
+        <v>2605</v>
+      </c>
+      <c r="G30" t="n">
+        <v>6001</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2024-12-12 10:59:37</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>8606</v>
+      </c>
+      <c r="C31" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" t="n">
+        <v>2605</v>
+      </c>
+      <c r="G31" t="n">
+        <v>6001</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2024-12-12 10:59:41</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>8606</v>
+      </c>
+      <c r="C32" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" t="n">
+        <v>2605</v>
+      </c>
+      <c r="G32" t="n">
+        <v>6001</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2024-12-12 10:10:11</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>8606</v>
+      </c>
+      <c r="C33" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" t="n">
+        <v>2605</v>
+      </c>
+      <c r="G33" t="n">
+        <v>6001</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2024-12-12 10:59:33</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>8606</v>
+      </c>
+      <c r="C34" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" t="n">
+        <v>2605</v>
+      </c>
+      <c r="G34" t="n">
+        <v>6001</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2024-12-12 10:59:37</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>8606</v>
+      </c>
+      <c r="C35" t="n">
+        <v>0</v>
+      </c>
+      <c r="D35" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" t="n">
+        <v>2605</v>
+      </c>
+      <c r="G35" t="n">
+        <v>6001</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2024-12-12 10:59:41</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>8606</v>
+      </c>
+      <c r="C36" t="n">
+        <v>0</v>
+      </c>
+      <c r="D36" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" t="n">
+        <v>2605</v>
+      </c>
+      <c r="G36" t="n">
+        <v>6001</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2024-12-12 10:10:11</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>8606</v>
+      </c>
+      <c r="C37" t="n">
+        <v>0</v>
+      </c>
+      <c r="D37" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" t="n">
+        <v>2605</v>
+      </c>
+      <c r="G37" t="n">
+        <v>6001</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2024-12-12 10:59:33</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>8606</v>
+      </c>
+      <c r="C38" t="n">
+        <v>0</v>
+      </c>
+      <c r="D38" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" t="n">
+        <v>2605</v>
+      </c>
+      <c r="G38" t="n">
+        <v>6001</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2024-12-12 10:59:37</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>8606</v>
+      </c>
+      <c r="C39" t="n">
+        <v>0</v>
+      </c>
+      <c r="D39" t="n">
+        <v>0</v>
+      </c>
+      <c r="E39" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" t="n">
+        <v>2605</v>
+      </c>
+      <c r="G39" t="n">
+        <v>6001</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2024-12-12 10:59:41</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>8606</v>
+      </c>
+      <c r="C40" t="n">
+        <v>0</v>
+      </c>
+      <c r="D40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" t="n">
+        <v>2605</v>
+      </c>
+      <c r="G40" t="n">
+        <v>6001</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2024-12-12 10:10:11</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>8606</v>
+      </c>
+      <c r="C41" t="n">
+        <v>0</v>
+      </c>
+      <c r="D41" t="n">
+        <v>0</v>
+      </c>
+      <c r="E41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" t="n">
+        <v>2605</v>
+      </c>
+      <c r="G41" t="n">
+        <v>6001</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2024-12-12 10:59:33</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>8606</v>
+      </c>
+      <c r="C42" t="n">
+        <v>0</v>
+      </c>
+      <c r="D42" t="n">
+        <v>0</v>
+      </c>
+      <c r="E42" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" t="n">
+        <v>2605</v>
+      </c>
+      <c r="G42" t="n">
+        <v>6001</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2024-12-12 10:59:37</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>8606</v>
+      </c>
+      <c r="C43" t="n">
+        <v>0</v>
+      </c>
+      <c r="D43" t="n">
+        <v>0</v>
+      </c>
+      <c r="E43" t="n">
+        <v>0</v>
+      </c>
+      <c r="F43" t="n">
+        <v>2605</v>
+      </c>
+      <c r="G43" t="n">
+        <v>6001</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2024-12-12 10:59:41</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>8606</v>
+      </c>
+      <c r="C44" t="n">
+        <v>0</v>
+      </c>
+      <c r="D44" t="n">
+        <v>0</v>
+      </c>
+      <c r="E44" t="n">
+        <v>0</v>
+      </c>
+      <c r="F44" t="n">
+        <v>2605</v>
+      </c>
+      <c r="G44" t="n">
+        <v>6001</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2024-12-12 10:10:11</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>8606</v>
+      </c>
+      <c r="C45" t="n">
+        <v>0</v>
+      </c>
+      <c r="D45" t="n">
+        <v>0</v>
+      </c>
+      <c r="E45" t="n">
+        <v>0</v>
+      </c>
+      <c r="F45" t="n">
+        <v>2605</v>
+      </c>
+      <c r="G45" t="n">
+        <v>6001</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2024-12-12 10:59:33</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>8606</v>
+      </c>
+      <c r="C46" t="n">
+        <v>0</v>
+      </c>
+      <c r="D46" t="n">
+        <v>0</v>
+      </c>
+      <c r="E46" t="n">
+        <v>0</v>
+      </c>
+      <c r="F46" t="n">
+        <v>2605</v>
+      </c>
+      <c r="G46" t="n">
+        <v>6001</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2024-12-12 10:59:37</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>8606</v>
+      </c>
+      <c r="C47" t="n">
+        <v>0</v>
+      </c>
+      <c r="D47" t="n">
+        <v>0</v>
+      </c>
+      <c r="E47" t="n">
+        <v>0</v>
+      </c>
+      <c r="F47" t="n">
+        <v>2605</v>
+      </c>
+      <c r="G47" t="n">
+        <v>6001</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2024-12-12 10:59:41</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>8606</v>
+      </c>
+      <c r="C48" t="n">
+        <v>0</v>
+      </c>
+      <c r="D48" t="n">
+        <v>0</v>
+      </c>
+      <c r="E48" t="n">
+        <v>0</v>
+      </c>
+      <c r="F48" t="n">
+        <v>2605</v>
+      </c>
+      <c r="G48" t="n">
         <v>6001</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Updated with feature alignment small test
</commit_message>
<xml_diff>
--- a/LOC tracking outputs/code_metrics.xlsx
+++ b/LOC tracking outputs/code_metrics.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -665,6 +665,181 @@
         <v>6347</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2024-12-12 14:22:25</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>8933</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>2714</v>
+      </c>
+      <c r="G10" t="n">
+        <v>6219</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2024-12-12 15:01:02</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>9125</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="n">
+        <v>2778</v>
+      </c>
+      <c r="G11" t="n">
+        <v>6347</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2024-12-12 15:02:08</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>9125</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="n">
+        <v>2778</v>
+      </c>
+      <c r="G12" t="n">
+        <v>6347</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2024-12-17 09:34:39</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>9392</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" t="n">
+        <v>2867</v>
+      </c>
+      <c r="G13" t="n">
+        <v>6525</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2024-12-12 14:22:25</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>8933</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" t="n">
+        <v>2714</v>
+      </c>
+      <c r="G14" t="n">
+        <v>6219</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2024-12-12 15:01:02</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>9125</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="n">
+        <v>2778</v>
+      </c>
+      <c r="G15" t="n">
+        <v>6347</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2024-12-17 09:34:39</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>9392</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
+        <v>2867</v>
+      </c>
+      <c r="G16" t="n">
+        <v>6525</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Feather to array work
</commit_message>
<xml_diff>
--- a/LOC tracking outputs/code_metrics.xlsx
+++ b/LOC tracking outputs/code_metrics.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -840,6 +840,1381 @@
         <v>6525</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2024-12-12 14:22:25</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>8933</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="n">
+        <v>2714</v>
+      </c>
+      <c r="G17" t="n">
+        <v>6219</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2024-12-12 15:01:02</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>9125</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" t="n">
+        <v>2778</v>
+      </c>
+      <c r="G18" t="n">
+        <v>6347</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2024-12-17 09:34:39</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>9392</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" t="n">
+        <v>2867</v>
+      </c>
+      <c r="G19" t="n">
+        <v>6525</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2024-12-20 13:39:15</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>12255</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" t="n">
+        <v>3086</v>
+      </c>
+      <c r="G20" t="n">
+        <v>9169</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2024-12-12 14:22:25</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>8933</v>
+      </c>
+      <c r="C21" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" t="n">
+        <v>2714</v>
+      </c>
+      <c r="G21" t="n">
+        <v>6219</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2024-12-12 15:01:02</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>9125</v>
+      </c>
+      <c r="C22" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" t="n">
+        <v>2778</v>
+      </c>
+      <c r="G22" t="n">
+        <v>6347</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2024-12-17 09:34:39</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>9392</v>
+      </c>
+      <c r="C23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" t="n">
+        <v>2867</v>
+      </c>
+      <c r="G23" t="n">
+        <v>6525</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2024-12-20 13:39:15</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>11609</v>
+      </c>
+      <c r="C24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" t="n">
+        <v>3086</v>
+      </c>
+      <c r="G24" t="n">
+        <v>8523</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2024-12-20 13:41:02</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>11609</v>
+      </c>
+      <c r="C25" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" t="n">
+        <v>3086</v>
+      </c>
+      <c r="G25" t="n">
+        <v>8523</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2024-12-12 14:22:25</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>8933</v>
+      </c>
+      <c r="C26" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" t="n">
+        <v>2714</v>
+      </c>
+      <c r="G26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2024-12-12 15:01:02</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>9125</v>
+      </c>
+      <c r="C27" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" t="n">
+        <v>2778</v>
+      </c>
+      <c r="G27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2024-12-17 09:34:39</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>9392</v>
+      </c>
+      <c r="C28" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" t="n">
+        <v>2867</v>
+      </c>
+      <c r="G28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2024-12-20 13:39:15</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>11609</v>
+      </c>
+      <c r="C29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" t="n">
+        <v>3086</v>
+      </c>
+      <c r="G29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2024-12-20 13:41:02</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>11609</v>
+      </c>
+      <c r="C30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" t="n">
+        <v>3086</v>
+      </c>
+      <c r="G30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2024-12-12 14:22:25</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>8933</v>
+      </c>
+      <c r="C31" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" t="n">
+        <v>2714</v>
+      </c>
+      <c r="G31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2024-12-12 15:01:02</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>9125</v>
+      </c>
+      <c r="C32" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" t="n">
+        <v>2778</v>
+      </c>
+      <c r="G32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2024-12-17 09:34:39</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>9392</v>
+      </c>
+      <c r="C33" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" t="n">
+        <v>2867</v>
+      </c>
+      <c r="G33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2024-12-20 13:39:15</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>11609</v>
+      </c>
+      <c r="C34" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" t="n">
+        <v>3086</v>
+      </c>
+      <c r="G34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2024-12-20 13:41:02</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>11609</v>
+      </c>
+      <c r="C35" t="n">
+        <v>0</v>
+      </c>
+      <c r="D35" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" t="n">
+        <v>3086</v>
+      </c>
+      <c r="G35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2024-12-12 14:22:25</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>8933</v>
+      </c>
+      <c r="C36" t="n">
+        <v>0</v>
+      </c>
+      <c r="D36" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" t="n">
+        <v>2714</v>
+      </c>
+      <c r="G36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2024-12-12 15:01:02</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>9125</v>
+      </c>
+      <c r="C37" t="n">
+        <v>0</v>
+      </c>
+      <c r="D37" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" t="n">
+        <v>2778</v>
+      </c>
+      <c r="G37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2024-12-17 09:34:39</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>9392</v>
+      </c>
+      <c r="C38" t="n">
+        <v>0</v>
+      </c>
+      <c r="D38" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" t="n">
+        <v>2867</v>
+      </c>
+      <c r="G38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2024-12-20 13:39:15</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>11609</v>
+      </c>
+      <c r="C39" t="n">
+        <v>0</v>
+      </c>
+      <c r="D39" t="n">
+        <v>0</v>
+      </c>
+      <c r="E39" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" t="n">
+        <v>3086</v>
+      </c>
+      <c r="G39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2024-12-20 13:41:02</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>11609</v>
+      </c>
+      <c r="C40" t="n">
+        <v>0</v>
+      </c>
+      <c r="D40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" t="n">
+        <v>3086</v>
+      </c>
+      <c r="G40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2024-12-12 14:22:25</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>8933</v>
+      </c>
+      <c r="C41" t="n">
+        <v>0</v>
+      </c>
+      <c r="D41" t="n">
+        <v>0</v>
+      </c>
+      <c r="E41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" t="n">
+        <v>2714</v>
+      </c>
+      <c r="G41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2024-12-12 15:01:02</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>9125</v>
+      </c>
+      <c r="C42" t="n">
+        <v>0</v>
+      </c>
+      <c r="D42" t="n">
+        <v>0</v>
+      </c>
+      <c r="E42" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" t="n">
+        <v>2778</v>
+      </c>
+      <c r="G42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2024-12-17 09:34:39</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>9392</v>
+      </c>
+      <c r="C43" t="n">
+        <v>0</v>
+      </c>
+      <c r="D43" t="n">
+        <v>0</v>
+      </c>
+      <c r="E43" t="n">
+        <v>0</v>
+      </c>
+      <c r="F43" t="n">
+        <v>2867</v>
+      </c>
+      <c r="G43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2024-12-20 13:39:15</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>11609</v>
+      </c>
+      <c r="C44" t="n">
+        <v>0</v>
+      </c>
+      <c r="D44" t="n">
+        <v>0</v>
+      </c>
+      <c r="E44" t="n">
+        <v>0</v>
+      </c>
+      <c r="F44" t="n">
+        <v>3086</v>
+      </c>
+      <c r="G44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2024-12-20 13:41:02</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>11609</v>
+      </c>
+      <c r="C45" t="n">
+        <v>0</v>
+      </c>
+      <c r="D45" t="n">
+        <v>0</v>
+      </c>
+      <c r="E45" t="n">
+        <v>0</v>
+      </c>
+      <c r="F45" t="n">
+        <v>3086</v>
+      </c>
+      <c r="G45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2024-12-12 14:22:25</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>8933</v>
+      </c>
+      <c r="C46" t="n">
+        <v>0</v>
+      </c>
+      <c r="D46" t="n">
+        <v>0</v>
+      </c>
+      <c r="E46" t="n">
+        <v>0</v>
+      </c>
+      <c r="F46" t="n">
+        <v>2714</v>
+      </c>
+      <c r="G46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2024-12-12 15:01:02</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>9125</v>
+      </c>
+      <c r="C47" t="n">
+        <v>0</v>
+      </c>
+      <c r="D47" t="n">
+        <v>0</v>
+      </c>
+      <c r="E47" t="n">
+        <v>0</v>
+      </c>
+      <c r="F47" t="n">
+        <v>2778</v>
+      </c>
+      <c r="G47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2024-12-17 09:34:39</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>9392</v>
+      </c>
+      <c r="C48" t="n">
+        <v>0</v>
+      </c>
+      <c r="D48" t="n">
+        <v>0</v>
+      </c>
+      <c r="E48" t="n">
+        <v>0</v>
+      </c>
+      <c r="F48" t="n">
+        <v>2867</v>
+      </c>
+      <c r="G48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2024-12-20 13:39:15</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>11609</v>
+      </c>
+      <c r="C49" t="n">
+        <v>0</v>
+      </c>
+      <c r="D49" t="n">
+        <v>0</v>
+      </c>
+      <c r="E49" t="n">
+        <v>0</v>
+      </c>
+      <c r="F49" t="n">
+        <v>3086</v>
+      </c>
+      <c r="G49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2024-12-20 13:41:02</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>11609</v>
+      </c>
+      <c r="C50" t="n">
+        <v>0</v>
+      </c>
+      <c r="D50" t="n">
+        <v>0</v>
+      </c>
+      <c r="E50" t="n">
+        <v>0</v>
+      </c>
+      <c r="F50" t="n">
+        <v>3086</v>
+      </c>
+      <c r="G50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2024-12-12 14:22:25</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>8933</v>
+      </c>
+      <c r="C51" t="n">
+        <v>0</v>
+      </c>
+      <c r="D51" t="n">
+        <v>0</v>
+      </c>
+      <c r="E51" t="n">
+        <v>0</v>
+      </c>
+      <c r="F51" t="n">
+        <v>2714</v>
+      </c>
+      <c r="G51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2024-12-12 15:01:02</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>9125</v>
+      </c>
+      <c r="C52" t="n">
+        <v>0</v>
+      </c>
+      <c r="D52" t="n">
+        <v>0</v>
+      </c>
+      <c r="E52" t="n">
+        <v>0</v>
+      </c>
+      <c r="F52" t="n">
+        <v>2778</v>
+      </c>
+      <c r="G52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2024-12-17 09:34:39</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>9392</v>
+      </c>
+      <c r="C53" t="n">
+        <v>0</v>
+      </c>
+      <c r="D53" t="n">
+        <v>0</v>
+      </c>
+      <c r="E53" t="n">
+        <v>0</v>
+      </c>
+      <c r="F53" t="n">
+        <v>2867</v>
+      </c>
+      <c r="G53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2024-12-20 13:39:15</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>11609</v>
+      </c>
+      <c r="C54" t="n">
+        <v>0</v>
+      </c>
+      <c r="D54" t="n">
+        <v>0</v>
+      </c>
+      <c r="E54" t="n">
+        <v>0</v>
+      </c>
+      <c r="F54" t="n">
+        <v>3086</v>
+      </c>
+      <c r="G54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2024-12-20 13:41:02</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>11609</v>
+      </c>
+      <c r="C55" t="n">
+        <v>0</v>
+      </c>
+      <c r="D55" t="n">
+        <v>0</v>
+      </c>
+      <c r="E55" t="n">
+        <v>0</v>
+      </c>
+      <c r="F55" t="n">
+        <v>3086</v>
+      </c>
+      <c r="G55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2024-12-12 14:22:25</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>8933</v>
+      </c>
+      <c r="C56" t="n">
+        <v>0</v>
+      </c>
+      <c r="D56" t="n">
+        <v>0</v>
+      </c>
+      <c r="E56" t="n">
+        <v>0</v>
+      </c>
+      <c r="F56" t="n">
+        <v>2714</v>
+      </c>
+      <c r="G56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2024-12-12 15:01:02</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>9125</v>
+      </c>
+      <c r="C57" t="n">
+        <v>0</v>
+      </c>
+      <c r="D57" t="n">
+        <v>0</v>
+      </c>
+      <c r="E57" t="n">
+        <v>0</v>
+      </c>
+      <c r="F57" t="n">
+        <v>2778</v>
+      </c>
+      <c r="G57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2024-12-17 09:34:39</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>9392</v>
+      </c>
+      <c r="C58" t="n">
+        <v>0</v>
+      </c>
+      <c r="D58" t="n">
+        <v>0</v>
+      </c>
+      <c r="E58" t="n">
+        <v>0</v>
+      </c>
+      <c r="F58" t="n">
+        <v>2867</v>
+      </c>
+      <c r="G58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2024-12-20 13:39:15</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>11609</v>
+      </c>
+      <c r="C59" t="n">
+        <v>0</v>
+      </c>
+      <c r="D59" t="n">
+        <v>0</v>
+      </c>
+      <c r="E59" t="n">
+        <v>0</v>
+      </c>
+      <c r="F59" t="n">
+        <v>3086</v>
+      </c>
+      <c r="G59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2024-12-20 13:41:02</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>11609</v>
+      </c>
+      <c r="C60" t="n">
+        <v>0</v>
+      </c>
+      <c r="D60" t="n">
+        <v>0</v>
+      </c>
+      <c r="E60" t="n">
+        <v>0</v>
+      </c>
+      <c r="F60" t="n">
+        <v>3086</v>
+      </c>
+      <c r="G60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2024-12-12 14:22:25</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>8933</v>
+      </c>
+      <c r="C61" t="n">
+        <v>0</v>
+      </c>
+      <c r="D61" t="n">
+        <v>0</v>
+      </c>
+      <c r="E61" t="n">
+        <v>0</v>
+      </c>
+      <c r="F61" t="n">
+        <v>2714</v>
+      </c>
+      <c r="G61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2024-12-12 15:01:02</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>9125</v>
+      </c>
+      <c r="C62" t="n">
+        <v>0</v>
+      </c>
+      <c r="D62" t="n">
+        <v>0</v>
+      </c>
+      <c r="E62" t="n">
+        <v>0</v>
+      </c>
+      <c r="F62" t="n">
+        <v>2778</v>
+      </c>
+      <c r="G62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2024-12-17 09:34:39</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>9392</v>
+      </c>
+      <c r="C63" t="n">
+        <v>0</v>
+      </c>
+      <c r="D63" t="n">
+        <v>0</v>
+      </c>
+      <c r="E63" t="n">
+        <v>0</v>
+      </c>
+      <c r="F63" t="n">
+        <v>2867</v>
+      </c>
+      <c r="G63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2024-12-20 13:39:15</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>11609</v>
+      </c>
+      <c r="C64" t="n">
+        <v>0</v>
+      </c>
+      <c r="D64" t="n">
+        <v>0</v>
+      </c>
+      <c r="E64" t="n">
+        <v>0</v>
+      </c>
+      <c r="F64" t="n">
+        <v>3086</v>
+      </c>
+      <c r="G64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2024-12-20 13:41:02</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>11609</v>
+      </c>
+      <c r="C65" t="n">
+        <v>0</v>
+      </c>
+      <c r="D65" t="n">
+        <v>0</v>
+      </c>
+      <c r="E65" t="n">
+        <v>0</v>
+      </c>
+      <c r="F65" t="n">
+        <v>3086</v>
+      </c>
+      <c r="G65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2024-12-12 14:22:25</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>8933</v>
+      </c>
+      <c r="C66" t="n">
+        <v>0</v>
+      </c>
+      <c r="D66" t="n">
+        <v>0</v>
+      </c>
+      <c r="E66" t="n">
+        <v>0</v>
+      </c>
+      <c r="F66" t="n">
+        <v>2714</v>
+      </c>
+      <c r="G66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2024-12-12 15:01:02</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>9125</v>
+      </c>
+      <c r="C67" t="n">
+        <v>0</v>
+      </c>
+      <c r="D67" t="n">
+        <v>0</v>
+      </c>
+      <c r="E67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F67" t="n">
+        <v>2778</v>
+      </c>
+      <c r="G67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2024-12-17 09:34:39</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>9392</v>
+      </c>
+      <c r="C68" t="n">
+        <v>0</v>
+      </c>
+      <c r="D68" t="n">
+        <v>0</v>
+      </c>
+      <c r="E68" t="n">
+        <v>0</v>
+      </c>
+      <c r="F68" t="n">
+        <v>2867</v>
+      </c>
+      <c r="G68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2024-12-20 13:39:15</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>11609</v>
+      </c>
+      <c r="C69" t="n">
+        <v>0</v>
+      </c>
+      <c r="D69" t="n">
+        <v>0</v>
+      </c>
+      <c r="E69" t="n">
+        <v>0</v>
+      </c>
+      <c r="F69" t="n">
+        <v>3086</v>
+      </c>
+      <c r="G69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2024-12-20 13:41:02</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>11609</v>
+      </c>
+      <c r="C70" t="n">
+        <v>0</v>
+      </c>
+      <c r="D70" t="n">
+        <v>0</v>
+      </c>
+      <c r="E70" t="n">
+        <v>0</v>
+      </c>
+      <c r="F70" t="n">
+        <v>3086</v>
+      </c>
+      <c r="G70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2024-12-12 14:22:25</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>8933</v>
+      </c>
+      <c r="C71" t="n">
+        <v>0</v>
+      </c>
+      <c r="D71" t="n">
+        <v>0</v>
+      </c>
+      <c r="E71" t="n">
+        <v>0</v>
+      </c>
+      <c r="F71" t="n">
+        <v>2714</v>
+      </c>
+      <c r="G71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2024-12-12 15:01:02</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>9125</v>
+      </c>
+      <c r="C72" t="n">
+        <v>0</v>
+      </c>
+      <c r="D72" t="n">
+        <v>0</v>
+      </c>
+      <c r="E72" t="n">
+        <v>0</v>
+      </c>
+      <c r="F72" t="n">
+        <v>2778</v>
+      </c>
+      <c r="G72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2024-12-17 09:34:39</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>9392</v>
+      </c>
+      <c r="C73" t="n">
+        <v>0</v>
+      </c>
+      <c r="D73" t="n">
+        <v>0</v>
+      </c>
+      <c r="E73" t="n">
+        <v>0</v>
+      </c>
+      <c r="F73" t="n">
+        <v>2867</v>
+      </c>
+      <c r="G73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2024-12-20 13:39:15</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>11609</v>
+      </c>
+      <c r="C74" t="n">
+        <v>0</v>
+      </c>
+      <c r="D74" t="n">
+        <v>0</v>
+      </c>
+      <c r="E74" t="n">
+        <v>0</v>
+      </c>
+      <c r="F74" t="n">
+        <v>3086</v>
+      </c>
+      <c r="G74" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2024-12-20 13:41:02</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>11609</v>
+      </c>
+      <c r="C75" t="n">
+        <v>0</v>
+      </c>
+      <c r="D75" t="n">
+        <v>0</v>
+      </c>
+      <c r="E75" t="n">
+        <v>0</v>
+      </c>
+      <c r="F75" t="n">
+        <v>3086</v>
+      </c>
+      <c r="G75" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Blank subtraction module started
</commit_message>
<xml_diff>
--- a/LOC tracking outputs/code_metrics.xlsx
+++ b/LOC tracking outputs/code_metrics.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G110"/>
+  <dimension ref="A1:G119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3020,6 +3020,213 @@
       </c>
       <c r="G110" t="inlineStr"/>
     </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2024-12-12 14:22:25</t>
+        </is>
+      </c>
+      <c r="B111" t="n">
+        <v>8933</v>
+      </c>
+      <c r="C111" t="n">
+        <v>0</v>
+      </c>
+      <c r="D111" t="n">
+        <v>0</v>
+      </c>
+      <c r="E111" t="n">
+        <v>0</v>
+      </c>
+      <c r="F111" t="n">
+        <v>2714</v>
+      </c>
+      <c r="G111" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2024-12-12 15:01:02</t>
+        </is>
+      </c>
+      <c r="B112" t="n">
+        <v>9125</v>
+      </c>
+      <c r="C112" t="n">
+        <v>0</v>
+      </c>
+      <c r="D112" t="n">
+        <v>0</v>
+      </c>
+      <c r="E112" t="n">
+        <v>0</v>
+      </c>
+      <c r="F112" t="n">
+        <v>2778</v>
+      </c>
+      <c r="G112" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>2024-12-17 09:34:39</t>
+        </is>
+      </c>
+      <c r="B113" t="n">
+        <v>9392</v>
+      </c>
+      <c r="C113" t="n">
+        <v>0</v>
+      </c>
+      <c r="D113" t="n">
+        <v>0</v>
+      </c>
+      <c r="E113" t="n">
+        <v>0</v>
+      </c>
+      <c r="F113" t="n">
+        <v>2867</v>
+      </c>
+      <c r="G113" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>2024-12-20 13:39:15</t>
+        </is>
+      </c>
+      <c r="B114" t="n">
+        <v>11609</v>
+      </c>
+      <c r="C114" t="n">
+        <v>0</v>
+      </c>
+      <c r="D114" t="n">
+        <v>0</v>
+      </c>
+      <c r="E114" t="n">
+        <v>0</v>
+      </c>
+      <c r="F114" t="n">
+        <v>3086</v>
+      </c>
+      <c r="G114" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>2024-12-20 13:41:02</t>
+        </is>
+      </c>
+      <c r="B115" t="n">
+        <v>11609</v>
+      </c>
+      <c r="C115" t="n">
+        <v>0</v>
+      </c>
+      <c r="D115" t="n">
+        <v>0</v>
+      </c>
+      <c r="E115" t="n">
+        <v>0</v>
+      </c>
+      <c r="F115" t="n">
+        <v>3086</v>
+      </c>
+      <c r="G115" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>2025-01-16 14:58:07</t>
+        </is>
+      </c>
+      <c r="B116" t="n">
+        <v>12131</v>
+      </c>
+      <c r="C116" t="n">
+        <v>0</v>
+      </c>
+      <c r="D116" t="n">
+        <v>0</v>
+      </c>
+      <c r="E116" t="n">
+        <v>0</v>
+      </c>
+      <c r="F116" t="n">
+        <v>3277</v>
+      </c>
+      <c r="G116" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>2025-01-16 15:00:07</t>
+        </is>
+      </c>
+      <c r="B117" t="n">
+        <v>12131</v>
+      </c>
+      <c r="C117" t="n">
+        <v>0</v>
+      </c>
+      <c r="D117" t="n">
+        <v>0</v>
+      </c>
+      <c r="E117" t="n">
+        <v>0</v>
+      </c>
+      <c r="F117" t="n">
+        <v>3277</v>
+      </c>
+      <c r="G117" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>2025-01-21 15:00:05</t>
+        </is>
+      </c>
+      <c r="B118" t="n">
+        <v>14226</v>
+      </c>
+      <c r="C118" t="n">
+        <v>0</v>
+      </c>
+      <c r="D118" t="n">
+        <v>0</v>
+      </c>
+      <c r="E118" t="n">
+        <v>0</v>
+      </c>
+      <c r="F118" t="n">
+        <v>3357</v>
+      </c>
+      <c r="G118" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>2025-01-24 08:09:58</t>
+        </is>
+      </c>
+      <c r="B119" t="n">
+        <v>15227</v>
+      </c>
+      <c r="C119" t="n">
+        <v>0</v>
+      </c>
+      <c r="D119" t="n">
+        <v>0</v>
+      </c>
+      <c r="E119" t="n">
+        <v>0</v>
+      </c>
+      <c r="F119" t="n">
+        <v>3478</v>
+      </c>
+      <c r="G119" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Modified the names of experimental groups
</commit_message>
<xml_diff>
--- a/LOC tracking outputs/code_metrics.xlsx
+++ b/LOC tracking outputs/code_metrics.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G119"/>
+  <dimension ref="A1:G123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3227,6 +3227,98 @@
       </c>
       <c r="G119" t="inlineStr"/>
     </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>2025-01-22 15:12:38</t>
+        </is>
+      </c>
+      <c r="B120" t="n">
+        <v>14445</v>
+      </c>
+      <c r="C120" t="n">
+        <v>0</v>
+      </c>
+      <c r="D120" t="n">
+        <v>0</v>
+      </c>
+      <c r="E120" t="n">
+        <v>0</v>
+      </c>
+      <c r="F120" t="n">
+        <v>3420</v>
+      </c>
+      <c r="G120" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>2025-01-22 15:13:06</t>
+        </is>
+      </c>
+      <c r="B121" t="n">
+        <v>14445</v>
+      </c>
+      <c r="C121" t="n">
+        <v>0</v>
+      </c>
+      <c r="D121" t="n">
+        <v>0</v>
+      </c>
+      <c r="E121" t="n">
+        <v>0</v>
+      </c>
+      <c r="F121" t="n">
+        <v>3420</v>
+      </c>
+      <c r="G121" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>2025-01-22 15:13:32</t>
+        </is>
+      </c>
+      <c r="B122" t="n">
+        <v>14445</v>
+      </c>
+      <c r="C122" t="n">
+        <v>0</v>
+      </c>
+      <c r="D122" t="n">
+        <v>0</v>
+      </c>
+      <c r="E122" t="n">
+        <v>0</v>
+      </c>
+      <c r="F122" t="n">
+        <v>3420</v>
+      </c>
+      <c r="G122" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>2025-01-25 08:17:46</t>
+        </is>
+      </c>
+      <c r="B123" t="n">
+        <v>16727</v>
+      </c>
+      <c r="C123" t="n">
+        <v>0</v>
+      </c>
+      <c r="D123" t="n">
+        <v>0</v>
+      </c>
+      <c r="E123" t="n">
+        <v>0</v>
+      </c>
+      <c r="F123" t="n">
+        <v>3853</v>
+      </c>
+      <c r="G123" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Working combining, needs work to improve utility
</commit_message>
<xml_diff>
--- a/LOC tracking outputs/code_metrics.xlsx
+++ b/LOC tracking outputs/code_metrics.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G123"/>
+  <dimension ref="A1:G133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3319,6 +3319,236 @@
       </c>
       <c r="G123" t="inlineStr"/>
     </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2024-12-12 14:22:25</t>
+        </is>
+      </c>
+      <c r="B124" t="n">
+        <v>8933</v>
+      </c>
+      <c r="C124" t="n">
+        <v>0</v>
+      </c>
+      <c r="D124" t="n">
+        <v>0</v>
+      </c>
+      <c r="E124" t="n">
+        <v>0</v>
+      </c>
+      <c r="F124" t="n">
+        <v>2714</v>
+      </c>
+      <c r="G124" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2024-12-12 15:01:02</t>
+        </is>
+      </c>
+      <c r="B125" t="n">
+        <v>9125</v>
+      </c>
+      <c r="C125" t="n">
+        <v>0</v>
+      </c>
+      <c r="D125" t="n">
+        <v>0</v>
+      </c>
+      <c r="E125" t="n">
+        <v>0</v>
+      </c>
+      <c r="F125" t="n">
+        <v>2778</v>
+      </c>
+      <c r="G125" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2024-12-17 09:34:39</t>
+        </is>
+      </c>
+      <c r="B126" t="n">
+        <v>9392</v>
+      </c>
+      <c r="C126" t="n">
+        <v>0</v>
+      </c>
+      <c r="D126" t="n">
+        <v>0</v>
+      </c>
+      <c r="E126" t="n">
+        <v>0</v>
+      </c>
+      <c r="F126" t="n">
+        <v>2867</v>
+      </c>
+      <c r="G126" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2024-12-20 13:39:15</t>
+        </is>
+      </c>
+      <c r="B127" t="n">
+        <v>11609</v>
+      </c>
+      <c r="C127" t="n">
+        <v>0</v>
+      </c>
+      <c r="D127" t="n">
+        <v>0</v>
+      </c>
+      <c r="E127" t="n">
+        <v>0</v>
+      </c>
+      <c r="F127" t="n">
+        <v>3086</v>
+      </c>
+      <c r="G127" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2024-12-20 13:41:02</t>
+        </is>
+      </c>
+      <c r="B128" t="n">
+        <v>11609</v>
+      </c>
+      <c r="C128" t="n">
+        <v>0</v>
+      </c>
+      <c r="D128" t="n">
+        <v>0</v>
+      </c>
+      <c r="E128" t="n">
+        <v>0</v>
+      </c>
+      <c r="F128" t="n">
+        <v>3086</v>
+      </c>
+      <c r="G128" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>2025-01-16 14:58:07</t>
+        </is>
+      </c>
+      <c r="B129" t="n">
+        <v>12131</v>
+      </c>
+      <c r="C129" t="n">
+        <v>0</v>
+      </c>
+      <c r="D129" t="n">
+        <v>0</v>
+      </c>
+      <c r="E129" t="n">
+        <v>0</v>
+      </c>
+      <c r="F129" t="n">
+        <v>3277</v>
+      </c>
+      <c r="G129" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>2025-01-16 15:00:07</t>
+        </is>
+      </c>
+      <c r="B130" t="n">
+        <v>12131</v>
+      </c>
+      <c r="C130" t="n">
+        <v>0</v>
+      </c>
+      <c r="D130" t="n">
+        <v>0</v>
+      </c>
+      <c r="E130" t="n">
+        <v>0</v>
+      </c>
+      <c r="F130" t="n">
+        <v>3277</v>
+      </c>
+      <c r="G130" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>2025-01-21 15:00:05</t>
+        </is>
+      </c>
+      <c r="B131" t="n">
+        <v>14226</v>
+      </c>
+      <c r="C131" t="n">
+        <v>0</v>
+      </c>
+      <c r="D131" t="n">
+        <v>0</v>
+      </c>
+      <c r="E131" t="n">
+        <v>0</v>
+      </c>
+      <c r="F131" t="n">
+        <v>3357</v>
+      </c>
+      <c r="G131" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>2025-01-24 08:09:58</t>
+        </is>
+      </c>
+      <c r="B132" t="n">
+        <v>15227</v>
+      </c>
+      <c r="C132" t="n">
+        <v>0</v>
+      </c>
+      <c r="D132" t="n">
+        <v>0</v>
+      </c>
+      <c r="E132" t="n">
+        <v>0</v>
+      </c>
+      <c r="F132" t="n">
+        <v>3478</v>
+      </c>
+      <c r="G132" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>2025-01-27 10:53:20</t>
+        </is>
+      </c>
+      <c r="B133" t="n">
+        <v>27977</v>
+      </c>
+      <c r="C133" t="n">
+        <v>0</v>
+      </c>
+      <c r="D133" t="n">
+        <v>0</v>
+      </c>
+      <c r="E133" t="n">
+        <v>0</v>
+      </c>
+      <c r="F133" t="n">
+        <v>4199</v>
+      </c>
+      <c r="G133" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Trying to get NA rows put in for where there is no match
</commit_message>
<xml_diff>
--- a/LOC tracking outputs/code_metrics.xlsx
+++ b/LOC tracking outputs/code_metrics.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G133"/>
+  <dimension ref="A1:G143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3549,6 +3549,236 @@
       </c>
       <c r="G133" t="inlineStr"/>
     </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>2024-12-12 15:01:02</t>
+        </is>
+      </c>
+      <c r="B134" t="n">
+        <v>9125</v>
+      </c>
+      <c r="C134" t="n">
+        <v>0</v>
+      </c>
+      <c r="D134" t="n">
+        <v>0</v>
+      </c>
+      <c r="E134" t="n">
+        <v>0</v>
+      </c>
+      <c r="F134" t="n">
+        <v>2778</v>
+      </c>
+      <c r="G134" t="inlineStr"/>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>2024-12-17 09:34:39</t>
+        </is>
+      </c>
+      <c r="B135" t="n">
+        <v>9392</v>
+      </c>
+      <c r="C135" t="n">
+        <v>0</v>
+      </c>
+      <c r="D135" t="n">
+        <v>0</v>
+      </c>
+      <c r="E135" t="n">
+        <v>0</v>
+      </c>
+      <c r="F135" t="n">
+        <v>2867</v>
+      </c>
+      <c r="G135" t="inlineStr"/>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>2024-12-20 13:39:15</t>
+        </is>
+      </c>
+      <c r="B136" t="n">
+        <v>11609</v>
+      </c>
+      <c r="C136" t="n">
+        <v>0</v>
+      </c>
+      <c r="D136" t="n">
+        <v>0</v>
+      </c>
+      <c r="E136" t="n">
+        <v>0</v>
+      </c>
+      <c r="F136" t="n">
+        <v>3086</v>
+      </c>
+      <c r="G136" t="inlineStr"/>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>2024-12-20 13:41:02</t>
+        </is>
+      </c>
+      <c r="B137" t="n">
+        <v>11609</v>
+      </c>
+      <c r="C137" t="n">
+        <v>0</v>
+      </c>
+      <c r="D137" t="n">
+        <v>0</v>
+      </c>
+      <c r="E137" t="n">
+        <v>0</v>
+      </c>
+      <c r="F137" t="n">
+        <v>3086</v>
+      </c>
+      <c r="G137" t="inlineStr"/>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>2025-01-16 14:58:07</t>
+        </is>
+      </c>
+      <c r="B138" t="n">
+        <v>12131</v>
+      </c>
+      <c r="C138" t="n">
+        <v>0</v>
+      </c>
+      <c r="D138" t="n">
+        <v>0</v>
+      </c>
+      <c r="E138" t="n">
+        <v>0</v>
+      </c>
+      <c r="F138" t="n">
+        <v>3277</v>
+      </c>
+      <c r="G138" t="inlineStr"/>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>2025-01-16 15:00:07</t>
+        </is>
+      </c>
+      <c r="B139" t="n">
+        <v>12131</v>
+      </c>
+      <c r="C139" t="n">
+        <v>0</v>
+      </c>
+      <c r="D139" t="n">
+        <v>0</v>
+      </c>
+      <c r="E139" t="n">
+        <v>0</v>
+      </c>
+      <c r="F139" t="n">
+        <v>3277</v>
+      </c>
+      <c r="G139" t="inlineStr"/>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>2025-01-21 15:00:05</t>
+        </is>
+      </c>
+      <c r="B140" t="n">
+        <v>14226</v>
+      </c>
+      <c r="C140" t="n">
+        <v>0</v>
+      </c>
+      <c r="D140" t="n">
+        <v>0</v>
+      </c>
+      <c r="E140" t="n">
+        <v>0</v>
+      </c>
+      <c r="F140" t="n">
+        <v>3357</v>
+      </c>
+      <c r="G140" t="inlineStr"/>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>2025-01-24 08:09:58</t>
+        </is>
+      </c>
+      <c r="B141" t="n">
+        <v>15227</v>
+      </c>
+      <c r="C141" t="n">
+        <v>0</v>
+      </c>
+      <c r="D141" t="n">
+        <v>0</v>
+      </c>
+      <c r="E141" t="n">
+        <v>0</v>
+      </c>
+      <c r="F141" t="n">
+        <v>3478</v>
+      </c>
+      <c r="G141" t="inlineStr"/>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>2025-01-27 10:53:20</t>
+        </is>
+      </c>
+      <c r="B142" t="n">
+        <v>27977</v>
+      </c>
+      <c r="C142" t="n">
+        <v>0</v>
+      </c>
+      <c r="D142" t="n">
+        <v>0</v>
+      </c>
+      <c r="E142" t="n">
+        <v>0</v>
+      </c>
+      <c r="F142" t="n">
+        <v>4199</v>
+      </c>
+      <c r="G142" t="inlineStr"/>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>2025-01-27 13:41:55</t>
+        </is>
+      </c>
+      <c r="B143" t="n">
+        <v>28113</v>
+      </c>
+      <c r="C143" t="n">
+        <v>0</v>
+      </c>
+      <c r="D143" t="n">
+        <v>0</v>
+      </c>
+      <c r="E143" t="n">
+        <v>0</v>
+      </c>
+      <c r="F143" t="n">
+        <v>4233</v>
+      </c>
+      <c r="G143" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Need to finish crude filters
</commit_message>
<xml_diff>
--- a/LOC tracking outputs/code_metrics.xlsx
+++ b/LOC tracking outputs/code_metrics.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G143"/>
+  <dimension ref="A1:G144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3779,6 +3779,29 @@
       </c>
       <c r="G143" t="inlineStr"/>
     </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>2025-01-27 21:06:55</t>
+        </is>
+      </c>
+      <c r="B144" t="n">
+        <v>18461</v>
+      </c>
+      <c r="C144" t="n">
+        <v>0</v>
+      </c>
+      <c r="D144" t="n">
+        <v>0</v>
+      </c>
+      <c r="E144" t="n">
+        <v>0</v>
+      </c>
+      <c r="F144" t="n">
+        <v>4264</v>
+      </c>
+      <c r="G144" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Reordered to produce a standard report, then remove SIL features remaining later in the workflow. Need to reconfig the count non-zero rows to work on this now
</commit_message>
<xml_diff>
--- a/LOC tracking outputs/code_metrics.xlsx
+++ b/LOC tracking outputs/code_metrics.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G144"/>
+  <dimension ref="A1:G154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3802,6 +3802,236 @@
       </c>
       <c r="G144" t="inlineStr"/>
     </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>2024-12-17 09:34:39</t>
+        </is>
+      </c>
+      <c r="B145" t="n">
+        <v>9392</v>
+      </c>
+      <c r="C145" t="n">
+        <v>0</v>
+      </c>
+      <c r="D145" t="n">
+        <v>0</v>
+      </c>
+      <c r="E145" t="n">
+        <v>0</v>
+      </c>
+      <c r="F145" t="n">
+        <v>2867</v>
+      </c>
+      <c r="G145" t="inlineStr"/>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>2024-12-20 13:39:15</t>
+        </is>
+      </c>
+      <c r="B146" t="n">
+        <v>11609</v>
+      </c>
+      <c r="C146" t="n">
+        <v>0</v>
+      </c>
+      <c r="D146" t="n">
+        <v>0</v>
+      </c>
+      <c r="E146" t="n">
+        <v>0</v>
+      </c>
+      <c r="F146" t="n">
+        <v>3086</v>
+      </c>
+      <c r="G146" t="inlineStr"/>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>2024-12-20 13:41:02</t>
+        </is>
+      </c>
+      <c r="B147" t="n">
+        <v>11609</v>
+      </c>
+      <c r="C147" t="n">
+        <v>0</v>
+      </c>
+      <c r="D147" t="n">
+        <v>0</v>
+      </c>
+      <c r="E147" t="n">
+        <v>0</v>
+      </c>
+      <c r="F147" t="n">
+        <v>3086</v>
+      </c>
+      <c r="G147" t="inlineStr"/>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>2025-01-16 14:58:07</t>
+        </is>
+      </c>
+      <c r="B148" t="n">
+        <v>12131</v>
+      </c>
+      <c r="C148" t="n">
+        <v>0</v>
+      </c>
+      <c r="D148" t="n">
+        <v>0</v>
+      </c>
+      <c r="E148" t="n">
+        <v>0</v>
+      </c>
+      <c r="F148" t="n">
+        <v>3277</v>
+      </c>
+      <c r="G148" t="inlineStr"/>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>2025-01-16 15:00:07</t>
+        </is>
+      </c>
+      <c r="B149" t="n">
+        <v>12131</v>
+      </c>
+      <c r="C149" t="n">
+        <v>0</v>
+      </c>
+      <c r="D149" t="n">
+        <v>0</v>
+      </c>
+      <c r="E149" t="n">
+        <v>0</v>
+      </c>
+      <c r="F149" t="n">
+        <v>3277</v>
+      </c>
+      <c r="G149" t="inlineStr"/>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>2025-01-21 15:00:05</t>
+        </is>
+      </c>
+      <c r="B150" t="n">
+        <v>14226</v>
+      </c>
+      <c r="C150" t="n">
+        <v>0</v>
+      </c>
+      <c r="D150" t="n">
+        <v>0</v>
+      </c>
+      <c r="E150" t="n">
+        <v>0</v>
+      </c>
+      <c r="F150" t="n">
+        <v>3357</v>
+      </c>
+      <c r="G150" t="inlineStr"/>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>2025-01-24 08:09:58</t>
+        </is>
+      </c>
+      <c r="B151" t="n">
+        <v>15227</v>
+      </c>
+      <c r="C151" t="n">
+        <v>0</v>
+      </c>
+      <c r="D151" t="n">
+        <v>0</v>
+      </c>
+      <c r="E151" t="n">
+        <v>0</v>
+      </c>
+      <c r="F151" t="n">
+        <v>3478</v>
+      </c>
+      <c r="G151" t="inlineStr"/>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>2025-01-27 10:53:20</t>
+        </is>
+      </c>
+      <c r="B152" t="n">
+        <v>27977</v>
+      </c>
+      <c r="C152" t="n">
+        <v>0</v>
+      </c>
+      <c r="D152" t="n">
+        <v>0</v>
+      </c>
+      <c r="E152" t="n">
+        <v>0</v>
+      </c>
+      <c r="F152" t="n">
+        <v>4199</v>
+      </c>
+      <c r="G152" t="inlineStr"/>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>2025-01-27 13:41:55</t>
+        </is>
+      </c>
+      <c r="B153" t="n">
+        <v>28113</v>
+      </c>
+      <c r="C153" t="n">
+        <v>0</v>
+      </c>
+      <c r="D153" t="n">
+        <v>0</v>
+      </c>
+      <c r="E153" t="n">
+        <v>0</v>
+      </c>
+      <c r="F153" t="n">
+        <v>4233</v>
+      </c>
+      <c r="G153" t="inlineStr"/>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>2025-01-28 09:24:55</t>
+        </is>
+      </c>
+      <c r="B154" t="n">
+        <v>28736</v>
+      </c>
+      <c r="C154" t="n">
+        <v>0</v>
+      </c>
+      <c r="D154" t="n">
+        <v>0</v>
+      </c>
+      <c r="E154" t="n">
+        <v>0</v>
+      </c>
+      <c r="F154" t="n">
+        <v>4370</v>
+      </c>
+      <c r="G154" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Grouping working well - integrated into main
</commit_message>
<xml_diff>
--- a/LOC tracking outputs/code_metrics.xlsx
+++ b/LOC tracking outputs/code_metrics.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G154"/>
+  <dimension ref="A1:G164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4032,6 +4032,236 @@
       </c>
       <c r="G154" t="inlineStr"/>
     </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>2024-12-20 13:39:15</t>
+        </is>
+      </c>
+      <c r="B155" t="n">
+        <v>11609</v>
+      </c>
+      <c r="C155" t="n">
+        <v>0</v>
+      </c>
+      <c r="D155" t="n">
+        <v>0</v>
+      </c>
+      <c r="E155" t="n">
+        <v>0</v>
+      </c>
+      <c r="F155" t="n">
+        <v>3086</v>
+      </c>
+      <c r="G155" t="inlineStr"/>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>2024-12-20 13:41:02</t>
+        </is>
+      </c>
+      <c r="B156" t="n">
+        <v>11609</v>
+      </c>
+      <c r="C156" t="n">
+        <v>0</v>
+      </c>
+      <c r="D156" t="n">
+        <v>0</v>
+      </c>
+      <c r="E156" t="n">
+        <v>0</v>
+      </c>
+      <c r="F156" t="n">
+        <v>3086</v>
+      </c>
+      <c r="G156" t="inlineStr"/>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>2025-01-16 14:58:07</t>
+        </is>
+      </c>
+      <c r="B157" t="n">
+        <v>12131</v>
+      </c>
+      <c r="C157" t="n">
+        <v>0</v>
+      </c>
+      <c r="D157" t="n">
+        <v>0</v>
+      </c>
+      <c r="E157" t="n">
+        <v>0</v>
+      </c>
+      <c r="F157" t="n">
+        <v>3277</v>
+      </c>
+      <c r="G157" t="inlineStr"/>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>2025-01-16 15:00:07</t>
+        </is>
+      </c>
+      <c r="B158" t="n">
+        <v>12131</v>
+      </c>
+      <c r="C158" t="n">
+        <v>0</v>
+      </c>
+      <c r="D158" t="n">
+        <v>0</v>
+      </c>
+      <c r="E158" t="n">
+        <v>0</v>
+      </c>
+      <c r="F158" t="n">
+        <v>3277</v>
+      </c>
+      <c r="G158" t="inlineStr"/>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>2025-01-21 15:00:05</t>
+        </is>
+      </c>
+      <c r="B159" t="n">
+        <v>14226</v>
+      </c>
+      <c r="C159" t="n">
+        <v>0</v>
+      </c>
+      <c r="D159" t="n">
+        <v>0</v>
+      </c>
+      <c r="E159" t="n">
+        <v>0</v>
+      </c>
+      <c r="F159" t="n">
+        <v>3357</v>
+      </c>
+      <c r="G159" t="inlineStr"/>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>2025-01-24 08:09:58</t>
+        </is>
+      </c>
+      <c r="B160" t="n">
+        <v>15227</v>
+      </c>
+      <c r="C160" t="n">
+        <v>0</v>
+      </c>
+      <c r="D160" t="n">
+        <v>0</v>
+      </c>
+      <c r="E160" t="n">
+        <v>0</v>
+      </c>
+      <c r="F160" t="n">
+        <v>3478</v>
+      </c>
+      <c r="G160" t="inlineStr"/>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>2025-01-27 10:53:20</t>
+        </is>
+      </c>
+      <c r="B161" t="n">
+        <v>27977</v>
+      </c>
+      <c r="C161" t="n">
+        <v>0</v>
+      </c>
+      <c r="D161" t="n">
+        <v>0</v>
+      </c>
+      <c r="E161" t="n">
+        <v>0</v>
+      </c>
+      <c r="F161" t="n">
+        <v>4199</v>
+      </c>
+      <c r="G161" t="inlineStr"/>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>2025-01-27 13:41:55</t>
+        </is>
+      </c>
+      <c r="B162" t="n">
+        <v>28113</v>
+      </c>
+      <c r="C162" t="n">
+        <v>0</v>
+      </c>
+      <c r="D162" t="n">
+        <v>0</v>
+      </c>
+      <c r="E162" t="n">
+        <v>0</v>
+      </c>
+      <c r="F162" t="n">
+        <v>4233</v>
+      </c>
+      <c r="G162" t="inlineStr"/>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>2025-01-28 09:24:55</t>
+        </is>
+      </c>
+      <c r="B163" t="n">
+        <v>28736</v>
+      </c>
+      <c r="C163" t="n">
+        <v>0</v>
+      </c>
+      <c r="D163" t="n">
+        <v>0</v>
+      </c>
+      <c r="E163" t="n">
+        <v>0</v>
+      </c>
+      <c r="F163" t="n">
+        <v>4370</v>
+      </c>
+      <c r="G163" t="inlineStr"/>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>2025-01-28 15:20:47</t>
+        </is>
+      </c>
+      <c r="B164" t="n">
+        <v>28522</v>
+      </c>
+      <c r="C164" t="n">
+        <v>0</v>
+      </c>
+      <c r="D164" t="n">
+        <v>0</v>
+      </c>
+      <c r="E164" t="n">
+        <v>0</v>
+      </c>
+      <c r="F164" t="n">
+        <v>4461</v>
+      </c>
+      <c r="G164" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Done until after bible study - cleaning tree
</commit_message>
<xml_diff>
--- a/LOC tracking outputs/code_metrics.xlsx
+++ b/LOC tracking outputs/code_metrics.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G164"/>
+  <dimension ref="A1:G174"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4262,6 +4262,236 @@
       </c>
       <c r="G164" t="inlineStr"/>
     </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>2024-12-20 13:41:02</t>
+        </is>
+      </c>
+      <c r="B165" t="n">
+        <v>11609</v>
+      </c>
+      <c r="C165" t="n">
+        <v>0</v>
+      </c>
+      <c r="D165" t="n">
+        <v>0</v>
+      </c>
+      <c r="E165" t="n">
+        <v>0</v>
+      </c>
+      <c r="F165" t="n">
+        <v>3086</v>
+      </c>
+      <c r="G165" t="inlineStr"/>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>2025-01-16 14:58:07</t>
+        </is>
+      </c>
+      <c r="B166" t="n">
+        <v>12131</v>
+      </c>
+      <c r="C166" t="n">
+        <v>0</v>
+      </c>
+      <c r="D166" t="n">
+        <v>0</v>
+      </c>
+      <c r="E166" t="n">
+        <v>0</v>
+      </c>
+      <c r="F166" t="n">
+        <v>3277</v>
+      </c>
+      <c r="G166" t="inlineStr"/>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>2025-01-16 15:00:07</t>
+        </is>
+      </c>
+      <c r="B167" t="n">
+        <v>12131</v>
+      </c>
+      <c r="C167" t="n">
+        <v>0</v>
+      </c>
+      <c r="D167" t="n">
+        <v>0</v>
+      </c>
+      <c r="E167" t="n">
+        <v>0</v>
+      </c>
+      <c r="F167" t="n">
+        <v>3277</v>
+      </c>
+      <c r="G167" t="inlineStr"/>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>2025-01-21 15:00:05</t>
+        </is>
+      </c>
+      <c r="B168" t="n">
+        <v>14226</v>
+      </c>
+      <c r="C168" t="n">
+        <v>0</v>
+      </c>
+      <c r="D168" t="n">
+        <v>0</v>
+      </c>
+      <c r="E168" t="n">
+        <v>0</v>
+      </c>
+      <c r="F168" t="n">
+        <v>3357</v>
+      </c>
+      <c r="G168" t="inlineStr"/>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>2025-01-24 08:09:58</t>
+        </is>
+      </c>
+      <c r="B169" t="n">
+        <v>15227</v>
+      </c>
+      <c r="C169" t="n">
+        <v>0</v>
+      </c>
+      <c r="D169" t="n">
+        <v>0</v>
+      </c>
+      <c r="E169" t="n">
+        <v>0</v>
+      </c>
+      <c r="F169" t="n">
+        <v>3478</v>
+      </c>
+      <c r="G169" t="inlineStr"/>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>2025-01-27 10:53:20</t>
+        </is>
+      </c>
+      <c r="B170" t="n">
+        <v>27977</v>
+      </c>
+      <c r="C170" t="n">
+        <v>0</v>
+      </c>
+      <c r="D170" t="n">
+        <v>0</v>
+      </c>
+      <c r="E170" t="n">
+        <v>0</v>
+      </c>
+      <c r="F170" t="n">
+        <v>4199</v>
+      </c>
+      <c r="G170" t="inlineStr"/>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>2025-01-27 13:41:55</t>
+        </is>
+      </c>
+      <c r="B171" t="n">
+        <v>28113</v>
+      </c>
+      <c r="C171" t="n">
+        <v>0</v>
+      </c>
+      <c r="D171" t="n">
+        <v>0</v>
+      </c>
+      <c r="E171" t="n">
+        <v>0</v>
+      </c>
+      <c r="F171" t="n">
+        <v>4233</v>
+      </c>
+      <c r="G171" t="inlineStr"/>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>2025-01-28 09:24:55</t>
+        </is>
+      </c>
+      <c r="B172" t="n">
+        <v>28736</v>
+      </c>
+      <c r="C172" t="n">
+        <v>0</v>
+      </c>
+      <c r="D172" t="n">
+        <v>0</v>
+      </c>
+      <c r="E172" t="n">
+        <v>0</v>
+      </c>
+      <c r="F172" t="n">
+        <v>4370</v>
+      </c>
+      <c r="G172" t="inlineStr"/>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>2025-01-28 15:20:47</t>
+        </is>
+      </c>
+      <c r="B173" t="n">
+        <v>28522</v>
+      </c>
+      <c r="C173" t="n">
+        <v>0</v>
+      </c>
+      <c r="D173" t="n">
+        <v>0</v>
+      </c>
+      <c r="E173" t="n">
+        <v>0</v>
+      </c>
+      <c r="F173" t="n">
+        <v>4461</v>
+      </c>
+      <c r="G173" t="inlineStr"/>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>2025-01-28 16:27:40</t>
+        </is>
+      </c>
+      <c r="B174" t="n">
+        <v>28946</v>
+      </c>
+      <c r="C174" t="n">
+        <v>0</v>
+      </c>
+      <c r="D174" t="n">
+        <v>0</v>
+      </c>
+      <c r="E174" t="n">
+        <v>0</v>
+      </c>
+      <c r="F174" t="n">
+        <v>4567</v>
+      </c>
+      <c r="G174" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Working with RT matching being an option for the standards comparison
</commit_message>
<xml_diff>
--- a/LOC tracking outputs/code_metrics.xlsx
+++ b/LOC tracking outputs/code_metrics.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G176"/>
+  <dimension ref="A1:G186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4538,6 +4538,236 @@
       </c>
       <c r="G176" t="inlineStr"/>
     </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>2025-01-16 14:58:07</t>
+        </is>
+      </c>
+      <c r="B177" t="n">
+        <v>12131</v>
+      </c>
+      <c r="C177" t="n">
+        <v>0</v>
+      </c>
+      <c r="D177" t="n">
+        <v>0</v>
+      </c>
+      <c r="E177" t="n">
+        <v>0</v>
+      </c>
+      <c r="F177" t="n">
+        <v>3277</v>
+      </c>
+      <c r="G177" t="inlineStr"/>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>2025-01-16 15:00:07</t>
+        </is>
+      </c>
+      <c r="B178" t="n">
+        <v>12131</v>
+      </c>
+      <c r="C178" t="n">
+        <v>0</v>
+      </c>
+      <c r="D178" t="n">
+        <v>0</v>
+      </c>
+      <c r="E178" t="n">
+        <v>0</v>
+      </c>
+      <c r="F178" t="n">
+        <v>3277</v>
+      </c>
+      <c r="G178" t="inlineStr"/>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>2025-01-21 15:00:05</t>
+        </is>
+      </c>
+      <c r="B179" t="n">
+        <v>14226</v>
+      </c>
+      <c r="C179" t="n">
+        <v>0</v>
+      </c>
+      <c r="D179" t="n">
+        <v>0</v>
+      </c>
+      <c r="E179" t="n">
+        <v>0</v>
+      </c>
+      <c r="F179" t="n">
+        <v>3357</v>
+      </c>
+      <c r="G179" t="inlineStr"/>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>2025-01-24 08:09:58</t>
+        </is>
+      </c>
+      <c r="B180" t="n">
+        <v>15227</v>
+      </c>
+      <c r="C180" t="n">
+        <v>0</v>
+      </c>
+      <c r="D180" t="n">
+        <v>0</v>
+      </c>
+      <c r="E180" t="n">
+        <v>0</v>
+      </c>
+      <c r="F180" t="n">
+        <v>3478</v>
+      </c>
+      <c r="G180" t="inlineStr"/>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>2025-01-27 10:53:20</t>
+        </is>
+      </c>
+      <c r="B181" t="n">
+        <v>27977</v>
+      </c>
+      <c r="C181" t="n">
+        <v>0</v>
+      </c>
+      <c r="D181" t="n">
+        <v>0</v>
+      </c>
+      <c r="E181" t="n">
+        <v>0</v>
+      </c>
+      <c r="F181" t="n">
+        <v>4199</v>
+      </c>
+      <c r="G181" t="inlineStr"/>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>2025-01-27 13:41:55</t>
+        </is>
+      </c>
+      <c r="B182" t="n">
+        <v>28113</v>
+      </c>
+      <c r="C182" t="n">
+        <v>0</v>
+      </c>
+      <c r="D182" t="n">
+        <v>0</v>
+      </c>
+      <c r="E182" t="n">
+        <v>0</v>
+      </c>
+      <c r="F182" t="n">
+        <v>4233</v>
+      </c>
+      <c r="G182" t="inlineStr"/>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>2025-01-28 09:24:55</t>
+        </is>
+      </c>
+      <c r="B183" t="n">
+        <v>28736</v>
+      </c>
+      <c r="C183" t="n">
+        <v>0</v>
+      </c>
+      <c r="D183" t="n">
+        <v>0</v>
+      </c>
+      <c r="E183" t="n">
+        <v>0</v>
+      </c>
+      <c r="F183" t="n">
+        <v>4370</v>
+      </c>
+      <c r="G183" t="inlineStr"/>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>2025-01-28 15:20:47</t>
+        </is>
+      </c>
+      <c r="B184" t="n">
+        <v>28522</v>
+      </c>
+      <c r="C184" t="n">
+        <v>0</v>
+      </c>
+      <c r="D184" t="n">
+        <v>0</v>
+      </c>
+      <c r="E184" t="n">
+        <v>0</v>
+      </c>
+      <c r="F184" t="n">
+        <v>4461</v>
+      </c>
+      <c r="G184" t="inlineStr"/>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>2025-01-28 16:27:40</t>
+        </is>
+      </c>
+      <c r="B185" t="n">
+        <v>28946</v>
+      </c>
+      <c r="C185" t="n">
+        <v>0</v>
+      </c>
+      <c r="D185" t="n">
+        <v>0</v>
+      </c>
+      <c r="E185" t="n">
+        <v>0</v>
+      </c>
+      <c r="F185" t="n">
+        <v>4567</v>
+      </c>
+      <c r="G185" t="inlineStr"/>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>2025-01-29 09:32:47</t>
+        </is>
+      </c>
+      <c r="B186" t="n">
+        <v>35054</v>
+      </c>
+      <c r="C186" t="n">
+        <v>0</v>
+      </c>
+      <c r="D186" t="n">
+        <v>0</v>
+      </c>
+      <c r="E186" t="n">
+        <v>0</v>
+      </c>
+      <c r="F186" t="n">
+        <v>4741</v>
+      </c>
+      <c r="G186" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated to include 1.29.25 powerpoint
</commit_message>
<xml_diff>
--- a/LOC tracking outputs/code_metrics.xlsx
+++ b/LOC tracking outputs/code_metrics.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G186"/>
+  <dimension ref="A1:G196"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4768,6 +4768,236 @@
       </c>
       <c r="G186" t="inlineStr"/>
     </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>2025-01-16 15:00:07</t>
+        </is>
+      </c>
+      <c r="B187" t="n">
+        <v>12131</v>
+      </c>
+      <c r="C187" t="n">
+        <v>0</v>
+      </c>
+      <c r="D187" t="n">
+        <v>0</v>
+      </c>
+      <c r="E187" t="n">
+        <v>0</v>
+      </c>
+      <c r="F187" t="n">
+        <v>3277</v>
+      </c>
+      <c r="G187" t="inlineStr"/>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>2025-01-21 15:00:05</t>
+        </is>
+      </c>
+      <c r="B188" t="n">
+        <v>14226</v>
+      </c>
+      <c r="C188" t="n">
+        <v>0</v>
+      </c>
+      <c r="D188" t="n">
+        <v>0</v>
+      </c>
+      <c r="E188" t="n">
+        <v>0</v>
+      </c>
+      <c r="F188" t="n">
+        <v>3357</v>
+      </c>
+      <c r="G188" t="inlineStr"/>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>2025-01-24 08:09:58</t>
+        </is>
+      </c>
+      <c r="B189" t="n">
+        <v>15227</v>
+      </c>
+      <c r="C189" t="n">
+        <v>0</v>
+      </c>
+      <c r="D189" t="n">
+        <v>0</v>
+      </c>
+      <c r="E189" t="n">
+        <v>0</v>
+      </c>
+      <c r="F189" t="n">
+        <v>3478</v>
+      </c>
+      <c r="G189" t="inlineStr"/>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>2025-01-27 10:53:20</t>
+        </is>
+      </c>
+      <c r="B190" t="n">
+        <v>27977</v>
+      </c>
+      <c r="C190" t="n">
+        <v>0</v>
+      </c>
+      <c r="D190" t="n">
+        <v>0</v>
+      </c>
+      <c r="E190" t="n">
+        <v>0</v>
+      </c>
+      <c r="F190" t="n">
+        <v>4199</v>
+      </c>
+      <c r="G190" t="inlineStr"/>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>2025-01-27 13:41:55</t>
+        </is>
+      </c>
+      <c r="B191" t="n">
+        <v>28113</v>
+      </c>
+      <c r="C191" t="n">
+        <v>0</v>
+      </c>
+      <c r="D191" t="n">
+        <v>0</v>
+      </c>
+      <c r="E191" t="n">
+        <v>0</v>
+      </c>
+      <c r="F191" t="n">
+        <v>4233</v>
+      </c>
+      <c r="G191" t="inlineStr"/>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>2025-01-28 09:24:55</t>
+        </is>
+      </c>
+      <c r="B192" t="n">
+        <v>28736</v>
+      </c>
+      <c r="C192" t="n">
+        <v>0</v>
+      </c>
+      <c r="D192" t="n">
+        <v>0</v>
+      </c>
+      <c r="E192" t="n">
+        <v>0</v>
+      </c>
+      <c r="F192" t="n">
+        <v>4370</v>
+      </c>
+      <c r="G192" t="inlineStr"/>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>2025-01-28 15:20:47</t>
+        </is>
+      </c>
+      <c r="B193" t="n">
+        <v>28522</v>
+      </c>
+      <c r="C193" t="n">
+        <v>0</v>
+      </c>
+      <c r="D193" t="n">
+        <v>0</v>
+      </c>
+      <c r="E193" t="n">
+        <v>0</v>
+      </c>
+      <c r="F193" t="n">
+        <v>4461</v>
+      </c>
+      <c r="G193" t="inlineStr"/>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>2025-01-28 16:27:40</t>
+        </is>
+      </c>
+      <c r="B194" t="n">
+        <v>28946</v>
+      </c>
+      <c r="C194" t="n">
+        <v>0</v>
+      </c>
+      <c r="D194" t="n">
+        <v>0</v>
+      </c>
+      <c r="E194" t="n">
+        <v>0</v>
+      </c>
+      <c r="F194" t="n">
+        <v>4567</v>
+      </c>
+      <c r="G194" t="inlineStr"/>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>2025-01-29 09:32:47</t>
+        </is>
+      </c>
+      <c r="B195" t="n">
+        <v>35054</v>
+      </c>
+      <c r="C195" t="n">
+        <v>0</v>
+      </c>
+      <c r="D195" t="n">
+        <v>0</v>
+      </c>
+      <c r="E195" t="n">
+        <v>0</v>
+      </c>
+      <c r="F195" t="n">
+        <v>4741</v>
+      </c>
+      <c r="G195" t="inlineStr"/>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>2025-01-29 15:15:52</t>
+        </is>
+      </c>
+      <c r="B196" t="n">
+        <v>38441</v>
+      </c>
+      <c r="C196" t="n">
+        <v>0</v>
+      </c>
+      <c r="D196" t="n">
+        <v>0</v>
+      </c>
+      <c r="E196" t="n">
+        <v>0</v>
+      </c>
+      <c r="F196" t="n">
+        <v>4946</v>
+      </c>
+      <c r="G196" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Working code with reading the csv
</commit_message>
<xml_diff>
--- a/LOC tracking outputs/code_metrics.xlsx
+++ b/LOC tracking outputs/code_metrics.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G196"/>
+  <dimension ref="A1:G236"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4998,6 +4998,926 @@
       </c>
       <c r="G196" t="inlineStr"/>
     </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>2025-01-21 15:00:05</t>
+        </is>
+      </c>
+      <c r="B197" t="n">
+        <v>14226</v>
+      </c>
+      <c r="C197" t="n">
+        <v>0</v>
+      </c>
+      <c r="D197" t="n">
+        <v>0</v>
+      </c>
+      <c r="E197" t="n">
+        <v>0</v>
+      </c>
+      <c r="F197" t="n">
+        <v>3357</v>
+      </c>
+      <c r="G197" t="inlineStr"/>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>2025-01-24 08:09:58</t>
+        </is>
+      </c>
+      <c r="B198" t="n">
+        <v>15227</v>
+      </c>
+      <c r="C198" t="n">
+        <v>0</v>
+      </c>
+      <c r="D198" t="n">
+        <v>0</v>
+      </c>
+      <c r="E198" t="n">
+        <v>0</v>
+      </c>
+      <c r="F198" t="n">
+        <v>3478</v>
+      </c>
+      <c r="G198" t="inlineStr"/>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>2025-01-27 10:53:20</t>
+        </is>
+      </c>
+      <c r="B199" t="n">
+        <v>27977</v>
+      </c>
+      <c r="C199" t="n">
+        <v>0</v>
+      </c>
+      <c r="D199" t="n">
+        <v>0</v>
+      </c>
+      <c r="E199" t="n">
+        <v>0</v>
+      </c>
+      <c r="F199" t="n">
+        <v>4199</v>
+      </c>
+      <c r="G199" t="inlineStr"/>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>2025-01-27 13:41:55</t>
+        </is>
+      </c>
+      <c r="B200" t="n">
+        <v>28113</v>
+      </c>
+      <c r="C200" t="n">
+        <v>0</v>
+      </c>
+      <c r="D200" t="n">
+        <v>0</v>
+      </c>
+      <c r="E200" t="n">
+        <v>0</v>
+      </c>
+      <c r="F200" t="n">
+        <v>4233</v>
+      </c>
+      <c r="G200" t="inlineStr"/>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>2025-01-28 09:24:55</t>
+        </is>
+      </c>
+      <c r="B201" t="n">
+        <v>28736</v>
+      </c>
+      <c r="C201" t="n">
+        <v>0</v>
+      </c>
+      <c r="D201" t="n">
+        <v>0</v>
+      </c>
+      <c r="E201" t="n">
+        <v>0</v>
+      </c>
+      <c r="F201" t="n">
+        <v>4370</v>
+      </c>
+      <c r="G201" t="inlineStr"/>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>2025-01-28 15:20:47</t>
+        </is>
+      </c>
+      <c r="B202" t="n">
+        <v>28522</v>
+      </c>
+      <c r="C202" t="n">
+        <v>0</v>
+      </c>
+      <c r="D202" t="n">
+        <v>0</v>
+      </c>
+      <c r="E202" t="n">
+        <v>0</v>
+      </c>
+      <c r="F202" t="n">
+        <v>4461</v>
+      </c>
+      <c r="G202" t="inlineStr"/>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>2025-01-28 16:27:40</t>
+        </is>
+      </c>
+      <c r="B203" t="n">
+        <v>28946</v>
+      </c>
+      <c r="C203" t="n">
+        <v>0</v>
+      </c>
+      <c r="D203" t="n">
+        <v>0</v>
+      </c>
+      <c r="E203" t="n">
+        <v>0</v>
+      </c>
+      <c r="F203" t="n">
+        <v>4567</v>
+      </c>
+      <c r="G203" t="inlineStr"/>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>2025-01-29 09:32:47</t>
+        </is>
+      </c>
+      <c r="B204" t="n">
+        <v>35054</v>
+      </c>
+      <c r="C204" t="n">
+        <v>0</v>
+      </c>
+      <c r="D204" t="n">
+        <v>0</v>
+      </c>
+      <c r="E204" t="n">
+        <v>0</v>
+      </c>
+      <c r="F204" t="n">
+        <v>4741</v>
+      </c>
+      <c r="G204" t="inlineStr"/>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>2025-01-29 15:15:52</t>
+        </is>
+      </c>
+      <c r="B205" t="n">
+        <v>38441</v>
+      </c>
+      <c r="C205" t="n">
+        <v>0</v>
+      </c>
+      <c r="D205" t="n">
+        <v>0</v>
+      </c>
+      <c r="E205" t="n">
+        <v>0</v>
+      </c>
+      <c r="F205" t="n">
+        <v>4946</v>
+      </c>
+      <c r="G205" t="inlineStr"/>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>2025-01-31 14:19:46</t>
+        </is>
+      </c>
+      <c r="B206" t="n">
+        <v>36066</v>
+      </c>
+      <c r="C206" t="n">
+        <v>0</v>
+      </c>
+      <c r="D206" t="n">
+        <v>0</v>
+      </c>
+      <c r="E206" t="n">
+        <v>0</v>
+      </c>
+      <c r="F206" t="n">
+        <v>5073</v>
+      </c>
+      <c r="G206" t="inlineStr"/>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>2025-01-21 15:00:05</t>
+        </is>
+      </c>
+      <c r="B207" t="n">
+        <v>14226</v>
+      </c>
+      <c r="C207" t="n">
+        <v>0</v>
+      </c>
+      <c r="D207" t="n">
+        <v>0</v>
+      </c>
+      <c r="E207" t="n">
+        <v>0</v>
+      </c>
+      <c r="F207" t="n">
+        <v>3357</v>
+      </c>
+      <c r="G207" t="inlineStr"/>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>2025-01-24 08:09:58</t>
+        </is>
+      </c>
+      <c r="B208" t="n">
+        <v>15227</v>
+      </c>
+      <c r="C208" t="n">
+        <v>0</v>
+      </c>
+      <c r="D208" t="n">
+        <v>0</v>
+      </c>
+      <c r="E208" t="n">
+        <v>0</v>
+      </c>
+      <c r="F208" t="n">
+        <v>3478</v>
+      </c>
+      <c r="G208" t="inlineStr"/>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>2025-01-27 10:53:20</t>
+        </is>
+      </c>
+      <c r="B209" t="n">
+        <v>27977</v>
+      </c>
+      <c r="C209" t="n">
+        <v>0</v>
+      </c>
+      <c r="D209" t="n">
+        <v>0</v>
+      </c>
+      <c r="E209" t="n">
+        <v>0</v>
+      </c>
+      <c r="F209" t="n">
+        <v>4199</v>
+      </c>
+      <c r="G209" t="inlineStr"/>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>2025-01-27 13:41:55</t>
+        </is>
+      </c>
+      <c r="B210" t="n">
+        <v>28113</v>
+      </c>
+      <c r="C210" t="n">
+        <v>0</v>
+      </c>
+      <c r="D210" t="n">
+        <v>0</v>
+      </c>
+      <c r="E210" t="n">
+        <v>0</v>
+      </c>
+      <c r="F210" t="n">
+        <v>4233</v>
+      </c>
+      <c r="G210" t="inlineStr"/>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>2025-01-28 09:24:55</t>
+        </is>
+      </c>
+      <c r="B211" t="n">
+        <v>28736</v>
+      </c>
+      <c r="C211" t="n">
+        <v>0</v>
+      </c>
+      <c r="D211" t="n">
+        <v>0</v>
+      </c>
+      <c r="E211" t="n">
+        <v>0</v>
+      </c>
+      <c r="F211" t="n">
+        <v>4370</v>
+      </c>
+      <c r="G211" t="inlineStr"/>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>2025-01-28 15:20:47</t>
+        </is>
+      </c>
+      <c r="B212" t="n">
+        <v>28522</v>
+      </c>
+      <c r="C212" t="n">
+        <v>0</v>
+      </c>
+      <c r="D212" t="n">
+        <v>0</v>
+      </c>
+      <c r="E212" t="n">
+        <v>0</v>
+      </c>
+      <c r="F212" t="n">
+        <v>4461</v>
+      </c>
+      <c r="G212" t="inlineStr"/>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>2025-01-28 16:27:40</t>
+        </is>
+      </c>
+      <c r="B213" t="n">
+        <v>28946</v>
+      </c>
+      <c r="C213" t="n">
+        <v>0</v>
+      </c>
+      <c r="D213" t="n">
+        <v>0</v>
+      </c>
+      <c r="E213" t="n">
+        <v>0</v>
+      </c>
+      <c r="F213" t="n">
+        <v>4567</v>
+      </c>
+      <c r="G213" t="inlineStr"/>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>2025-01-29 09:32:47</t>
+        </is>
+      </c>
+      <c r="B214" t="n">
+        <v>35054</v>
+      </c>
+      <c r="C214" t="n">
+        <v>0</v>
+      </c>
+      <c r="D214" t="n">
+        <v>0</v>
+      </c>
+      <c r="E214" t="n">
+        <v>0</v>
+      </c>
+      <c r="F214" t="n">
+        <v>4741</v>
+      </c>
+      <c r="G214" t="inlineStr"/>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>2025-01-29 15:15:52</t>
+        </is>
+      </c>
+      <c r="B215" t="n">
+        <v>38441</v>
+      </c>
+      <c r="C215" t="n">
+        <v>0</v>
+      </c>
+      <c r="D215" t="n">
+        <v>0</v>
+      </c>
+      <c r="E215" t="n">
+        <v>0</v>
+      </c>
+      <c r="F215" t="n">
+        <v>4946</v>
+      </c>
+      <c r="G215" t="inlineStr"/>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>2025-01-31 14:19:46</t>
+        </is>
+      </c>
+      <c r="B216" t="n">
+        <v>36066</v>
+      </c>
+      <c r="C216" t="n">
+        <v>0</v>
+      </c>
+      <c r="D216" t="n">
+        <v>0</v>
+      </c>
+      <c r="E216" t="n">
+        <v>0</v>
+      </c>
+      <c r="F216" t="n">
+        <v>5073</v>
+      </c>
+      <c r="G216" t="inlineStr"/>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>2025-01-21 15:00:05</t>
+        </is>
+      </c>
+      <c r="B217" t="n">
+        <v>14226</v>
+      </c>
+      <c r="C217" t="n">
+        <v>0</v>
+      </c>
+      <c r="D217" t="n">
+        <v>0</v>
+      </c>
+      <c r="E217" t="n">
+        <v>0</v>
+      </c>
+      <c r="F217" t="n">
+        <v>3357</v>
+      </c>
+      <c r="G217" t="inlineStr"/>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>2025-01-24 08:09:58</t>
+        </is>
+      </c>
+      <c r="B218" t="n">
+        <v>15227</v>
+      </c>
+      <c r="C218" t="n">
+        <v>0</v>
+      </c>
+      <c r="D218" t="n">
+        <v>0</v>
+      </c>
+      <c r="E218" t="n">
+        <v>0</v>
+      </c>
+      <c r="F218" t="n">
+        <v>3478</v>
+      </c>
+      <c r="G218" t="inlineStr"/>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>2025-01-27 10:53:20</t>
+        </is>
+      </c>
+      <c r="B219" t="n">
+        <v>27977</v>
+      </c>
+      <c r="C219" t="n">
+        <v>0</v>
+      </c>
+      <c r="D219" t="n">
+        <v>0</v>
+      </c>
+      <c r="E219" t="n">
+        <v>0</v>
+      </c>
+      <c r="F219" t="n">
+        <v>4199</v>
+      </c>
+      <c r="G219" t="inlineStr"/>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>2025-01-27 13:41:55</t>
+        </is>
+      </c>
+      <c r="B220" t="n">
+        <v>28113</v>
+      </c>
+      <c r="C220" t="n">
+        <v>0</v>
+      </c>
+      <c r="D220" t="n">
+        <v>0</v>
+      </c>
+      <c r="E220" t="n">
+        <v>0</v>
+      </c>
+      <c r="F220" t="n">
+        <v>4233</v>
+      </c>
+      <c r="G220" t="inlineStr"/>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>2025-01-28 09:24:55</t>
+        </is>
+      </c>
+      <c r="B221" t="n">
+        <v>28736</v>
+      </c>
+      <c r="C221" t="n">
+        <v>0</v>
+      </c>
+      <c r="D221" t="n">
+        <v>0</v>
+      </c>
+      <c r="E221" t="n">
+        <v>0</v>
+      </c>
+      <c r="F221" t="n">
+        <v>4370</v>
+      </c>
+      <c r="G221" t="inlineStr"/>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>2025-01-28 15:20:47</t>
+        </is>
+      </c>
+      <c r="B222" t="n">
+        <v>28522</v>
+      </c>
+      <c r="C222" t="n">
+        <v>0</v>
+      </c>
+      <c r="D222" t="n">
+        <v>0</v>
+      </c>
+      <c r="E222" t="n">
+        <v>0</v>
+      </c>
+      <c r="F222" t="n">
+        <v>4461</v>
+      </c>
+      <c r="G222" t="inlineStr"/>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>2025-01-28 16:27:40</t>
+        </is>
+      </c>
+      <c r="B223" t="n">
+        <v>28946</v>
+      </c>
+      <c r="C223" t="n">
+        <v>0</v>
+      </c>
+      <c r="D223" t="n">
+        <v>0</v>
+      </c>
+      <c r="E223" t="n">
+        <v>0</v>
+      </c>
+      <c r="F223" t="n">
+        <v>4567</v>
+      </c>
+      <c r="G223" t="inlineStr"/>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>2025-01-29 09:32:47</t>
+        </is>
+      </c>
+      <c r="B224" t="n">
+        <v>35054</v>
+      </c>
+      <c r="C224" t="n">
+        <v>0</v>
+      </c>
+      <c r="D224" t="n">
+        <v>0</v>
+      </c>
+      <c r="E224" t="n">
+        <v>0</v>
+      </c>
+      <c r="F224" t="n">
+        <v>4741</v>
+      </c>
+      <c r="G224" t="inlineStr"/>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>2025-01-29 15:15:52</t>
+        </is>
+      </c>
+      <c r="B225" t="n">
+        <v>38441</v>
+      </c>
+      <c r="C225" t="n">
+        <v>0</v>
+      </c>
+      <c r="D225" t="n">
+        <v>0</v>
+      </c>
+      <c r="E225" t="n">
+        <v>0</v>
+      </c>
+      <c r="F225" t="n">
+        <v>4946</v>
+      </c>
+      <c r="G225" t="inlineStr"/>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>2025-01-31 14:19:46</t>
+        </is>
+      </c>
+      <c r="B226" t="n">
+        <v>36066</v>
+      </c>
+      <c r="C226" t="n">
+        <v>0</v>
+      </c>
+      <c r="D226" t="n">
+        <v>0</v>
+      </c>
+      <c r="E226" t="n">
+        <v>0</v>
+      </c>
+      <c r="F226" t="n">
+        <v>5073</v>
+      </c>
+      <c r="G226" t="inlineStr"/>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>2025-01-21 15:00:05</t>
+        </is>
+      </c>
+      <c r="B227" t="n">
+        <v>14226</v>
+      </c>
+      <c r="C227" t="n">
+        <v>0</v>
+      </c>
+      <c r="D227" t="n">
+        <v>0</v>
+      </c>
+      <c r="E227" t="n">
+        <v>0</v>
+      </c>
+      <c r="F227" t="n">
+        <v>3357</v>
+      </c>
+      <c r="G227" t="inlineStr"/>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>2025-01-24 08:09:58</t>
+        </is>
+      </c>
+      <c r="B228" t="n">
+        <v>15227</v>
+      </c>
+      <c r="C228" t="n">
+        <v>0</v>
+      </c>
+      <c r="D228" t="n">
+        <v>0</v>
+      </c>
+      <c r="E228" t="n">
+        <v>0</v>
+      </c>
+      <c r="F228" t="n">
+        <v>3478</v>
+      </c>
+      <c r="G228" t="inlineStr"/>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>2025-01-27 10:53:20</t>
+        </is>
+      </c>
+      <c r="B229" t="n">
+        <v>27977</v>
+      </c>
+      <c r="C229" t="n">
+        <v>0</v>
+      </c>
+      <c r="D229" t="n">
+        <v>0</v>
+      </c>
+      <c r="E229" t="n">
+        <v>0</v>
+      </c>
+      <c r="F229" t="n">
+        <v>4199</v>
+      </c>
+      <c r="G229" t="inlineStr"/>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>2025-01-27 13:41:55</t>
+        </is>
+      </c>
+      <c r="B230" t="n">
+        <v>28113</v>
+      </c>
+      <c r="C230" t="n">
+        <v>0</v>
+      </c>
+      <c r="D230" t="n">
+        <v>0</v>
+      </c>
+      <c r="E230" t="n">
+        <v>0</v>
+      </c>
+      <c r="F230" t="n">
+        <v>4233</v>
+      </c>
+      <c r="G230" t="inlineStr"/>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>2025-01-28 09:24:55</t>
+        </is>
+      </c>
+      <c r="B231" t="n">
+        <v>28736</v>
+      </c>
+      <c r="C231" t="n">
+        <v>0</v>
+      </c>
+      <c r="D231" t="n">
+        <v>0</v>
+      </c>
+      <c r="E231" t="n">
+        <v>0</v>
+      </c>
+      <c r="F231" t="n">
+        <v>4370</v>
+      </c>
+      <c r="G231" t="inlineStr"/>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>2025-01-28 15:20:47</t>
+        </is>
+      </c>
+      <c r="B232" t="n">
+        <v>28522</v>
+      </c>
+      <c r="C232" t="n">
+        <v>0</v>
+      </c>
+      <c r="D232" t="n">
+        <v>0</v>
+      </c>
+      <c r="E232" t="n">
+        <v>0</v>
+      </c>
+      <c r="F232" t="n">
+        <v>4461</v>
+      </c>
+      <c r="G232" t="inlineStr"/>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>2025-01-28 16:27:40</t>
+        </is>
+      </c>
+      <c r="B233" t="n">
+        <v>28946</v>
+      </c>
+      <c r="C233" t="n">
+        <v>0</v>
+      </c>
+      <c r="D233" t="n">
+        <v>0</v>
+      </c>
+      <c r="E233" t="n">
+        <v>0</v>
+      </c>
+      <c r="F233" t="n">
+        <v>4567</v>
+      </c>
+      <c r="G233" t="inlineStr"/>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>2025-01-29 09:32:47</t>
+        </is>
+      </c>
+      <c r="B234" t="n">
+        <v>35054</v>
+      </c>
+      <c r="C234" t="n">
+        <v>0</v>
+      </c>
+      <c r="D234" t="n">
+        <v>0</v>
+      </c>
+      <c r="E234" t="n">
+        <v>0</v>
+      </c>
+      <c r="F234" t="n">
+        <v>4741</v>
+      </c>
+      <c r="G234" t="inlineStr"/>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>2025-01-29 15:15:52</t>
+        </is>
+      </c>
+      <c r="B235" t="n">
+        <v>38441</v>
+      </c>
+      <c r="C235" t="n">
+        <v>0</v>
+      </c>
+      <c r="D235" t="n">
+        <v>0</v>
+      </c>
+      <c r="E235" t="n">
+        <v>0</v>
+      </c>
+      <c r="F235" t="n">
+        <v>4946</v>
+      </c>
+      <c r="G235" t="inlineStr"/>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>2025-01-31 14:19:46</t>
+        </is>
+      </c>
+      <c r="B236" t="n">
+        <v>36066</v>
+      </c>
+      <c r="C236" t="n">
+        <v>0</v>
+      </c>
+      <c r="D236" t="n">
+        <v>0</v>
+      </c>
+      <c r="E236" t="n">
+        <v>0</v>
+      </c>
+      <c r="F236" t="n">
+        <v>5073</v>
+      </c>
+      <c r="G236" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Working selection and hiding of the different groups, still very buggy though
</commit_message>
<xml_diff>
--- a/LOC tracking outputs/code_metrics.xlsx
+++ b/LOC tracking outputs/code_metrics.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G236"/>
+  <dimension ref="A1:G239"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5918,6 +5918,75 @@
       </c>
       <c r="G236" t="inlineStr"/>
     </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>2025-01-27 21:06:55</t>
+        </is>
+      </c>
+      <c r="B237" t="n">
+        <v>18461</v>
+      </c>
+      <c r="C237" t="n">
+        <v>0</v>
+      </c>
+      <c r="D237" t="n">
+        <v>0</v>
+      </c>
+      <c r="E237" t="n">
+        <v>0</v>
+      </c>
+      <c r="F237" t="n">
+        <v>4264</v>
+      </c>
+      <c r="G237" t="inlineStr"/>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>2025-01-28 23:23:35</t>
+        </is>
+      </c>
+      <c r="B238" t="n">
+        <v>19566</v>
+      </c>
+      <c r="C238" t="n">
+        <v>0</v>
+      </c>
+      <c r="D238" t="n">
+        <v>0</v>
+      </c>
+      <c r="E238" t="n">
+        <v>0</v>
+      </c>
+      <c r="F238" t="n">
+        <v>4666</v>
+      </c>
+      <c r="G238" t="inlineStr"/>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>2025-02-03 20:54:27</t>
+        </is>
+      </c>
+      <c r="B239" t="n">
+        <v>37061</v>
+      </c>
+      <c r="C239" t="n">
+        <v>0</v>
+      </c>
+      <c r="D239" t="n">
+        <v>0</v>
+      </c>
+      <c r="E239" t="n">
+        <v>0</v>
+      </c>
+      <c r="F239" t="n">
+        <v>5358</v>
+      </c>
+      <c r="G239" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Everything working well, moving onto sample selection
</commit_message>
<xml_diff>
--- a/LOC tracking outputs/code_metrics.xlsx
+++ b/LOC tracking outputs/code_metrics.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G239"/>
+  <dimension ref="A1:G243"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5987,6 +5987,98 @@
       </c>
       <c r="G239" t="inlineStr"/>
     </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>2025-01-27 21:06:55</t>
+        </is>
+      </c>
+      <c r="B240" t="n">
+        <v>18461</v>
+      </c>
+      <c r="C240" t="n">
+        <v>0</v>
+      </c>
+      <c r="D240" t="n">
+        <v>0</v>
+      </c>
+      <c r="E240" t="n">
+        <v>0</v>
+      </c>
+      <c r="F240" t="n">
+        <v>4264</v>
+      </c>
+      <c r="G240" t="inlineStr"/>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>2025-01-28 23:23:35</t>
+        </is>
+      </c>
+      <c r="B241" t="n">
+        <v>19566</v>
+      </c>
+      <c r="C241" t="n">
+        <v>0</v>
+      </c>
+      <c r="D241" t="n">
+        <v>0</v>
+      </c>
+      <c r="E241" t="n">
+        <v>0</v>
+      </c>
+      <c r="F241" t="n">
+        <v>4666</v>
+      </c>
+      <c r="G241" t="inlineStr"/>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>2025-02-03 20:54:27</t>
+        </is>
+      </c>
+      <c r="B242" t="n">
+        <v>37061</v>
+      </c>
+      <c r="C242" t="n">
+        <v>0</v>
+      </c>
+      <c r="D242" t="n">
+        <v>0</v>
+      </c>
+      <c r="E242" t="n">
+        <v>0</v>
+      </c>
+      <c r="F242" t="n">
+        <v>5358</v>
+      </c>
+      <c r="G242" t="inlineStr"/>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>2025-02-04 13:00:53</t>
+        </is>
+      </c>
+      <c r="B243" t="n">
+        <v>37389</v>
+      </c>
+      <c r="C243" t="n">
+        <v>0</v>
+      </c>
+      <c r="D243" t="n">
+        <v>0</v>
+      </c>
+      <c r="E243" t="n">
+        <v>0</v>
+      </c>
+      <c r="F243" t="n">
+        <v>5440</v>
+      </c>
+      <c r="G243" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Deleted unnecessary definition of update graph
</commit_message>
<xml_diff>
--- a/LOC tracking outputs/code_metrics.xlsx
+++ b/LOC tracking outputs/code_metrics.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G243"/>
+  <dimension ref="A1:G253"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6079,6 +6079,236 @@
       </c>
       <c r="G243" t="inlineStr"/>
     </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>2025-01-27 10:53:20</t>
+        </is>
+      </c>
+      <c r="B244" t="n">
+        <v>27977</v>
+      </c>
+      <c r="C244" t="n">
+        <v>0</v>
+      </c>
+      <c r="D244" t="n">
+        <v>0</v>
+      </c>
+      <c r="E244" t="n">
+        <v>0</v>
+      </c>
+      <c r="F244" t="n">
+        <v>4199</v>
+      </c>
+      <c r="G244" t="inlineStr"/>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>2025-01-27 13:41:55</t>
+        </is>
+      </c>
+      <c r="B245" t="n">
+        <v>28113</v>
+      </c>
+      <c r="C245" t="n">
+        <v>0</v>
+      </c>
+      <c r="D245" t="n">
+        <v>0</v>
+      </c>
+      <c r="E245" t="n">
+        <v>0</v>
+      </c>
+      <c r="F245" t="n">
+        <v>4233</v>
+      </c>
+      <c r="G245" t="inlineStr"/>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>2025-01-28 09:24:55</t>
+        </is>
+      </c>
+      <c r="B246" t="n">
+        <v>28736</v>
+      </c>
+      <c r="C246" t="n">
+        <v>0</v>
+      </c>
+      <c r="D246" t="n">
+        <v>0</v>
+      </c>
+      <c r="E246" t="n">
+        <v>0</v>
+      </c>
+      <c r="F246" t="n">
+        <v>4370</v>
+      </c>
+      <c r="G246" t="inlineStr"/>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>2025-01-28 15:20:47</t>
+        </is>
+      </c>
+      <c r="B247" t="n">
+        <v>28522</v>
+      </c>
+      <c r="C247" t="n">
+        <v>0</v>
+      </c>
+      <c r="D247" t="n">
+        <v>0</v>
+      </c>
+      <c r="E247" t="n">
+        <v>0</v>
+      </c>
+      <c r="F247" t="n">
+        <v>4461</v>
+      </c>
+      <c r="G247" t="inlineStr"/>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>2025-01-28 16:27:40</t>
+        </is>
+      </c>
+      <c r="B248" t="n">
+        <v>28946</v>
+      </c>
+      <c r="C248" t="n">
+        <v>0</v>
+      </c>
+      <c r="D248" t="n">
+        <v>0</v>
+      </c>
+      <c r="E248" t="n">
+        <v>0</v>
+      </c>
+      <c r="F248" t="n">
+        <v>4567</v>
+      </c>
+      <c r="G248" t="inlineStr"/>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>2025-01-29 09:32:47</t>
+        </is>
+      </c>
+      <c r="B249" t="n">
+        <v>35054</v>
+      </c>
+      <c r="C249" t="n">
+        <v>0</v>
+      </c>
+      <c r="D249" t="n">
+        <v>0</v>
+      </c>
+      <c r="E249" t="n">
+        <v>0</v>
+      </c>
+      <c r="F249" t="n">
+        <v>4741</v>
+      </c>
+      <c r="G249" t="inlineStr"/>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>2025-01-29 15:15:52</t>
+        </is>
+      </c>
+      <c r="B250" t="n">
+        <v>38441</v>
+      </c>
+      <c r="C250" t="n">
+        <v>0</v>
+      </c>
+      <c r="D250" t="n">
+        <v>0</v>
+      </c>
+      <c r="E250" t="n">
+        <v>0</v>
+      </c>
+      <c r="F250" t="n">
+        <v>4946</v>
+      </c>
+      <c r="G250" t="inlineStr"/>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>2025-01-31 14:19:46</t>
+        </is>
+      </c>
+      <c r="B251" t="n">
+        <v>36066</v>
+      </c>
+      <c r="C251" t="n">
+        <v>0</v>
+      </c>
+      <c r="D251" t="n">
+        <v>0</v>
+      </c>
+      <c r="E251" t="n">
+        <v>0</v>
+      </c>
+      <c r="F251" t="n">
+        <v>5073</v>
+      </c>
+      <c r="G251" t="inlineStr"/>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>2025-01-31 18:30:54</t>
+        </is>
+      </c>
+      <c r="B252" t="n">
+        <v>36188</v>
+      </c>
+      <c r="C252" t="n">
+        <v>0</v>
+      </c>
+      <c r="D252" t="n">
+        <v>0</v>
+      </c>
+      <c r="E252" t="n">
+        <v>0</v>
+      </c>
+      <c r="F252" t="n">
+        <v>5060</v>
+      </c>
+      <c r="G252" t="inlineStr"/>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>2025-02-05 15:05:41</t>
+        </is>
+      </c>
+      <c r="B253" t="n">
+        <v>38127</v>
+      </c>
+      <c r="C253" t="n">
+        <v>0</v>
+      </c>
+      <c r="D253" t="n">
+        <v>0</v>
+      </c>
+      <c r="E253" t="n">
+        <v>0</v>
+      </c>
+      <c r="F253" t="n">
+        <v>5578</v>
+      </c>
+      <c r="G253" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Mass - only groups showing up well
</commit_message>
<xml_diff>
--- a/LOC tracking outputs/code_metrics.xlsx
+++ b/LOC tracking outputs/code_metrics.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G253"/>
+  <dimension ref="A1:G263"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6309,6 +6309,236 @@
       </c>
       <c r="G253" t="inlineStr"/>
     </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>2025-01-27 13:41:55</t>
+        </is>
+      </c>
+      <c r="B254" t="n">
+        <v>28113</v>
+      </c>
+      <c r="C254" t="n">
+        <v>0</v>
+      </c>
+      <c r="D254" t="n">
+        <v>0</v>
+      </c>
+      <c r="E254" t="n">
+        <v>0</v>
+      </c>
+      <c r="F254" t="n">
+        <v>4233</v>
+      </c>
+      <c r="G254" t="inlineStr"/>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>2025-01-28 09:24:55</t>
+        </is>
+      </c>
+      <c r="B255" t="n">
+        <v>28736</v>
+      </c>
+      <c r="C255" t="n">
+        <v>0</v>
+      </c>
+      <c r="D255" t="n">
+        <v>0</v>
+      </c>
+      <c r="E255" t="n">
+        <v>0</v>
+      </c>
+      <c r="F255" t="n">
+        <v>4370</v>
+      </c>
+      <c r="G255" t="inlineStr"/>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>2025-01-28 15:20:47</t>
+        </is>
+      </c>
+      <c r="B256" t="n">
+        <v>28522</v>
+      </c>
+      <c r="C256" t="n">
+        <v>0</v>
+      </c>
+      <c r="D256" t="n">
+        <v>0</v>
+      </c>
+      <c r="E256" t="n">
+        <v>0</v>
+      </c>
+      <c r="F256" t="n">
+        <v>4461</v>
+      </c>
+      <c r="G256" t="inlineStr"/>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>2025-01-28 16:27:40</t>
+        </is>
+      </c>
+      <c r="B257" t="n">
+        <v>28946</v>
+      </c>
+      <c r="C257" t="n">
+        <v>0</v>
+      </c>
+      <c r="D257" t="n">
+        <v>0</v>
+      </c>
+      <c r="E257" t="n">
+        <v>0</v>
+      </c>
+      <c r="F257" t="n">
+        <v>4567</v>
+      </c>
+      <c r="G257" t="inlineStr"/>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>2025-01-29 09:32:47</t>
+        </is>
+      </c>
+      <c r="B258" t="n">
+        <v>35054</v>
+      </c>
+      <c r="C258" t="n">
+        <v>0</v>
+      </c>
+      <c r="D258" t="n">
+        <v>0</v>
+      </c>
+      <c r="E258" t="n">
+        <v>0</v>
+      </c>
+      <c r="F258" t="n">
+        <v>4741</v>
+      </c>
+      <c r="G258" t="inlineStr"/>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>2025-01-29 15:15:52</t>
+        </is>
+      </c>
+      <c r="B259" t="n">
+        <v>38441</v>
+      </c>
+      <c r="C259" t="n">
+        <v>0</v>
+      </c>
+      <c r="D259" t="n">
+        <v>0</v>
+      </c>
+      <c r="E259" t="n">
+        <v>0</v>
+      </c>
+      <c r="F259" t="n">
+        <v>4946</v>
+      </c>
+      <c r="G259" t="inlineStr"/>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>2025-01-31 14:19:46</t>
+        </is>
+      </c>
+      <c r="B260" t="n">
+        <v>36066</v>
+      </c>
+      <c r="C260" t="n">
+        <v>0</v>
+      </c>
+      <c r="D260" t="n">
+        <v>0</v>
+      </c>
+      <c r="E260" t="n">
+        <v>0</v>
+      </c>
+      <c r="F260" t="n">
+        <v>5073</v>
+      </c>
+      <c r="G260" t="inlineStr"/>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>2025-01-31 18:30:54</t>
+        </is>
+      </c>
+      <c r="B261" t="n">
+        <v>36188</v>
+      </c>
+      <c r="C261" t="n">
+        <v>0</v>
+      </c>
+      <c r="D261" t="n">
+        <v>0</v>
+      </c>
+      <c r="E261" t="n">
+        <v>0</v>
+      </c>
+      <c r="F261" t="n">
+        <v>5060</v>
+      </c>
+      <c r="G261" t="inlineStr"/>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>2025-02-05 15:05:41</t>
+        </is>
+      </c>
+      <c r="B262" t="n">
+        <v>38127</v>
+      </c>
+      <c r="C262" t="n">
+        <v>0</v>
+      </c>
+      <c r="D262" t="n">
+        <v>0</v>
+      </c>
+      <c r="E262" t="n">
+        <v>0</v>
+      </c>
+      <c r="F262" t="n">
+        <v>5578</v>
+      </c>
+      <c r="G262" t="inlineStr"/>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>2025-02-12 09:01:26</t>
+        </is>
+      </c>
+      <c r="B263" t="n">
+        <v>115652</v>
+      </c>
+      <c r="C263" t="n">
+        <v>0</v>
+      </c>
+      <c r="D263" t="n">
+        <v>44</v>
+      </c>
+      <c r="E263" t="n">
+        <v>0</v>
+      </c>
+      <c r="F263" t="n">
+        <v>5827</v>
+      </c>
+      <c r="G263" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Samples showing intensity for the homologous series points
</commit_message>
<xml_diff>
--- a/LOC tracking outputs/code_metrics.xlsx
+++ b/LOC tracking outputs/code_metrics.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G263"/>
+  <dimension ref="A1:G272"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6539,6 +6539,213 @@
       </c>
       <c r="G263" t="inlineStr"/>
     </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>2025-01-27 21:06:55</t>
+        </is>
+      </c>
+      <c r="B264" t="n">
+        <v>18461</v>
+      </c>
+      <c r="C264" t="n">
+        <v>0</v>
+      </c>
+      <c r="D264" t="n">
+        <v>0</v>
+      </c>
+      <c r="E264" t="n">
+        <v>0</v>
+      </c>
+      <c r="F264" t="n">
+        <v>4264</v>
+      </c>
+      <c r="G264" t="inlineStr"/>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>2025-01-28 23:23:35</t>
+        </is>
+      </c>
+      <c r="B265" t="n">
+        <v>19566</v>
+      </c>
+      <c r="C265" t="n">
+        <v>0</v>
+      </c>
+      <c r="D265" t="n">
+        <v>0</v>
+      </c>
+      <c r="E265" t="n">
+        <v>0</v>
+      </c>
+      <c r="F265" t="n">
+        <v>4666</v>
+      </c>
+      <c r="G265" t="inlineStr"/>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>2025-02-03 20:54:27</t>
+        </is>
+      </c>
+      <c r="B266" t="n">
+        <v>37061</v>
+      </c>
+      <c r="C266" t="n">
+        <v>0</v>
+      </c>
+      <c r="D266" t="n">
+        <v>0</v>
+      </c>
+      <c r="E266" t="n">
+        <v>0</v>
+      </c>
+      <c r="F266" t="n">
+        <v>5358</v>
+      </c>
+      <c r="G266" t="inlineStr"/>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>2025-02-04 13:00:53</t>
+        </is>
+      </c>
+      <c r="B267" t="n">
+        <v>37389</v>
+      </c>
+      <c r="C267" t="n">
+        <v>0</v>
+      </c>
+      <c r="D267" t="n">
+        <v>0</v>
+      </c>
+      <c r="E267" t="n">
+        <v>0</v>
+      </c>
+      <c r="F267" t="n">
+        <v>5440</v>
+      </c>
+      <c r="G267" t="inlineStr"/>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>2025-02-05 21:11:20</t>
+        </is>
+      </c>
+      <c r="B268" t="n">
+        <v>38059</v>
+      </c>
+      <c r="C268" t="n">
+        <v>0</v>
+      </c>
+      <c r="D268" t="n">
+        <v>23</v>
+      </c>
+      <c r="E268" t="n">
+        <v>0</v>
+      </c>
+      <c r="F268" t="n">
+        <v>5581</v>
+      </c>
+      <c r="G268" t="inlineStr"/>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>2025-02-08 15:33:17</t>
+        </is>
+      </c>
+      <c r="B269" t="n">
+        <v>37696</v>
+      </c>
+      <c r="C269" t="n">
+        <v>0</v>
+      </c>
+      <c r="D269" t="n">
+        <v>44</v>
+      </c>
+      <c r="E269" t="n">
+        <v>0</v>
+      </c>
+      <c r="F269" t="n">
+        <v>5755</v>
+      </c>
+      <c r="G269" t="inlineStr"/>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>2025-02-11 14:27:34</t>
+        </is>
+      </c>
+      <c r="B270" t="n">
+        <v>115528</v>
+      </c>
+      <c r="C270" t="n">
+        <v>0</v>
+      </c>
+      <c r="D270" t="n">
+        <v>44</v>
+      </c>
+      <c r="E270" t="n">
+        <v>0</v>
+      </c>
+      <c r="F270" t="n">
+        <v>5839</v>
+      </c>
+      <c r="G270" t="inlineStr"/>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>2025-02-12 15:57:09</t>
+        </is>
+      </c>
+      <c r="B271" t="n">
+        <v>116424</v>
+      </c>
+      <c r="C271" t="n">
+        <v>0</v>
+      </c>
+      <c r="D271" t="n">
+        <v>44</v>
+      </c>
+      <c r="E271" t="n">
+        <v>0</v>
+      </c>
+      <c r="F271" t="n">
+        <v>6063</v>
+      </c>
+      <c r="G271" t="inlineStr"/>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>2025-02-13 14:21:15</t>
+        </is>
+      </c>
+      <c r="B272" t="n">
+        <v>117804</v>
+      </c>
+      <c r="C272" t="n">
+        <v>0</v>
+      </c>
+      <c r="D272" t="n">
+        <v>44</v>
+      </c>
+      <c r="E272" t="n">
+        <v>0</v>
+      </c>
+      <c r="F272" t="n">
+        <v>6159</v>
+      </c>
+      <c r="G272" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Showing the repeating unit - rt sfs being buggy
</commit_message>
<xml_diff>
--- a/LOC tracking outputs/code_metrics.xlsx
+++ b/LOC tracking outputs/code_metrics.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G272"/>
+  <dimension ref="A1:G282"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6746,6 +6746,236 @@
       </c>
       <c r="G272" t="inlineStr"/>
     </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>2025-01-27 21:06:55</t>
+        </is>
+      </c>
+      <c r="B273" t="n">
+        <v>18461</v>
+      </c>
+      <c r="C273" t="n">
+        <v>0</v>
+      </c>
+      <c r="D273" t="n">
+        <v>0</v>
+      </c>
+      <c r="E273" t="n">
+        <v>0</v>
+      </c>
+      <c r="F273" t="n">
+        <v>4264</v>
+      </c>
+      <c r="G273" t="inlineStr"/>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>2025-01-28 23:23:35</t>
+        </is>
+      </c>
+      <c r="B274" t="n">
+        <v>19566</v>
+      </c>
+      <c r="C274" t="n">
+        <v>0</v>
+      </c>
+      <c r="D274" t="n">
+        <v>0</v>
+      </c>
+      <c r="E274" t="n">
+        <v>0</v>
+      </c>
+      <c r="F274" t="n">
+        <v>4666</v>
+      </c>
+      <c r="G274" t="inlineStr"/>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>2025-02-03 20:54:27</t>
+        </is>
+      </c>
+      <c r="B275" t="n">
+        <v>37061</v>
+      </c>
+      <c r="C275" t="n">
+        <v>0</v>
+      </c>
+      <c r="D275" t="n">
+        <v>0</v>
+      </c>
+      <c r="E275" t="n">
+        <v>0</v>
+      </c>
+      <c r="F275" t="n">
+        <v>5358</v>
+      </c>
+      <c r="G275" t="inlineStr"/>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>2025-02-04 13:00:53</t>
+        </is>
+      </c>
+      <c r="B276" t="n">
+        <v>37389</v>
+      </c>
+      <c r="C276" t="n">
+        <v>0</v>
+      </c>
+      <c r="D276" t="n">
+        <v>0</v>
+      </c>
+      <c r="E276" t="n">
+        <v>0</v>
+      </c>
+      <c r="F276" t="n">
+        <v>5440</v>
+      </c>
+      <c r="G276" t="inlineStr"/>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>2025-02-05 21:11:20</t>
+        </is>
+      </c>
+      <c r="B277" t="n">
+        <v>38059</v>
+      </c>
+      <c r="C277" t="n">
+        <v>0</v>
+      </c>
+      <c r="D277" t="n">
+        <v>23</v>
+      </c>
+      <c r="E277" t="n">
+        <v>0</v>
+      </c>
+      <c r="F277" t="n">
+        <v>5581</v>
+      </c>
+      <c r="G277" t="inlineStr"/>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>2025-02-08 15:33:17</t>
+        </is>
+      </c>
+      <c r="B278" t="n">
+        <v>37696</v>
+      </c>
+      <c r="C278" t="n">
+        <v>0</v>
+      </c>
+      <c r="D278" t="n">
+        <v>44</v>
+      </c>
+      <c r="E278" t="n">
+        <v>0</v>
+      </c>
+      <c r="F278" t="n">
+        <v>5755</v>
+      </c>
+      <c r="G278" t="inlineStr"/>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>2025-02-11 14:27:34</t>
+        </is>
+      </c>
+      <c r="B279" t="n">
+        <v>115528</v>
+      </c>
+      <c r="C279" t="n">
+        <v>0</v>
+      </c>
+      <c r="D279" t="n">
+        <v>44</v>
+      </c>
+      <c r="E279" t="n">
+        <v>0</v>
+      </c>
+      <c r="F279" t="n">
+        <v>5839</v>
+      </c>
+      <c r="G279" t="inlineStr"/>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>2025-02-12 15:57:09</t>
+        </is>
+      </c>
+      <c r="B280" t="n">
+        <v>116424</v>
+      </c>
+      <c r="C280" t="n">
+        <v>0</v>
+      </c>
+      <c r="D280" t="n">
+        <v>44</v>
+      </c>
+      <c r="E280" t="n">
+        <v>0</v>
+      </c>
+      <c r="F280" t="n">
+        <v>6063</v>
+      </c>
+      <c r="G280" t="inlineStr"/>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>2025-02-13 14:21:15</t>
+        </is>
+      </c>
+      <c r="B281" t="n">
+        <v>117804</v>
+      </c>
+      <c r="C281" t="n">
+        <v>0</v>
+      </c>
+      <c r="D281" t="n">
+        <v>44</v>
+      </c>
+      <c r="E281" t="n">
+        <v>0</v>
+      </c>
+      <c r="F281" t="n">
+        <v>6159</v>
+      </c>
+      <c r="G281" t="inlineStr"/>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>2025-02-13 16:27:20</t>
+        </is>
+      </c>
+      <c r="B282" t="n">
+        <v>117699</v>
+      </c>
+      <c r="C282" t="n">
+        <v>0</v>
+      </c>
+      <c r="D282" t="n">
+        <v>61</v>
+      </c>
+      <c r="E282" t="n">
+        <v>0</v>
+      </c>
+      <c r="F282" t="n">
+        <v>6121</v>
+      </c>
+      <c r="G282" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Module import working on the library search module
</commit_message>
<xml_diff>
--- a/LOC tracking outputs/code_metrics.xlsx
+++ b/LOC tracking outputs/code_metrics.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G292"/>
+  <dimension ref="A1:G302"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7206,6 +7206,236 @@
       </c>
       <c r="G292" t="inlineStr"/>
     </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>2025-02-03 20:54:27</t>
+        </is>
+      </c>
+      <c r="B293" t="n">
+        <v>37061</v>
+      </c>
+      <c r="C293" t="n">
+        <v>0</v>
+      </c>
+      <c r="D293" t="n">
+        <v>0</v>
+      </c>
+      <c r="E293" t="n">
+        <v>0</v>
+      </c>
+      <c r="F293" t="n">
+        <v>5358</v>
+      </c>
+      <c r="G293" t="inlineStr"/>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>2025-02-04 13:00:53</t>
+        </is>
+      </c>
+      <c r="B294" t="n">
+        <v>37389</v>
+      </c>
+      <c r="C294" t="n">
+        <v>0</v>
+      </c>
+      <c r="D294" t="n">
+        <v>0</v>
+      </c>
+      <c r="E294" t="n">
+        <v>0</v>
+      </c>
+      <c r="F294" t="n">
+        <v>5440</v>
+      </c>
+      <c r="G294" t="inlineStr"/>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>2025-02-05 21:11:20</t>
+        </is>
+      </c>
+      <c r="B295" t="n">
+        <v>38059</v>
+      </c>
+      <c r="C295" t="n">
+        <v>0</v>
+      </c>
+      <c r="D295" t="n">
+        <v>23</v>
+      </c>
+      <c r="E295" t="n">
+        <v>0</v>
+      </c>
+      <c r="F295" t="n">
+        <v>5581</v>
+      </c>
+      <c r="G295" t="inlineStr"/>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>2025-02-08 15:33:17</t>
+        </is>
+      </c>
+      <c r="B296" t="n">
+        <v>37696</v>
+      </c>
+      <c r="C296" t="n">
+        <v>0</v>
+      </c>
+      <c r="D296" t="n">
+        <v>44</v>
+      </c>
+      <c r="E296" t="n">
+        <v>0</v>
+      </c>
+      <c r="F296" t="n">
+        <v>5755</v>
+      </c>
+      <c r="G296" t="inlineStr"/>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>2025-02-11 14:27:34</t>
+        </is>
+      </c>
+      <c r="B297" t="n">
+        <v>115528</v>
+      </c>
+      <c r="C297" t="n">
+        <v>0</v>
+      </c>
+      <c r="D297" t="n">
+        <v>44</v>
+      </c>
+      <c r="E297" t="n">
+        <v>0</v>
+      </c>
+      <c r="F297" t="n">
+        <v>5839</v>
+      </c>
+      <c r="G297" t="inlineStr"/>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>2025-02-12 15:57:09</t>
+        </is>
+      </c>
+      <c r="B298" t="n">
+        <v>116424</v>
+      </c>
+      <c r="C298" t="n">
+        <v>0</v>
+      </c>
+      <c r="D298" t="n">
+        <v>44</v>
+      </c>
+      <c r="E298" t="n">
+        <v>0</v>
+      </c>
+      <c r="F298" t="n">
+        <v>6063</v>
+      </c>
+      <c r="G298" t="inlineStr"/>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>2025-02-13 14:21:15</t>
+        </is>
+      </c>
+      <c r="B299" t="n">
+        <v>117804</v>
+      </c>
+      <c r="C299" t="n">
+        <v>0</v>
+      </c>
+      <c r="D299" t="n">
+        <v>44</v>
+      </c>
+      <c r="E299" t="n">
+        <v>0</v>
+      </c>
+      <c r="F299" t="n">
+        <v>6159</v>
+      </c>
+      <c r="G299" t="inlineStr"/>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>2025-02-13 16:27:20</t>
+        </is>
+      </c>
+      <c r="B300" t="n">
+        <v>117699</v>
+      </c>
+      <c r="C300" t="n">
+        <v>0</v>
+      </c>
+      <c r="D300" t="n">
+        <v>61</v>
+      </c>
+      <c r="E300" t="n">
+        <v>0</v>
+      </c>
+      <c r="F300" t="n">
+        <v>6121</v>
+      </c>
+      <c r="G300" t="inlineStr"/>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>2025-02-13 20:57:10</t>
+        </is>
+      </c>
+      <c r="B301" t="n">
+        <v>118337</v>
+      </c>
+      <c r="C301" t="n">
+        <v>0</v>
+      </c>
+      <c r="D301" t="n">
+        <v>61</v>
+      </c>
+      <c r="E301" t="n">
+        <v>0</v>
+      </c>
+      <c r="F301" t="n">
+        <v>6226</v>
+      </c>
+      <c r="G301" t="inlineStr"/>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>2025-02-14 15:55:05</t>
+        </is>
+      </c>
+      <c r="B302" t="n">
+        <v>117682</v>
+      </c>
+      <c r="C302" t="n">
+        <v>0</v>
+      </c>
+      <c r="D302" t="n">
+        <v>61</v>
+      </c>
+      <c r="E302" t="n">
+        <v>0</v>
+      </c>
+      <c r="F302" t="n">
+        <v>6095</v>
+      </c>
+      <c r="G302" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Legend showing clearly, but has an "all data" point
</commit_message>
<xml_diff>
--- a/LOC tracking outputs/code_metrics.xlsx
+++ b/LOC tracking outputs/code_metrics.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G302"/>
+  <dimension ref="A1:G312"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7436,6 +7436,236 @@
       </c>
       <c r="G302" t="inlineStr"/>
     </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>2025-02-05 21:11:20</t>
+        </is>
+      </c>
+      <c r="B303" t="n">
+        <v>38059</v>
+      </c>
+      <c r="C303" t="n">
+        <v>0</v>
+      </c>
+      <c r="D303" t="n">
+        <v>23</v>
+      </c>
+      <c r="E303" t="n">
+        <v>0</v>
+      </c>
+      <c r="F303" t="n">
+        <v>5581</v>
+      </c>
+      <c r="G303" t="inlineStr"/>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>2025-02-08 15:33:17</t>
+        </is>
+      </c>
+      <c r="B304" t="n">
+        <v>37696</v>
+      </c>
+      <c r="C304" t="n">
+        <v>0</v>
+      </c>
+      <c r="D304" t="n">
+        <v>44</v>
+      </c>
+      <c r="E304" t="n">
+        <v>0</v>
+      </c>
+      <c r="F304" t="n">
+        <v>5755</v>
+      </c>
+      <c r="G304" t="inlineStr"/>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>2025-02-11 14:27:34</t>
+        </is>
+      </c>
+      <c r="B305" t="n">
+        <v>115528</v>
+      </c>
+      <c r="C305" t="n">
+        <v>0</v>
+      </c>
+      <c r="D305" t="n">
+        <v>44</v>
+      </c>
+      <c r="E305" t="n">
+        <v>0</v>
+      </c>
+      <c r="F305" t="n">
+        <v>5839</v>
+      </c>
+      <c r="G305" t="inlineStr"/>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>2025-02-12 15:57:09</t>
+        </is>
+      </c>
+      <c r="B306" t="n">
+        <v>116424</v>
+      </c>
+      <c r="C306" t="n">
+        <v>0</v>
+      </c>
+      <c r="D306" t="n">
+        <v>44</v>
+      </c>
+      <c r="E306" t="n">
+        <v>0</v>
+      </c>
+      <c r="F306" t="n">
+        <v>6063</v>
+      </c>
+      <c r="G306" t="inlineStr"/>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>2025-02-13 14:21:15</t>
+        </is>
+      </c>
+      <c r="B307" t="n">
+        <v>117804</v>
+      </c>
+      <c r="C307" t="n">
+        <v>0</v>
+      </c>
+      <c r="D307" t="n">
+        <v>44</v>
+      </c>
+      <c r="E307" t="n">
+        <v>0</v>
+      </c>
+      <c r="F307" t="n">
+        <v>6159</v>
+      </c>
+      <c r="G307" t="inlineStr"/>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>2025-02-13 16:27:20</t>
+        </is>
+      </c>
+      <c r="B308" t="n">
+        <v>117699</v>
+      </c>
+      <c r="C308" t="n">
+        <v>0</v>
+      </c>
+      <c r="D308" t="n">
+        <v>61</v>
+      </c>
+      <c r="E308" t="n">
+        <v>0</v>
+      </c>
+      <c r="F308" t="n">
+        <v>6121</v>
+      </c>
+      <c r="G308" t="inlineStr"/>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>2025-02-13 20:57:10</t>
+        </is>
+      </c>
+      <c r="B309" t="n">
+        <v>118337</v>
+      </c>
+      <c r="C309" t="n">
+        <v>0</v>
+      </c>
+      <c r="D309" t="n">
+        <v>61</v>
+      </c>
+      <c r="E309" t="n">
+        <v>0</v>
+      </c>
+      <c r="F309" t="n">
+        <v>6226</v>
+      </c>
+      <c r="G309" t="inlineStr"/>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>2025-02-14 15:55:05</t>
+        </is>
+      </c>
+      <c r="B310" t="n">
+        <v>117682</v>
+      </c>
+      <c r="C310" t="n">
+        <v>0</v>
+      </c>
+      <c r="D310" t="n">
+        <v>61</v>
+      </c>
+      <c r="E310" t="n">
+        <v>0</v>
+      </c>
+      <c r="F310" t="n">
+        <v>6095</v>
+      </c>
+      <c r="G310" t="inlineStr"/>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>2025-02-14 17:28:03</t>
+        </is>
+      </c>
+      <c r="B311" t="n">
+        <v>118070</v>
+      </c>
+      <c r="C311" t="n">
+        <v>0</v>
+      </c>
+      <c r="D311" t="n">
+        <v>61</v>
+      </c>
+      <c r="E311" t="n">
+        <v>0</v>
+      </c>
+      <c r="F311" t="n">
+        <v>6171</v>
+      </c>
+      <c r="G311" t="inlineStr"/>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>2025-02-14 19:22:07</t>
+        </is>
+      </c>
+      <c r="B312" t="n">
+        <v>118610</v>
+      </c>
+      <c r="C312" t="n">
+        <v>0</v>
+      </c>
+      <c r="D312" t="n">
+        <v>61</v>
+      </c>
+      <c r="E312" t="n">
+        <v>0</v>
+      </c>
+      <c r="F312" t="n">
+        <v>6279</v>
+      </c>
+      <c r="G312" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Done for the week - still a lot to do with IMSpector gadget
</commit_message>
<xml_diff>
--- a/LOC tracking outputs/code_metrics.xlsx
+++ b/LOC tracking outputs/code_metrics.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G312"/>
+  <dimension ref="A1:G322"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7666,6 +7666,236 @@
       </c>
       <c r="G312" t="inlineStr"/>
     </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>2025-02-11 14:27:34</t>
+        </is>
+      </c>
+      <c r="B313" t="n">
+        <v>115528</v>
+      </c>
+      <c r="C313" t="n">
+        <v>0</v>
+      </c>
+      <c r="D313" t="n">
+        <v>44</v>
+      </c>
+      <c r="E313" t="n">
+        <v>0</v>
+      </c>
+      <c r="F313" t="n">
+        <v>5839</v>
+      </c>
+      <c r="G313" t="inlineStr"/>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>2025-02-12 15:57:09</t>
+        </is>
+      </c>
+      <c r="B314" t="n">
+        <v>116424</v>
+      </c>
+      <c r="C314" t="n">
+        <v>0</v>
+      </c>
+      <c r="D314" t="n">
+        <v>44</v>
+      </c>
+      <c r="E314" t="n">
+        <v>0</v>
+      </c>
+      <c r="F314" t="n">
+        <v>6063</v>
+      </c>
+      <c r="G314" t="inlineStr"/>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>2025-02-13 14:21:15</t>
+        </is>
+      </c>
+      <c r="B315" t="n">
+        <v>117804</v>
+      </c>
+      <c r="C315" t="n">
+        <v>0</v>
+      </c>
+      <c r="D315" t="n">
+        <v>44</v>
+      </c>
+      <c r="E315" t="n">
+        <v>0</v>
+      </c>
+      <c r="F315" t="n">
+        <v>6159</v>
+      </c>
+      <c r="G315" t="inlineStr"/>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>2025-02-13 16:27:20</t>
+        </is>
+      </c>
+      <c r="B316" t="n">
+        <v>117699</v>
+      </c>
+      <c r="C316" t="n">
+        <v>0</v>
+      </c>
+      <c r="D316" t="n">
+        <v>61</v>
+      </c>
+      <c r="E316" t="n">
+        <v>0</v>
+      </c>
+      <c r="F316" t="n">
+        <v>6121</v>
+      </c>
+      <c r="G316" t="inlineStr"/>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>2025-02-13 20:57:10</t>
+        </is>
+      </c>
+      <c r="B317" t="n">
+        <v>118337</v>
+      </c>
+      <c r="C317" t="n">
+        <v>0</v>
+      </c>
+      <c r="D317" t="n">
+        <v>61</v>
+      </c>
+      <c r="E317" t="n">
+        <v>0</v>
+      </c>
+      <c r="F317" t="n">
+        <v>6226</v>
+      </c>
+      <c r="G317" t="inlineStr"/>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>2025-02-14 15:55:05</t>
+        </is>
+      </c>
+      <c r="B318" t="n">
+        <v>117682</v>
+      </c>
+      <c r="C318" t="n">
+        <v>0</v>
+      </c>
+      <c r="D318" t="n">
+        <v>61</v>
+      </c>
+      <c r="E318" t="n">
+        <v>0</v>
+      </c>
+      <c r="F318" t="n">
+        <v>6095</v>
+      </c>
+      <c r="G318" t="inlineStr"/>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>2025-02-14 17:28:03</t>
+        </is>
+      </c>
+      <c r="B319" t="n">
+        <v>118070</v>
+      </c>
+      <c r="C319" t="n">
+        <v>0</v>
+      </c>
+      <c r="D319" t="n">
+        <v>61</v>
+      </c>
+      <c r="E319" t="n">
+        <v>0</v>
+      </c>
+      <c r="F319" t="n">
+        <v>6171</v>
+      </c>
+      <c r="G319" t="inlineStr"/>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>2025-02-14 19:22:07</t>
+        </is>
+      </c>
+      <c r="B320" t="n">
+        <v>118610</v>
+      </c>
+      <c r="C320" t="n">
+        <v>0</v>
+      </c>
+      <c r="D320" t="n">
+        <v>61</v>
+      </c>
+      <c r="E320" t="n">
+        <v>0</v>
+      </c>
+      <c r="F320" t="n">
+        <v>6279</v>
+      </c>
+      <c r="G320" t="inlineStr"/>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>2025-02-15 17:31:47</t>
+        </is>
+      </c>
+      <c r="B321" t="n">
+        <v>118755</v>
+      </c>
+      <c r="C321" t="n">
+        <v>0</v>
+      </c>
+      <c r="D321" t="n">
+        <v>61</v>
+      </c>
+      <c r="E321" t="n">
+        <v>0</v>
+      </c>
+      <c r="F321" t="n">
+        <v>6308</v>
+      </c>
+      <c r="G321" t="inlineStr"/>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>2025-02-15 22:17:41</t>
+        </is>
+      </c>
+      <c r="B322" t="n">
+        <v>118975</v>
+      </c>
+      <c r="C322" t="n">
+        <v>0</v>
+      </c>
+      <c r="D322" t="n">
+        <v>61</v>
+      </c>
+      <c r="E322" t="n">
+        <v>0</v>
+      </c>
+      <c r="F322" t="n">
+        <v>6350</v>
+      </c>
+      <c r="G322" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
library searching ready to get integrated into the main dash app
</commit_message>
<xml_diff>
--- a/LOC tracking outputs/code_metrics.xlsx
+++ b/LOC tracking outputs/code_metrics.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G322"/>
+  <dimension ref="A1:G332"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7896,6 +7896,236 @@
       </c>
       <c r="G322" t="inlineStr"/>
     </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>2025-02-12 15:57:09</t>
+        </is>
+      </c>
+      <c r="B323" t="n">
+        <v>116424</v>
+      </c>
+      <c r="C323" t="n">
+        <v>0</v>
+      </c>
+      <c r="D323" t="n">
+        <v>44</v>
+      </c>
+      <c r="E323" t="n">
+        <v>0</v>
+      </c>
+      <c r="F323" t="n">
+        <v>6063</v>
+      </c>
+      <c r="G323" t="inlineStr"/>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>2025-02-13 14:21:15</t>
+        </is>
+      </c>
+      <c r="B324" t="n">
+        <v>117804</v>
+      </c>
+      <c r="C324" t="n">
+        <v>0</v>
+      </c>
+      <c r="D324" t="n">
+        <v>44</v>
+      </c>
+      <c r="E324" t="n">
+        <v>0</v>
+      </c>
+      <c r="F324" t="n">
+        <v>6159</v>
+      </c>
+      <c r="G324" t="inlineStr"/>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>2025-02-13 16:27:20</t>
+        </is>
+      </c>
+      <c r="B325" t="n">
+        <v>117699</v>
+      </c>
+      <c r="C325" t="n">
+        <v>0</v>
+      </c>
+      <c r="D325" t="n">
+        <v>61</v>
+      </c>
+      <c r="E325" t="n">
+        <v>0</v>
+      </c>
+      <c r="F325" t="n">
+        <v>6121</v>
+      </c>
+      <c r="G325" t="inlineStr"/>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>2025-02-13 20:57:10</t>
+        </is>
+      </c>
+      <c r="B326" t="n">
+        <v>118337</v>
+      </c>
+      <c r="C326" t="n">
+        <v>0</v>
+      </c>
+      <c r="D326" t="n">
+        <v>61</v>
+      </c>
+      <c r="E326" t="n">
+        <v>0</v>
+      </c>
+      <c r="F326" t="n">
+        <v>6226</v>
+      </c>
+      <c r="G326" t="inlineStr"/>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>2025-02-14 15:55:05</t>
+        </is>
+      </c>
+      <c r="B327" t="n">
+        <v>117682</v>
+      </c>
+      <c r="C327" t="n">
+        <v>0</v>
+      </c>
+      <c r="D327" t="n">
+        <v>61</v>
+      </c>
+      <c r="E327" t="n">
+        <v>0</v>
+      </c>
+      <c r="F327" t="n">
+        <v>6095</v>
+      </c>
+      <c r="G327" t="inlineStr"/>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>2025-02-14 17:28:03</t>
+        </is>
+      </c>
+      <c r="B328" t="n">
+        <v>118070</v>
+      </c>
+      <c r="C328" t="n">
+        <v>0</v>
+      </c>
+      <c r="D328" t="n">
+        <v>61</v>
+      </c>
+      <c r="E328" t="n">
+        <v>0</v>
+      </c>
+      <c r="F328" t="n">
+        <v>6171</v>
+      </c>
+      <c r="G328" t="inlineStr"/>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>2025-02-14 19:22:07</t>
+        </is>
+      </c>
+      <c r="B329" t="n">
+        <v>118610</v>
+      </c>
+      <c r="C329" t="n">
+        <v>0</v>
+      </c>
+      <c r="D329" t="n">
+        <v>61</v>
+      </c>
+      <c r="E329" t="n">
+        <v>0</v>
+      </c>
+      <c r="F329" t="n">
+        <v>6279</v>
+      </c>
+      <c r="G329" t="inlineStr"/>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>2025-02-15 17:31:47</t>
+        </is>
+      </c>
+      <c r="B330" t="n">
+        <v>118755</v>
+      </c>
+      <c r="C330" t="n">
+        <v>0</v>
+      </c>
+      <c r="D330" t="n">
+        <v>61</v>
+      </c>
+      <c r="E330" t="n">
+        <v>0</v>
+      </c>
+      <c r="F330" t="n">
+        <v>6308</v>
+      </c>
+      <c r="G330" t="inlineStr"/>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>2025-02-15 22:17:41</t>
+        </is>
+      </c>
+      <c r="B331" t="n">
+        <v>118975</v>
+      </c>
+      <c r="C331" t="n">
+        <v>0</v>
+      </c>
+      <c r="D331" t="n">
+        <v>61</v>
+      </c>
+      <c r="E331" t="n">
+        <v>0</v>
+      </c>
+      <c r="F331" t="n">
+        <v>6350</v>
+      </c>
+      <c r="G331" t="inlineStr"/>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>2025-02-17 21:45:40</t>
+        </is>
+      </c>
+      <c r="B332" t="n">
+        <v>120210</v>
+      </c>
+      <c r="C332" t="n">
+        <v>0</v>
+      </c>
+      <c r="D332" t="n">
+        <v>61</v>
+      </c>
+      <c r="E332" t="n">
+        <v>0</v>
+      </c>
+      <c r="F332" t="n">
+        <v>6395</v>
+      </c>
+      <c r="G332" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Removed LOC tracking outputs from gitignore
</commit_message>
<xml_diff>
--- a/LOC tracking outputs/code_metrics.xlsx
+++ b/LOC tracking outputs/code_metrics.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G342"/>
+  <dimension ref="A1:G348"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8356,6 +8356,144 @@
       </c>
       <c r="G342" t="inlineStr"/>
     </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>2025-01-22 15:12:38</t>
+        </is>
+      </c>
+      <c r="B343" t="n">
+        <v>14445</v>
+      </c>
+      <c r="C343" t="n">
+        <v>0</v>
+      </c>
+      <c r="D343" t="n">
+        <v>0</v>
+      </c>
+      <c r="E343" t="n">
+        <v>0</v>
+      </c>
+      <c r="F343" t="n">
+        <v>3420</v>
+      </c>
+      <c r="G343" t="inlineStr"/>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>2025-01-22 15:13:06</t>
+        </is>
+      </c>
+      <c r="B344" t="n">
+        <v>14445</v>
+      </c>
+      <c r="C344" t="n">
+        <v>0</v>
+      </c>
+      <c r="D344" t="n">
+        <v>0</v>
+      </c>
+      <c r="E344" t="n">
+        <v>0</v>
+      </c>
+      <c r="F344" t="n">
+        <v>3420</v>
+      </c>
+      <c r="G344" t="inlineStr"/>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>2025-01-22 15:13:32</t>
+        </is>
+      </c>
+      <c r="B345" t="n">
+        <v>14445</v>
+      </c>
+      <c r="C345" t="n">
+        <v>0</v>
+      </c>
+      <c r="D345" t="n">
+        <v>0</v>
+      </c>
+      <c r="E345" t="n">
+        <v>0</v>
+      </c>
+      <c r="F345" t="n">
+        <v>3420</v>
+      </c>
+      <c r="G345" t="inlineStr"/>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>2025-01-25 08:17:46</t>
+        </is>
+      </c>
+      <c r="B346" t="n">
+        <v>16727</v>
+      </c>
+      <c r="C346" t="n">
+        <v>0</v>
+      </c>
+      <c r="D346" t="n">
+        <v>0</v>
+      </c>
+      <c r="E346" t="n">
+        <v>0</v>
+      </c>
+      <c r="F346" t="n">
+        <v>3853</v>
+      </c>
+      <c r="G346" t="inlineStr"/>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>2025-01-25 21:20:49</t>
+        </is>
+      </c>
+      <c r="B347" t="n">
+        <v>17381</v>
+      </c>
+      <c r="C347" t="n">
+        <v>0</v>
+      </c>
+      <c r="D347" t="n">
+        <v>0</v>
+      </c>
+      <c r="E347" t="n">
+        <v>0</v>
+      </c>
+      <c r="F347" t="n">
+        <v>4015</v>
+      </c>
+      <c r="G347" t="inlineStr"/>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>2025-02-19 08:54:02</t>
+        </is>
+      </c>
+      <c r="B348" t="n">
+        <v>123626</v>
+      </c>
+      <c r="C348" t="n">
+        <v>0</v>
+      </c>
+      <c r="D348" t="n">
+        <v>61</v>
+      </c>
+      <c r="E348" t="n">
+        <v>0</v>
+      </c>
+      <c r="F348" t="n">
+        <v>6921</v>
+      </c>
+      <c r="G348" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Library importing function working
</commit_message>
<xml_diff>
--- a/LOC tracking outputs/code_metrics.xlsx
+++ b/LOC tracking outputs/code_metrics.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G348"/>
+  <dimension ref="A1:G355"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8494,6 +8494,167 @@
       </c>
       <c r="G348" t="inlineStr"/>
     </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>2025-02-19 11:35:45</t>
+        </is>
+      </c>
+      <c r="B349" t="n">
+        <v>14445</v>
+      </c>
+      <c r="C349" t="n">
+        <v>0</v>
+      </c>
+      <c r="D349" t="n">
+        <v>0</v>
+      </c>
+      <c r="E349" t="n">
+        <v>0</v>
+      </c>
+      <c r="F349" t="n">
+        <v>3420</v>
+      </c>
+      <c r="G349" t="inlineStr"/>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>2025-02-19 11:35:45</t>
+        </is>
+      </c>
+      <c r="B350" t="n">
+        <v>14445</v>
+      </c>
+      <c r="C350" t="n">
+        <v>0</v>
+      </c>
+      <c r="D350" t="n">
+        <v>0</v>
+      </c>
+      <c r="E350" t="n">
+        <v>0</v>
+      </c>
+      <c r="F350" t="n">
+        <v>3420</v>
+      </c>
+      <c r="G350" t="inlineStr"/>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>2025-02-19 11:35:45</t>
+        </is>
+      </c>
+      <c r="B351" t="n">
+        <v>14445</v>
+      </c>
+      <c r="C351" t="n">
+        <v>0</v>
+      </c>
+      <c r="D351" t="n">
+        <v>0</v>
+      </c>
+      <c r="E351" t="n">
+        <v>0</v>
+      </c>
+      <c r="F351" t="n">
+        <v>3420</v>
+      </c>
+      <c r="G351" t="inlineStr"/>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>2025-02-19 11:35:45</t>
+        </is>
+      </c>
+      <c r="B352" t="n">
+        <v>16727</v>
+      </c>
+      <c r="C352" t="n">
+        <v>0</v>
+      </c>
+      <c r="D352" t="n">
+        <v>0</v>
+      </c>
+      <c r="E352" t="n">
+        <v>0</v>
+      </c>
+      <c r="F352" t="n">
+        <v>3853</v>
+      </c>
+      <c r="G352" t="inlineStr"/>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>2025-02-19 11:35:45</t>
+        </is>
+      </c>
+      <c r="B353" t="n">
+        <v>17381</v>
+      </c>
+      <c r="C353" t="n">
+        <v>0</v>
+      </c>
+      <c r="D353" t="n">
+        <v>0</v>
+      </c>
+      <c r="E353" t="n">
+        <v>0</v>
+      </c>
+      <c r="F353" t="n">
+        <v>4015</v>
+      </c>
+      <c r="G353" t="inlineStr"/>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>2025-02-19 11:35:45</t>
+        </is>
+      </c>
+      <c r="B354" t="n">
+        <v>123626</v>
+      </c>
+      <c r="C354" t="n">
+        <v>0</v>
+      </c>
+      <c r="D354" t="n">
+        <v>61</v>
+      </c>
+      <c r="E354" t="n">
+        <v>0</v>
+      </c>
+      <c r="F354" t="n">
+        <v>6921</v>
+      </c>
+      <c r="G354" t="inlineStr"/>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>2025-02-19 14:24:57</t>
+        </is>
+      </c>
+      <c r="B355" t="n">
+        <v>122974</v>
+      </c>
+      <c r="C355" t="n">
+        <v>0</v>
+      </c>
+      <c r="D355" t="n">
+        <v>123</v>
+      </c>
+      <c r="E355" t="n">
+        <v>0</v>
+      </c>
+      <c r="F355" t="n">
+        <v>6876</v>
+      </c>
+      <c r="G355" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
App layout updated with the rest of the graph still functioning
</commit_message>
<xml_diff>
--- a/LOC tracking outputs/code_metrics.xlsx
+++ b/LOC tracking outputs/code_metrics.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G364"/>
+  <dimension ref="A1:G375"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8501,42 +8501,42 @@
         </is>
       </c>
       <c r="B349" t="n">
-        <v>14445</v>
+        <v>123626</v>
       </c>
       <c r="C349" t="n">
         <v>0</v>
       </c>
       <c r="D349" t="n">
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="E349" t="n">
         <v>0</v>
       </c>
       <c r="F349" t="n">
-        <v>3420</v>
+        <v>6921</v>
       </c>
       <c r="G349" t="inlineStr"/>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>2025-02-19 11:35:45</t>
+          <t>2025-02-19 14:24:57</t>
         </is>
       </c>
       <c r="B350" t="n">
-        <v>14445</v>
+        <v>122974</v>
       </c>
       <c r="C350" t="n">
         <v>0</v>
       </c>
       <c r="D350" t="n">
-        <v>0</v>
+        <v>123</v>
       </c>
       <c r="E350" t="n">
         <v>0</v>
       </c>
       <c r="F350" t="n">
-        <v>3420</v>
+        <v>6876</v>
       </c>
       <c r="G350" t="inlineStr"/>
     </row>
@@ -8547,111 +8547,111 @@
         </is>
       </c>
       <c r="B351" t="n">
-        <v>14445</v>
+        <v>123626</v>
       </c>
       <c r="C351" t="n">
         <v>0</v>
       </c>
       <c r="D351" t="n">
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="E351" t="n">
         <v>0</v>
       </c>
       <c r="F351" t="n">
-        <v>3420</v>
+        <v>6921</v>
       </c>
       <c r="G351" t="inlineStr"/>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>2025-02-19 11:35:45</t>
+          <t>2025-02-19 14:24:57</t>
         </is>
       </c>
       <c r="B352" t="n">
-        <v>16727</v>
+        <v>122974</v>
       </c>
       <c r="C352" t="n">
         <v>0</v>
       </c>
       <c r="D352" t="n">
-        <v>0</v>
+        <v>123</v>
       </c>
       <c r="E352" t="n">
         <v>0</v>
       </c>
       <c r="F352" t="n">
-        <v>3853</v>
+        <v>6876</v>
       </c>
       <c r="G352" t="inlineStr"/>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>2025-02-19 11:35:45</t>
+          <t>2025-02-19 16:25:13</t>
         </is>
       </c>
       <c r="B353" t="n">
-        <v>17381</v>
+        <v>123576</v>
       </c>
       <c r="C353" t="n">
         <v>0</v>
       </c>
       <c r="D353" t="n">
-        <v>0</v>
+        <v>123</v>
       </c>
       <c r="E353" t="n">
         <v>0</v>
       </c>
       <c r="F353" t="n">
-        <v>4015</v>
+        <v>6887</v>
       </c>
       <c r="G353" t="inlineStr"/>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>2025-02-19 11:35:45</t>
+          <t>2025-02-20 13:33:30</t>
         </is>
       </c>
       <c r="B354" t="n">
-        <v>123626</v>
+        <v>124032</v>
       </c>
       <c r="C354" t="n">
         <v>0</v>
       </c>
       <c r="D354" t="n">
-        <v>61</v>
+        <v>123</v>
       </c>
       <c r="E354" t="n">
         <v>0</v>
       </c>
       <c r="F354" t="n">
-        <v>6921</v>
+        <v>6932</v>
       </c>
       <c r="G354" t="inlineStr"/>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>2025-02-19 14:24:57</t>
+          <t>2025-02-19 11:35:45</t>
         </is>
       </c>
       <c r="B355" t="n">
-        <v>122974</v>
+        <v>17381</v>
       </c>
       <c r="C355" t="n">
         <v>0</v>
       </c>
       <c r="D355" t="n">
-        <v>123</v>
+        <v>0</v>
       </c>
       <c r="E355" t="n">
         <v>0</v>
       </c>
       <c r="F355" t="n">
-        <v>6876</v>
+        <v>4015</v>
       </c>
       <c r="G355" t="inlineStr"/>
     </row>
@@ -8662,111 +8662,111 @@
         </is>
       </c>
       <c r="B356" t="n">
-        <v>14445</v>
+        <v>123626</v>
       </c>
       <c r="C356" t="n">
         <v>0</v>
       </c>
       <c r="D356" t="n">
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="E356" t="n">
         <v>0</v>
       </c>
       <c r="F356" t="n">
-        <v>3420</v>
+        <v>6921</v>
       </c>
       <c r="G356" t="inlineStr"/>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t>2025-02-19 11:35:45</t>
+          <t>2025-02-19 14:24:57</t>
         </is>
       </c>
       <c r="B357" t="n">
-        <v>14445</v>
+        <v>122974</v>
       </c>
       <c r="C357" t="n">
         <v>0</v>
       </c>
       <c r="D357" t="n">
-        <v>0</v>
+        <v>123</v>
       </c>
       <c r="E357" t="n">
         <v>0</v>
       </c>
       <c r="F357" t="n">
-        <v>3420</v>
+        <v>6876</v>
       </c>
       <c r="G357" t="inlineStr"/>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
         <is>
-          <t>2025-02-19 11:35:45</t>
+          <t>2025-02-19 16:25:13</t>
         </is>
       </c>
       <c r="B358" t="n">
-        <v>14445</v>
+        <v>123576</v>
       </c>
       <c r="C358" t="n">
         <v>0</v>
       </c>
       <c r="D358" t="n">
-        <v>0</v>
+        <v>123</v>
       </c>
       <c r="E358" t="n">
         <v>0</v>
       </c>
       <c r="F358" t="n">
-        <v>3420</v>
+        <v>6887</v>
       </c>
       <c r="G358" t="inlineStr"/>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
-          <t>2025-02-19 11:35:45</t>
+          <t>2025-02-20 13:33:30</t>
         </is>
       </c>
       <c r="B359" t="n">
-        <v>16727</v>
+        <v>124032</v>
       </c>
       <c r="C359" t="n">
         <v>0</v>
       </c>
       <c r="D359" t="n">
-        <v>0</v>
+        <v>123</v>
       </c>
       <c r="E359" t="n">
         <v>0</v>
       </c>
       <c r="F359" t="n">
-        <v>3853</v>
+        <v>6932</v>
       </c>
       <c r="G359" t="inlineStr"/>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>2025-02-19 11:35:45</t>
+          <t>2025-02-20 14:44:09</t>
         </is>
       </c>
       <c r="B360" t="n">
-        <v>17381</v>
+        <v>124902</v>
       </c>
       <c r="C360" t="n">
         <v>0</v>
       </c>
       <c r="D360" t="n">
-        <v>0</v>
+        <v>123</v>
       </c>
       <c r="E360" t="n">
         <v>0</v>
       </c>
       <c r="F360" t="n">
-        <v>4015</v>
+        <v>6988</v>
       </c>
       <c r="G360" t="inlineStr"/>
     </row>
@@ -8861,6 +8861,259 @@
         <v>6932</v>
       </c>
       <c r="G364" t="inlineStr"/>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>2025-02-20 14:44:09</t>
+        </is>
+      </c>
+      <c r="B365" t="n">
+        <v>124902</v>
+      </c>
+      <c r="C365" t="n">
+        <v>0</v>
+      </c>
+      <c r="D365" t="n">
+        <v>123</v>
+      </c>
+      <c r="E365" t="n">
+        <v>0</v>
+      </c>
+      <c r="F365" t="n">
+        <v>6988</v>
+      </c>
+      <c r="G365" t="inlineStr"/>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>2025-02-19 11:35:45</t>
+        </is>
+      </c>
+      <c r="B366" t="n">
+        <v>14445</v>
+      </c>
+      <c r="C366" t="n">
+        <v>0</v>
+      </c>
+      <c r="D366" t="n">
+        <v>0</v>
+      </c>
+      <c r="E366" t="n">
+        <v>0</v>
+      </c>
+      <c r="F366" t="n">
+        <v>3420</v>
+      </c>
+      <c r="G366" t="inlineStr"/>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>2025-02-19 11:35:45</t>
+        </is>
+      </c>
+      <c r="B367" t="n">
+        <v>14445</v>
+      </c>
+      <c r="C367" t="n">
+        <v>0</v>
+      </c>
+      <c r="D367" t="n">
+        <v>0</v>
+      </c>
+      <c r="E367" t="n">
+        <v>0</v>
+      </c>
+      <c r="F367" t="n">
+        <v>3420</v>
+      </c>
+      <c r="G367" t="inlineStr"/>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>2025-02-19 11:35:45</t>
+        </is>
+      </c>
+      <c r="B368" t="n">
+        <v>14445</v>
+      </c>
+      <c r="C368" t="n">
+        <v>0</v>
+      </c>
+      <c r="D368" t="n">
+        <v>0</v>
+      </c>
+      <c r="E368" t="n">
+        <v>0</v>
+      </c>
+      <c r="F368" t="n">
+        <v>3420</v>
+      </c>
+      <c r="G368" t="inlineStr"/>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>2025-02-19 11:35:45</t>
+        </is>
+      </c>
+      <c r="B369" t="n">
+        <v>16727</v>
+      </c>
+      <c r="C369" t="n">
+        <v>0</v>
+      </c>
+      <c r="D369" t="n">
+        <v>0</v>
+      </c>
+      <c r="E369" t="n">
+        <v>0</v>
+      </c>
+      <c r="F369" t="n">
+        <v>3853</v>
+      </c>
+      <c r="G369" t="inlineStr"/>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>2025-02-19 11:35:45</t>
+        </is>
+      </c>
+      <c r="B370" t="n">
+        <v>17381</v>
+      </c>
+      <c r="C370" t="n">
+        <v>0</v>
+      </c>
+      <c r="D370" t="n">
+        <v>0</v>
+      </c>
+      <c r="E370" t="n">
+        <v>0</v>
+      </c>
+      <c r="F370" t="n">
+        <v>4015</v>
+      </c>
+      <c r="G370" t="inlineStr"/>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>2025-02-19 11:35:45</t>
+        </is>
+      </c>
+      <c r="B371" t="n">
+        <v>123626</v>
+      </c>
+      <c r="C371" t="n">
+        <v>0</v>
+      </c>
+      <c r="D371" t="n">
+        <v>61</v>
+      </c>
+      <c r="E371" t="n">
+        <v>0</v>
+      </c>
+      <c r="F371" t="n">
+        <v>6921</v>
+      </c>
+      <c r="G371" t="inlineStr"/>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>2025-02-19 14:24:57</t>
+        </is>
+      </c>
+      <c r="B372" t="n">
+        <v>122974</v>
+      </c>
+      <c r="C372" t="n">
+        <v>0</v>
+      </c>
+      <c r="D372" t="n">
+        <v>123</v>
+      </c>
+      <c r="E372" t="n">
+        <v>0</v>
+      </c>
+      <c r="F372" t="n">
+        <v>6876</v>
+      </c>
+      <c r="G372" t="inlineStr"/>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>2025-02-19 16:25:13</t>
+        </is>
+      </c>
+      <c r="B373" t="n">
+        <v>123576</v>
+      </c>
+      <c r="C373" t="n">
+        <v>0</v>
+      </c>
+      <c r="D373" t="n">
+        <v>123</v>
+      </c>
+      <c r="E373" t="n">
+        <v>0</v>
+      </c>
+      <c r="F373" t="n">
+        <v>6887</v>
+      </c>
+      <c r="G373" t="inlineStr"/>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>2025-02-20 13:33:30</t>
+        </is>
+      </c>
+      <c r="B374" t="n">
+        <v>124032</v>
+      </c>
+      <c r="C374" t="n">
+        <v>0</v>
+      </c>
+      <c r="D374" t="n">
+        <v>123</v>
+      </c>
+      <c r="E374" t="n">
+        <v>0</v>
+      </c>
+      <c r="F374" t="n">
+        <v>6932</v>
+      </c>
+      <c r="G374" t="inlineStr"/>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>2025-02-20 14:44:09</t>
+        </is>
+      </c>
+      <c r="B375" t="n">
+        <v>124902</v>
+      </c>
+      <c r="C375" t="n">
+        <v>0</v>
+      </c>
+      <c r="D375" t="n">
+        <v>123</v>
+      </c>
+      <c r="E375" t="n">
+        <v>0</v>
+      </c>
+      <c r="F375" t="n">
+        <v>6988</v>
+      </c>
+      <c r="G375" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Did a count and made a graph
</commit_message>
<xml_diff>
--- a/LOC tracking outputs/code_metrics.xlsx
+++ b/LOC tracking outputs/code_metrics.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G375"/>
+  <dimension ref="A1:G385"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9115,6 +9115,236 @@
       </c>
       <c r="G375" t="inlineStr"/>
     </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>2025-02-19 11:35:45</t>
+        </is>
+      </c>
+      <c r="B376" t="n">
+        <v>14445</v>
+      </c>
+      <c r="C376" t="n">
+        <v>0</v>
+      </c>
+      <c r="D376" t="n">
+        <v>0</v>
+      </c>
+      <c r="E376" t="n">
+        <v>0</v>
+      </c>
+      <c r="F376" t="n">
+        <v>3420</v>
+      </c>
+      <c r="G376" t="inlineStr"/>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>2025-02-19 11:35:45</t>
+        </is>
+      </c>
+      <c r="B377" t="n">
+        <v>16727</v>
+      </c>
+      <c r="C377" t="n">
+        <v>0</v>
+      </c>
+      <c r="D377" t="n">
+        <v>0</v>
+      </c>
+      <c r="E377" t="n">
+        <v>0</v>
+      </c>
+      <c r="F377" t="n">
+        <v>3853</v>
+      </c>
+      <c r="G377" t="inlineStr"/>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>2025-02-19 11:35:45</t>
+        </is>
+      </c>
+      <c r="B378" t="n">
+        <v>17381</v>
+      </c>
+      <c r="C378" t="n">
+        <v>0</v>
+      </c>
+      <c r="D378" t="n">
+        <v>0</v>
+      </c>
+      <c r="E378" t="n">
+        <v>0</v>
+      </c>
+      <c r="F378" t="n">
+        <v>4015</v>
+      </c>
+      <c r="G378" t="inlineStr"/>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>2025-02-19 11:35:45</t>
+        </is>
+      </c>
+      <c r="B379" t="n">
+        <v>123626</v>
+      </c>
+      <c r="C379" t="n">
+        <v>0</v>
+      </c>
+      <c r="D379" t="n">
+        <v>61</v>
+      </c>
+      <c r="E379" t="n">
+        <v>0</v>
+      </c>
+      <c r="F379" t="n">
+        <v>6921</v>
+      </c>
+      <c r="G379" t="inlineStr"/>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>2025-02-19 14:24:57</t>
+        </is>
+      </c>
+      <c r="B380" t="n">
+        <v>122974</v>
+      </c>
+      <c r="C380" t="n">
+        <v>0</v>
+      </c>
+      <c r="D380" t="n">
+        <v>123</v>
+      </c>
+      <c r="E380" t="n">
+        <v>0</v>
+      </c>
+      <c r="F380" t="n">
+        <v>6876</v>
+      </c>
+      <c r="G380" t="inlineStr"/>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>2025-02-19 16:25:13</t>
+        </is>
+      </c>
+      <c r="B381" t="n">
+        <v>123576</v>
+      </c>
+      <c r="C381" t="n">
+        <v>0</v>
+      </c>
+      <c r="D381" t="n">
+        <v>123</v>
+      </c>
+      <c r="E381" t="n">
+        <v>0</v>
+      </c>
+      <c r="F381" t="n">
+        <v>6887</v>
+      </c>
+      <c r="G381" t="inlineStr"/>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>2025-02-20 13:33:30</t>
+        </is>
+      </c>
+      <c r="B382" t="n">
+        <v>124032</v>
+      </c>
+      <c r="C382" t="n">
+        <v>0</v>
+      </c>
+      <c r="D382" t="n">
+        <v>123</v>
+      </c>
+      <c r="E382" t="n">
+        <v>0</v>
+      </c>
+      <c r="F382" t="n">
+        <v>6932</v>
+      </c>
+      <c r="G382" t="inlineStr"/>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>2025-02-20 14:44:09</t>
+        </is>
+      </c>
+      <c r="B383" t="n">
+        <v>124902</v>
+      </c>
+      <c r="C383" t="n">
+        <v>0</v>
+      </c>
+      <c r="D383" t="n">
+        <v>123</v>
+      </c>
+      <c r="E383" t="n">
+        <v>0</v>
+      </c>
+      <c r="F383" t="n">
+        <v>6988</v>
+      </c>
+      <c r="G383" t="inlineStr"/>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>2025-02-20 17:06:05</t>
+        </is>
+      </c>
+      <c r="B384" t="n">
+        <v>125077</v>
+      </c>
+      <c r="C384" t="n">
+        <v>0</v>
+      </c>
+      <c r="D384" t="n">
+        <v>123</v>
+      </c>
+      <c r="E384" t="n">
+        <v>0</v>
+      </c>
+      <c r="F384" t="n">
+        <v>7023</v>
+      </c>
+      <c r="G384" t="inlineStr"/>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>2025-02-20 18:46:45</t>
+        </is>
+      </c>
+      <c r="B385" t="n">
+        <v>125037</v>
+      </c>
+      <c r="C385" t="n">
+        <v>0</v>
+      </c>
+      <c r="D385" t="n">
+        <v>123</v>
+      </c>
+      <c r="E385" t="n">
+        <v>0</v>
+      </c>
+      <c r="F385" t="n">
+        <v>7015</v>
+      </c>
+      <c r="G385" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Legend contains the correct format, needs to be reorganized
</commit_message>
<xml_diff>
--- a/LOC tracking outputs/code_metrics.xlsx
+++ b/LOC tracking outputs/code_metrics.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G385"/>
+  <dimension ref="A1:G395"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9345,6 +9345,236 @@
       </c>
       <c r="G385" t="inlineStr"/>
     </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>2025-02-21 08:38:30</t>
+        </is>
+      </c>
+      <c r="B386" t="n">
+        <v>16727</v>
+      </c>
+      <c r="C386" t="n">
+        <v>0</v>
+      </c>
+      <c r="D386" t="n">
+        <v>0</v>
+      </c>
+      <c r="E386" t="n">
+        <v>0</v>
+      </c>
+      <c r="F386" t="n">
+        <v>3853</v>
+      </c>
+      <c r="G386" t="inlineStr"/>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>2025-02-21 08:38:30</t>
+        </is>
+      </c>
+      <c r="B387" t="n">
+        <v>17381</v>
+      </c>
+      <c r="C387" t="n">
+        <v>0</v>
+      </c>
+      <c r="D387" t="n">
+        <v>0</v>
+      </c>
+      <c r="E387" t="n">
+        <v>0</v>
+      </c>
+      <c r="F387" t="n">
+        <v>4015</v>
+      </c>
+      <c r="G387" t="inlineStr"/>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>2025-02-21 08:38:30</t>
+        </is>
+      </c>
+      <c r="B388" t="n">
+        <v>123626</v>
+      </c>
+      <c r="C388" t="n">
+        <v>0</v>
+      </c>
+      <c r="D388" t="n">
+        <v>61</v>
+      </c>
+      <c r="E388" t="n">
+        <v>0</v>
+      </c>
+      <c r="F388" t="n">
+        <v>6921</v>
+      </c>
+      <c r="G388" t="inlineStr"/>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>2025-02-21 08:38:45</t>
+        </is>
+      </c>
+      <c r="B389" t="n">
+        <v>122974</v>
+      </c>
+      <c r="C389" t="n">
+        <v>0</v>
+      </c>
+      <c r="D389" t="n">
+        <v>123</v>
+      </c>
+      <c r="E389" t="n">
+        <v>0</v>
+      </c>
+      <c r="F389" t="n">
+        <v>6876</v>
+      </c>
+      <c r="G389" t="inlineStr"/>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>2025-02-21 08:38:45</t>
+        </is>
+      </c>
+      <c r="B390" t="n">
+        <v>123576</v>
+      </c>
+      <c r="C390" t="n">
+        <v>0</v>
+      </c>
+      <c r="D390" t="n">
+        <v>123</v>
+      </c>
+      <c r="E390" t="n">
+        <v>0</v>
+      </c>
+      <c r="F390" t="n">
+        <v>6887</v>
+      </c>
+      <c r="G390" t="inlineStr"/>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>2025-02-21 08:38:45</t>
+        </is>
+      </c>
+      <c r="B391" t="n">
+        <v>124032</v>
+      </c>
+      <c r="C391" t="n">
+        <v>0</v>
+      </c>
+      <c r="D391" t="n">
+        <v>123</v>
+      </c>
+      <c r="E391" t="n">
+        <v>0</v>
+      </c>
+      <c r="F391" t="n">
+        <v>6932</v>
+      </c>
+      <c r="G391" t="inlineStr"/>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>2025-02-21 08:38:45</t>
+        </is>
+      </c>
+      <c r="B392" t="n">
+        <v>124902</v>
+      </c>
+      <c r="C392" t="n">
+        <v>0</v>
+      </c>
+      <c r="D392" t="n">
+        <v>123</v>
+      </c>
+      <c r="E392" t="n">
+        <v>0</v>
+      </c>
+      <c r="F392" t="n">
+        <v>6988</v>
+      </c>
+      <c r="G392" t="inlineStr"/>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>2025-02-21 08:38:45</t>
+        </is>
+      </c>
+      <c r="B393" t="n">
+        <v>125077</v>
+      </c>
+      <c r="C393" t="n">
+        <v>0</v>
+      </c>
+      <c r="D393" t="n">
+        <v>123</v>
+      </c>
+      <c r="E393" t="n">
+        <v>0</v>
+      </c>
+      <c r="F393" t="n">
+        <v>7023</v>
+      </c>
+      <c r="G393" t="inlineStr"/>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>2025-02-21 08:38:45</t>
+        </is>
+      </c>
+      <c r="B394" t="n">
+        <v>125037</v>
+      </c>
+      <c r="C394" t="n">
+        <v>0</v>
+      </c>
+      <c r="D394" t="n">
+        <v>123</v>
+      </c>
+      <c r="E394" t="n">
+        <v>0</v>
+      </c>
+      <c r="F394" t="n">
+        <v>7015</v>
+      </c>
+      <c r="G394" t="inlineStr"/>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>2025-02-24 11:11:02</t>
+        </is>
+      </c>
+      <c r="B395" t="n">
+        <v>126251</v>
+      </c>
+      <c r="C395" t="n">
+        <v>0</v>
+      </c>
+      <c r="D395" t="n">
+        <v>123</v>
+      </c>
+      <c r="E395" t="n">
+        <v>0</v>
+      </c>
+      <c r="F395" t="n">
+        <v>7264</v>
+      </c>
+      <c r="G395" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adding back in sample intensities
</commit_message>
<xml_diff>
--- a/LOC tracking outputs/code_metrics.xlsx
+++ b/LOC tracking outputs/code_metrics.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G395"/>
+  <dimension ref="A1:G405"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9575,6 +9575,236 @@
       </c>
       <c r="G395" t="inlineStr"/>
     </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>2025-02-21 12:46:05</t>
+        </is>
+      </c>
+      <c r="B396" t="n">
+        <v>123626</v>
+      </c>
+      <c r="C396" t="n">
+        <v>0</v>
+      </c>
+      <c r="D396" t="n">
+        <v>61</v>
+      </c>
+      <c r="E396" t="n">
+        <v>0</v>
+      </c>
+      <c r="F396" t="n">
+        <v>6921</v>
+      </c>
+      <c r="G396" t="inlineStr"/>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>2025-02-21 12:48:34</t>
+        </is>
+      </c>
+      <c r="B397" t="n">
+        <v>122974</v>
+      </c>
+      <c r="C397" t="n">
+        <v>0</v>
+      </c>
+      <c r="D397" t="n">
+        <v>123</v>
+      </c>
+      <c r="E397" t="n">
+        <v>0</v>
+      </c>
+      <c r="F397" t="n">
+        <v>6876</v>
+      </c>
+      <c r="G397" t="inlineStr"/>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>2025-02-21 12:48:34</t>
+        </is>
+      </c>
+      <c r="B398" t="n">
+        <v>123576</v>
+      </c>
+      <c r="C398" t="n">
+        <v>0</v>
+      </c>
+      <c r="D398" t="n">
+        <v>123</v>
+      </c>
+      <c r="E398" t="n">
+        <v>0</v>
+      </c>
+      <c r="F398" t="n">
+        <v>6887</v>
+      </c>
+      <c r="G398" t="inlineStr"/>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>2025-02-21 12:48:34</t>
+        </is>
+      </c>
+      <c r="B399" t="n">
+        <v>124032</v>
+      </c>
+      <c r="C399" t="n">
+        <v>0</v>
+      </c>
+      <c r="D399" t="n">
+        <v>123</v>
+      </c>
+      <c r="E399" t="n">
+        <v>0</v>
+      </c>
+      <c r="F399" t="n">
+        <v>6932</v>
+      </c>
+      <c r="G399" t="inlineStr"/>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>2025-02-21 12:48:34</t>
+        </is>
+      </c>
+      <c r="B400" t="n">
+        <v>124902</v>
+      </c>
+      <c r="C400" t="n">
+        <v>0</v>
+      </c>
+      <c r="D400" t="n">
+        <v>123</v>
+      </c>
+      <c r="E400" t="n">
+        <v>0</v>
+      </c>
+      <c r="F400" t="n">
+        <v>6988</v>
+      </c>
+      <c r="G400" t="inlineStr"/>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>2025-02-21 12:48:34</t>
+        </is>
+      </c>
+      <c r="B401" t="n">
+        <v>125077</v>
+      </c>
+      <c r="C401" t="n">
+        <v>0</v>
+      </c>
+      <c r="D401" t="n">
+        <v>123</v>
+      </c>
+      <c r="E401" t="n">
+        <v>0</v>
+      </c>
+      <c r="F401" t="n">
+        <v>7023</v>
+      </c>
+      <c r="G401" t="inlineStr"/>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>2025-02-21 12:48:34</t>
+        </is>
+      </c>
+      <c r="B402" t="n">
+        <v>125037</v>
+      </c>
+      <c r="C402" t="n">
+        <v>0</v>
+      </c>
+      <c r="D402" t="n">
+        <v>123</v>
+      </c>
+      <c r="E402" t="n">
+        <v>0</v>
+      </c>
+      <c r="F402" t="n">
+        <v>7015</v>
+      </c>
+      <c r="G402" t="inlineStr"/>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>2025-02-24 14:09:42</t>
+        </is>
+      </c>
+      <c r="B403" t="n">
+        <v>126251</v>
+      </c>
+      <c r="C403" t="n">
+        <v>0</v>
+      </c>
+      <c r="D403" t="n">
+        <v>123</v>
+      </c>
+      <c r="E403" t="n">
+        <v>0</v>
+      </c>
+      <c r="F403" t="n">
+        <v>7264</v>
+      </c>
+      <c r="G403" t="inlineStr"/>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>2025-02-24 14:09:42</t>
+        </is>
+      </c>
+      <c r="B404" t="n">
+        <v>126461</v>
+      </c>
+      <c r="C404" t="n">
+        <v>0</v>
+      </c>
+      <c r="D404" t="n">
+        <v>123</v>
+      </c>
+      <c r="E404" t="n">
+        <v>0</v>
+      </c>
+      <c r="F404" t="n">
+        <v>7306</v>
+      </c>
+      <c r="G404" t="inlineStr"/>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>2025-02-24 14:31:41</t>
+        </is>
+      </c>
+      <c r="B405" t="n">
+        <v>126473</v>
+      </c>
+      <c r="C405" t="n">
+        <v>0</v>
+      </c>
+      <c r="D405" t="n">
+        <v>123</v>
+      </c>
+      <c r="E405" t="n">
+        <v>0</v>
+      </c>
+      <c r="F405" t="n">
+        <v>7341</v>
+      </c>
+      <c r="G405" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Working limit on consecutive points in the CCS v m/z plot
</commit_message>
<xml_diff>
--- a/LOC tracking outputs/code_metrics.xlsx
+++ b/LOC tracking outputs/code_metrics.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G405"/>
+  <dimension ref="A1:G415"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9805,6 +9805,236 @@
       </c>
       <c r="G405" t="inlineStr"/>
     </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>2025-02-21 08:38:45</t>
+        </is>
+      </c>
+      <c r="B406" t="n">
+        <v>122974</v>
+      </c>
+      <c r="C406" t="n">
+        <v>0</v>
+      </c>
+      <c r="D406" t="n">
+        <v>123</v>
+      </c>
+      <c r="E406" t="n">
+        <v>0</v>
+      </c>
+      <c r="F406" t="n">
+        <v>6876</v>
+      </c>
+      <c r="G406" t="inlineStr"/>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>2025-02-21 08:38:45</t>
+        </is>
+      </c>
+      <c r="B407" t="n">
+        <v>123576</v>
+      </c>
+      <c r="C407" t="n">
+        <v>0</v>
+      </c>
+      <c r="D407" t="n">
+        <v>123</v>
+      </c>
+      <c r="E407" t="n">
+        <v>0</v>
+      </c>
+      <c r="F407" t="n">
+        <v>6887</v>
+      </c>
+      <c r="G407" t="inlineStr"/>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>2025-02-21 08:38:45</t>
+        </is>
+      </c>
+      <c r="B408" t="n">
+        <v>124032</v>
+      </c>
+      <c r="C408" t="n">
+        <v>0</v>
+      </c>
+      <c r="D408" t="n">
+        <v>123</v>
+      </c>
+      <c r="E408" t="n">
+        <v>0</v>
+      </c>
+      <c r="F408" t="n">
+        <v>6932</v>
+      </c>
+      <c r="G408" t="inlineStr"/>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>2025-02-21 08:38:45</t>
+        </is>
+      </c>
+      <c r="B409" t="n">
+        <v>124902</v>
+      </c>
+      <c r="C409" t="n">
+        <v>0</v>
+      </c>
+      <c r="D409" t="n">
+        <v>123</v>
+      </c>
+      <c r="E409" t="n">
+        <v>0</v>
+      </c>
+      <c r="F409" t="n">
+        <v>6988</v>
+      </c>
+      <c r="G409" t="inlineStr"/>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>2025-02-21 08:38:45</t>
+        </is>
+      </c>
+      <c r="B410" t="n">
+        <v>125077</v>
+      </c>
+      <c r="C410" t="n">
+        <v>0</v>
+      </c>
+      <c r="D410" t="n">
+        <v>123</v>
+      </c>
+      <c r="E410" t="n">
+        <v>0</v>
+      </c>
+      <c r="F410" t="n">
+        <v>7023</v>
+      </c>
+      <c r="G410" t="inlineStr"/>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>2025-02-21 08:38:45</t>
+        </is>
+      </c>
+      <c r="B411" t="n">
+        <v>125037</v>
+      </c>
+      <c r="C411" t="n">
+        <v>0</v>
+      </c>
+      <c r="D411" t="n">
+        <v>123</v>
+      </c>
+      <c r="E411" t="n">
+        <v>0</v>
+      </c>
+      <c r="F411" t="n">
+        <v>7015</v>
+      </c>
+      <c r="G411" t="inlineStr"/>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>2025-02-24 11:11:02</t>
+        </is>
+      </c>
+      <c r="B412" t="n">
+        <v>126251</v>
+      </c>
+      <c r="C412" t="n">
+        <v>0</v>
+      </c>
+      <c r="D412" t="n">
+        <v>123</v>
+      </c>
+      <c r="E412" t="n">
+        <v>0</v>
+      </c>
+      <c r="F412" t="n">
+        <v>7264</v>
+      </c>
+      <c r="G412" t="inlineStr"/>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>2025-02-24 11:47:48</t>
+        </is>
+      </c>
+      <c r="B413" t="n">
+        <v>126461</v>
+      </c>
+      <c r="C413" t="n">
+        <v>0</v>
+      </c>
+      <c r="D413" t="n">
+        <v>123</v>
+      </c>
+      <c r="E413" t="n">
+        <v>0</v>
+      </c>
+      <c r="F413" t="n">
+        <v>7306</v>
+      </c>
+      <c r="G413" t="inlineStr"/>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>2025-02-25 10:33:53</t>
+        </is>
+      </c>
+      <c r="B414" t="n">
+        <v>126473</v>
+      </c>
+      <c r="C414" t="n">
+        <v>0</v>
+      </c>
+      <c r="D414" t="n">
+        <v>123</v>
+      </c>
+      <c r="E414" t="n">
+        <v>0</v>
+      </c>
+      <c r="F414" t="n">
+        <v>7341</v>
+      </c>
+      <c r="G414" t="inlineStr"/>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>2025-02-26 10:47:27</t>
+        </is>
+      </c>
+      <c r="B415" t="n">
+        <v>124119</v>
+      </c>
+      <c r="C415" t="n">
+        <v>0</v>
+      </c>
+      <c r="D415" t="n">
+        <v>123</v>
+      </c>
+      <c r="E415" t="n">
+        <v>0</v>
+      </c>
+      <c r="F415" t="n">
+        <v>7335</v>
+      </c>
+      <c r="G415" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Did a count and corrected the code metrics
</commit_message>
<xml_diff>
--- a/LOC tracking outputs/code_metrics.xlsx
+++ b/LOC tracking outputs/code_metrics.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G385"/>
+  <dimension ref="A1:G397"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8359,218 +8359,218 @@
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>2025-01-22 15:12:38</t>
+          <t>2025-02-19 08:54:02</t>
         </is>
       </c>
       <c r="B343" t="n">
-        <v>14445</v>
+        <v>123626</v>
       </c>
       <c r="C343" t="n">
         <v>0</v>
       </c>
       <c r="D343" t="n">
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="E343" t="n">
         <v>0</v>
       </c>
       <c r="F343" t="n">
-        <v>3420</v>
+        <v>6921</v>
       </c>
       <c r="G343" t="inlineStr"/>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>2025-01-22 15:13:06</t>
+          <t>2025-02-19 11:35:45</t>
         </is>
       </c>
       <c r="B344" t="n">
-        <v>14445</v>
+        <v>123626</v>
       </c>
       <c r="C344" t="n">
         <v>0</v>
       </c>
       <c r="D344" t="n">
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="E344" t="n">
         <v>0</v>
       </c>
       <c r="F344" t="n">
-        <v>3420</v>
+        <v>6921</v>
       </c>
       <c r="G344" t="inlineStr"/>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>2025-01-22 15:13:32</t>
+          <t>2025-02-19 14:24:57</t>
         </is>
       </c>
       <c r="B345" t="n">
-        <v>14445</v>
+        <v>122974</v>
       </c>
       <c r="C345" t="n">
         <v>0</v>
       </c>
       <c r="D345" t="n">
-        <v>0</v>
+        <v>123</v>
       </c>
       <c r="E345" t="n">
         <v>0</v>
       </c>
       <c r="F345" t="n">
-        <v>3420</v>
+        <v>6876</v>
       </c>
       <c r="G345" t="inlineStr"/>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>2025-01-25 08:17:46</t>
+          <t>2025-02-19 11:35:45</t>
         </is>
       </c>
       <c r="B346" t="n">
-        <v>16727</v>
+        <v>123626</v>
       </c>
       <c r="C346" t="n">
         <v>0</v>
       </c>
       <c r="D346" t="n">
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="E346" t="n">
         <v>0</v>
       </c>
       <c r="F346" t="n">
-        <v>3853</v>
+        <v>6921</v>
       </c>
       <c r="G346" t="inlineStr"/>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>2025-01-25 21:20:49</t>
+          <t>2025-02-19 14:24:57</t>
         </is>
       </c>
       <c r="B347" t="n">
-        <v>17381</v>
+        <v>122974</v>
       </c>
       <c r="C347" t="n">
         <v>0</v>
       </c>
       <c r="D347" t="n">
-        <v>0</v>
+        <v>123</v>
       </c>
       <c r="E347" t="n">
         <v>0</v>
       </c>
       <c r="F347" t="n">
-        <v>4015</v>
+        <v>6876</v>
       </c>
       <c r="G347" t="inlineStr"/>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>2025-02-19 08:54:02</t>
+          <t>2025-02-19 16:25:13</t>
         </is>
       </c>
       <c r="B348" t="n">
-        <v>123626</v>
+        <v>123576</v>
       </c>
       <c r="C348" t="n">
         <v>0</v>
       </c>
       <c r="D348" t="n">
-        <v>61</v>
+        <v>123</v>
       </c>
       <c r="E348" t="n">
         <v>0</v>
       </c>
       <c r="F348" t="n">
-        <v>6921</v>
+        <v>6887</v>
       </c>
       <c r="G348" t="inlineStr"/>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>2025-02-19 11:35:45</t>
+          <t>2025-02-20 13:33:30</t>
         </is>
       </c>
       <c r="B349" t="n">
-        <v>123626</v>
+        <v>124032</v>
       </c>
       <c r="C349" t="n">
         <v>0</v>
       </c>
       <c r="D349" t="n">
-        <v>61</v>
+        <v>123</v>
       </c>
       <c r="E349" t="n">
         <v>0</v>
       </c>
       <c r="F349" t="n">
-        <v>6921</v>
+        <v>6932</v>
       </c>
       <c r="G349" t="inlineStr"/>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>2025-02-19 14:24:57</t>
+          <t>2025-02-19 11:35:45</t>
         </is>
       </c>
       <c r="B350" t="n">
-        <v>122974</v>
+        <v>123626</v>
       </c>
       <c r="C350" t="n">
         <v>0</v>
       </c>
       <c r="D350" t="n">
-        <v>123</v>
+        <v>61</v>
       </c>
       <c r="E350" t="n">
         <v>0</v>
       </c>
       <c r="F350" t="n">
-        <v>6876</v>
+        <v>6921</v>
       </c>
       <c r="G350" t="inlineStr"/>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>2025-02-19 11:35:45</t>
+          <t>2025-02-19 14:24:57</t>
         </is>
       </c>
       <c r="B351" t="n">
-        <v>123626</v>
+        <v>122974</v>
       </c>
       <c r="C351" t="n">
         <v>0</v>
       </c>
       <c r="D351" t="n">
-        <v>61</v>
+        <v>123</v>
       </c>
       <c r="E351" t="n">
         <v>0</v>
       </c>
       <c r="F351" t="n">
-        <v>6921</v>
+        <v>6876</v>
       </c>
       <c r="G351" t="inlineStr"/>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>2025-02-19 14:24:57</t>
+          <t>2025-02-19 16:25:13</t>
         </is>
       </c>
       <c r="B352" t="n">
-        <v>122974</v>
+        <v>123576</v>
       </c>
       <c r="C352" t="n">
         <v>0</v>
@@ -8582,18 +8582,18 @@
         <v>0</v>
       </c>
       <c r="F352" t="n">
-        <v>6876</v>
+        <v>6887</v>
       </c>
       <c r="G352" t="inlineStr"/>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>2025-02-19 16:25:13</t>
+          <t>2025-02-20 13:33:30</t>
         </is>
       </c>
       <c r="B353" t="n">
-        <v>123576</v>
+        <v>124032</v>
       </c>
       <c r="C353" t="n">
         <v>0</v>
@@ -8605,18 +8605,18 @@
         <v>0</v>
       </c>
       <c r="F353" t="n">
-        <v>6887</v>
+        <v>6932</v>
       </c>
       <c r="G353" t="inlineStr"/>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>2025-02-20 13:33:30</t>
+          <t>2025-02-20 14:44:09</t>
         </is>
       </c>
       <c r="B354" t="n">
-        <v>124032</v>
+        <v>124902</v>
       </c>
       <c r="C354" t="n">
         <v>0</v>
@@ -8628,7 +8628,7 @@
         <v>0</v>
       </c>
       <c r="F354" t="n">
-        <v>6932</v>
+        <v>6988</v>
       </c>
       <c r="G354" t="inlineStr"/>
     </row>
@@ -8639,53 +8639,53 @@
         </is>
       </c>
       <c r="B355" t="n">
-        <v>17381</v>
+        <v>123626</v>
       </c>
       <c r="C355" t="n">
         <v>0</v>
       </c>
       <c r="D355" t="n">
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="E355" t="n">
         <v>0</v>
       </c>
       <c r="F355" t="n">
-        <v>4015</v>
+        <v>6921</v>
       </c>
       <c r="G355" t="inlineStr"/>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
-          <t>2025-02-19 11:35:45</t>
+          <t>2025-02-19 14:24:57</t>
         </is>
       </c>
       <c r="B356" t="n">
-        <v>123626</v>
+        <v>122974</v>
       </c>
       <c r="C356" t="n">
         <v>0</v>
       </c>
       <c r="D356" t="n">
-        <v>61</v>
+        <v>123</v>
       </c>
       <c r="E356" t="n">
         <v>0</v>
       </c>
       <c r="F356" t="n">
-        <v>6921</v>
+        <v>6876</v>
       </c>
       <c r="G356" t="inlineStr"/>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t>2025-02-19 14:24:57</t>
+          <t>2025-02-19 16:25:13</t>
         </is>
       </c>
       <c r="B357" t="n">
-        <v>122974</v>
+        <v>123576</v>
       </c>
       <c r="C357" t="n">
         <v>0</v>
@@ -8697,18 +8697,18 @@
         <v>0</v>
       </c>
       <c r="F357" t="n">
-        <v>6876</v>
+        <v>6887</v>
       </c>
       <c r="G357" t="inlineStr"/>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
         <is>
-          <t>2025-02-19 16:25:13</t>
+          <t>2025-02-20 13:33:30</t>
         </is>
       </c>
       <c r="B358" t="n">
-        <v>123576</v>
+        <v>124032</v>
       </c>
       <c r="C358" t="n">
         <v>0</v>
@@ -8720,18 +8720,18 @@
         <v>0</v>
       </c>
       <c r="F358" t="n">
-        <v>6887</v>
+        <v>6932</v>
       </c>
       <c r="G358" t="inlineStr"/>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
-          <t>2025-02-20 13:33:30</t>
+          <t>2025-02-20 14:44:09</t>
         </is>
       </c>
       <c r="B359" t="n">
-        <v>124032</v>
+        <v>124902</v>
       </c>
       <c r="C359" t="n">
         <v>0</v>
@@ -8743,64 +8743,64 @@
         <v>0</v>
       </c>
       <c r="F359" t="n">
-        <v>6932</v>
+        <v>6988</v>
       </c>
       <c r="G359" t="inlineStr"/>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>2025-02-20 14:44:09</t>
+          <t>2025-02-19 11:35:45</t>
         </is>
       </c>
       <c r="B360" t="n">
-        <v>124902</v>
+        <v>123626</v>
       </c>
       <c r="C360" t="n">
         <v>0</v>
       </c>
       <c r="D360" t="n">
-        <v>123</v>
+        <v>61</v>
       </c>
       <c r="E360" t="n">
         <v>0</v>
       </c>
       <c r="F360" t="n">
-        <v>6988</v>
+        <v>6921</v>
       </c>
       <c r="G360" t="inlineStr"/>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t>2025-02-19 11:35:45</t>
+          <t>2025-02-19 14:24:57</t>
         </is>
       </c>
       <c r="B361" t="n">
-        <v>123626</v>
+        <v>122974</v>
       </c>
       <c r="C361" t="n">
         <v>0</v>
       </c>
       <c r="D361" t="n">
-        <v>61</v>
+        <v>123</v>
       </c>
       <c r="E361" t="n">
         <v>0</v>
       </c>
       <c r="F361" t="n">
-        <v>6921</v>
+        <v>6876</v>
       </c>
       <c r="G361" t="inlineStr"/>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>2025-02-19 14:24:57</t>
+          <t>2025-02-19 16:25:13</t>
         </is>
       </c>
       <c r="B362" t="n">
-        <v>122974</v>
+        <v>123576</v>
       </c>
       <c r="C362" t="n">
         <v>0</v>
@@ -8812,18 +8812,18 @@
         <v>0</v>
       </c>
       <c r="F362" t="n">
-        <v>6876</v>
+        <v>6887</v>
       </c>
       <c r="G362" t="inlineStr"/>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
         <is>
-          <t>2025-02-19 16:25:13</t>
+          <t>2025-02-20 13:33:30</t>
         </is>
       </c>
       <c r="B363" t="n">
-        <v>123576</v>
+        <v>124032</v>
       </c>
       <c r="C363" t="n">
         <v>0</v>
@@ -8835,18 +8835,18 @@
         <v>0</v>
       </c>
       <c r="F363" t="n">
-        <v>6887</v>
+        <v>6932</v>
       </c>
       <c r="G363" t="inlineStr"/>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>2025-02-20 13:33:30</t>
+          <t>2025-02-20 14:44:09</t>
         </is>
       </c>
       <c r="B364" t="n">
-        <v>124032</v>
+        <v>124902</v>
       </c>
       <c r="C364" t="n">
         <v>0</v>
@@ -8858,202 +8858,202 @@
         <v>0</v>
       </c>
       <c r="F364" t="n">
-        <v>6932</v>
+        <v>6988</v>
       </c>
       <c r="G364" t="inlineStr"/>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
         <is>
-          <t>2025-02-20 14:44:09</t>
+          <t>2025-02-19 11:35:45</t>
         </is>
       </c>
       <c r="B365" t="n">
-        <v>124902</v>
+        <v>123626</v>
       </c>
       <c r="C365" t="n">
         <v>0</v>
       </c>
       <c r="D365" t="n">
-        <v>123</v>
+        <v>61</v>
       </c>
       <c r="E365" t="n">
         <v>0</v>
       </c>
       <c r="F365" t="n">
-        <v>6988</v>
+        <v>6921</v>
       </c>
       <c r="G365" t="inlineStr"/>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>2025-02-19 11:35:45</t>
+          <t>2025-02-19 14:24:57</t>
         </is>
       </c>
       <c r="B366" t="n">
-        <v>14445</v>
+        <v>122974</v>
       </c>
       <c r="C366" t="n">
         <v>0</v>
       </c>
       <c r="D366" t="n">
-        <v>0</v>
+        <v>123</v>
       </c>
       <c r="E366" t="n">
         <v>0</v>
       </c>
       <c r="F366" t="n">
-        <v>3420</v>
+        <v>6876</v>
       </c>
       <c r="G366" t="inlineStr"/>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
-          <t>2025-02-19 11:35:45</t>
+          <t>2025-02-19 16:25:13</t>
         </is>
       </c>
       <c r="B367" t="n">
-        <v>14445</v>
+        <v>123576</v>
       </c>
       <c r="C367" t="n">
         <v>0</v>
       </c>
       <c r="D367" t="n">
-        <v>0</v>
+        <v>123</v>
       </c>
       <c r="E367" t="n">
         <v>0</v>
       </c>
       <c r="F367" t="n">
-        <v>3420</v>
+        <v>6887</v>
       </c>
       <c r="G367" t="inlineStr"/>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
         <is>
-          <t>2025-02-19 11:35:45</t>
+          <t>2025-02-20 13:33:30</t>
         </is>
       </c>
       <c r="B368" t="n">
-        <v>14445</v>
+        <v>124032</v>
       </c>
       <c r="C368" t="n">
         <v>0</v>
       </c>
       <c r="D368" t="n">
-        <v>0</v>
+        <v>123</v>
       </c>
       <c r="E368" t="n">
         <v>0</v>
       </c>
       <c r="F368" t="n">
-        <v>3420</v>
+        <v>6932</v>
       </c>
       <c r="G368" t="inlineStr"/>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
         <is>
-          <t>2025-02-19 11:35:45</t>
+          <t>2025-02-20 14:44:09</t>
         </is>
       </c>
       <c r="B369" t="n">
-        <v>16727</v>
+        <v>124902</v>
       </c>
       <c r="C369" t="n">
         <v>0</v>
       </c>
       <c r="D369" t="n">
-        <v>0</v>
+        <v>123</v>
       </c>
       <c r="E369" t="n">
         <v>0</v>
       </c>
       <c r="F369" t="n">
-        <v>3853</v>
+        <v>6988</v>
       </c>
       <c r="G369" t="inlineStr"/>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
         <is>
-          <t>2025-02-19 11:35:45</t>
+          <t>2025-02-20 17:06:05</t>
         </is>
       </c>
       <c r="B370" t="n">
-        <v>17381</v>
+        <v>125077</v>
       </c>
       <c r="C370" t="n">
         <v>0</v>
       </c>
       <c r="D370" t="n">
-        <v>0</v>
+        <v>123</v>
       </c>
       <c r="E370" t="n">
         <v>0</v>
       </c>
       <c r="F370" t="n">
-        <v>4015</v>
+        <v>7023</v>
       </c>
       <c r="G370" t="inlineStr"/>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
         <is>
-          <t>2025-02-19 11:35:45</t>
+          <t>2025-02-20 18:46:45</t>
         </is>
       </c>
       <c r="B371" t="n">
-        <v>123626</v>
+        <v>125037</v>
       </c>
       <c r="C371" t="n">
         <v>0</v>
       </c>
       <c r="D371" t="n">
-        <v>61</v>
+        <v>123</v>
       </c>
       <c r="E371" t="n">
         <v>0</v>
       </c>
       <c r="F371" t="n">
-        <v>6921</v>
+        <v>7015</v>
       </c>
       <c r="G371" t="inlineStr"/>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
         <is>
-          <t>2025-02-19 14:24:57</t>
+          <t>2025-02-28 12:32:07</t>
         </is>
       </c>
       <c r="B372" t="n">
-        <v>122974</v>
+        <v>123626</v>
       </c>
       <c r="C372" t="n">
         <v>0</v>
       </c>
       <c r="D372" t="n">
-        <v>123</v>
+        <v>61</v>
       </c>
       <c r="E372" t="n">
         <v>0</v>
       </c>
       <c r="F372" t="n">
-        <v>6876</v>
+        <v>6921</v>
       </c>
       <c r="G372" t="inlineStr"/>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
         <is>
-          <t>2025-02-19 16:25:13</t>
+          <t>2025-02-21 12:48:34</t>
         </is>
       </c>
       <c r="B373" t="n">
-        <v>123576</v>
+        <v>122974</v>
       </c>
       <c r="C373" t="n">
         <v>0</v>
@@ -9065,18 +9065,18 @@
         <v>0</v>
       </c>
       <c r="F373" t="n">
-        <v>6887</v>
+        <v>6876</v>
       </c>
       <c r="G373" t="inlineStr"/>
     </row>
     <row r="374">
       <c r="A374" t="inlineStr">
         <is>
-          <t>2025-02-20 13:33:30</t>
+          <t>2025-02-21 12:48:34</t>
         </is>
       </c>
       <c r="B374" t="n">
-        <v>124032</v>
+        <v>123576</v>
       </c>
       <c r="C374" t="n">
         <v>0</v>
@@ -9088,18 +9088,18 @@
         <v>0</v>
       </c>
       <c r="F374" t="n">
-        <v>6932</v>
+        <v>6887</v>
       </c>
       <c r="G374" t="inlineStr"/>
     </row>
     <row r="375">
       <c r="A375" t="inlineStr">
         <is>
-          <t>2025-02-20 14:44:09</t>
+          <t>2025-02-21 12:48:34</t>
         </is>
       </c>
       <c r="B375" t="n">
-        <v>124902</v>
+        <v>124032</v>
       </c>
       <c r="C375" t="n">
         <v>0</v>
@@ -9111,156 +9111,156 @@
         <v>0</v>
       </c>
       <c r="F375" t="n">
-        <v>6988</v>
+        <v>6932</v>
       </c>
       <c r="G375" t="inlineStr"/>
     </row>
     <row r="376">
       <c r="A376" t="inlineStr">
         <is>
-          <t>2025-02-19 11:35:45</t>
+          <t>2025-02-21 12:48:34</t>
         </is>
       </c>
       <c r="B376" t="n">
-        <v>14445</v>
+        <v>124902</v>
       </c>
       <c r="C376" t="n">
         <v>0</v>
       </c>
       <c r="D376" t="n">
-        <v>0</v>
+        <v>123</v>
       </c>
       <c r="E376" t="n">
         <v>0</v>
       </c>
       <c r="F376" t="n">
-        <v>3420</v>
+        <v>6988</v>
       </c>
       <c r="G376" t="inlineStr"/>
     </row>
     <row r="377">
       <c r="A377" t="inlineStr">
         <is>
-          <t>2025-02-19 11:35:45</t>
+          <t>2025-02-21 12:48:34</t>
         </is>
       </c>
       <c r="B377" t="n">
-        <v>16727</v>
+        <v>125077</v>
       </c>
       <c r="C377" t="n">
         <v>0</v>
       </c>
       <c r="D377" t="n">
-        <v>0</v>
+        <v>123</v>
       </c>
       <c r="E377" t="n">
         <v>0</v>
       </c>
       <c r="F377" t="n">
-        <v>3853</v>
+        <v>7023</v>
       </c>
       <c r="G377" t="inlineStr"/>
     </row>
     <row r="378">
       <c r="A378" t="inlineStr">
         <is>
-          <t>2025-02-19 11:35:45</t>
+          <t>2025-02-21 12:48:34</t>
         </is>
       </c>
       <c r="B378" t="n">
-        <v>17381</v>
+        <v>125037</v>
       </c>
       <c r="C378" t="n">
         <v>0</v>
       </c>
       <c r="D378" t="n">
-        <v>0</v>
+        <v>123</v>
       </c>
       <c r="E378" t="n">
         <v>0</v>
       </c>
       <c r="F378" t="n">
-        <v>4015</v>
+        <v>7015</v>
       </c>
       <c r="G378" t="inlineStr"/>
     </row>
     <row r="379">
       <c r="A379" t="inlineStr">
         <is>
-          <t>2025-02-19 11:35:45</t>
+          <t>2025-02-28 19:52:54</t>
         </is>
       </c>
       <c r="B379" t="n">
-        <v>123626</v>
+        <v>128311</v>
       </c>
       <c r="C379" t="n">
         <v>0</v>
       </c>
       <c r="D379" t="n">
-        <v>61</v>
+        <v>164</v>
       </c>
       <c r="E379" t="n">
         <v>0</v>
       </c>
       <c r="F379" t="n">
-        <v>6921</v>
+        <v>7667</v>
       </c>
       <c r="G379" t="inlineStr"/>
     </row>
     <row r="380">
       <c r="A380" t="inlineStr">
         <is>
-          <t>2025-02-19 14:24:57</t>
+          <t>2025-02-28 12:32:07</t>
         </is>
       </c>
       <c r="B380" t="n">
-        <v>122974</v>
+        <v>17381</v>
       </c>
       <c r="C380" t="n">
         <v>0</v>
       </c>
       <c r="D380" t="n">
-        <v>123</v>
+        <v>0</v>
       </c>
       <c r="E380" t="n">
         <v>0</v>
       </c>
       <c r="F380" t="n">
-        <v>6876</v>
+        <v>4015</v>
       </c>
       <c r="G380" t="inlineStr"/>
     </row>
     <row r="381">
       <c r="A381" t="inlineStr">
         <is>
-          <t>2025-02-19 16:25:13</t>
+          <t>2025-02-28 12:32:07</t>
         </is>
       </c>
       <c r="B381" t="n">
-        <v>123576</v>
+        <v>123626</v>
       </c>
       <c r="C381" t="n">
         <v>0</v>
       </c>
       <c r="D381" t="n">
-        <v>123</v>
+        <v>61</v>
       </c>
       <c r="E381" t="n">
         <v>0</v>
       </c>
       <c r="F381" t="n">
-        <v>6887</v>
+        <v>6921</v>
       </c>
       <c r="G381" t="inlineStr"/>
     </row>
     <row r="382">
       <c r="A382" t="inlineStr">
         <is>
-          <t>2025-02-20 13:33:30</t>
+          <t>2025-02-21 12:48:34</t>
         </is>
       </c>
       <c r="B382" t="n">
-        <v>124032</v>
+        <v>122974</v>
       </c>
       <c r="C382" t="n">
         <v>0</v>
@@ -9272,18 +9272,18 @@
         <v>0</v>
       </c>
       <c r="F382" t="n">
-        <v>6932</v>
+        <v>6876</v>
       </c>
       <c r="G382" t="inlineStr"/>
     </row>
     <row r="383">
       <c r="A383" t="inlineStr">
         <is>
-          <t>2025-02-20 14:44:09</t>
+          <t>2025-02-21 12:48:34</t>
         </is>
       </c>
       <c r="B383" t="n">
-        <v>124902</v>
+        <v>123576</v>
       </c>
       <c r="C383" t="n">
         <v>0</v>
@@ -9295,18 +9295,18 @@
         <v>0</v>
       </c>
       <c r="F383" t="n">
-        <v>6988</v>
+        <v>6887</v>
       </c>
       <c r="G383" t="inlineStr"/>
     </row>
     <row r="384">
       <c r="A384" t="inlineStr">
         <is>
-          <t>2025-02-20 17:06:05</t>
+          <t>2025-02-21 12:48:34</t>
         </is>
       </c>
       <c r="B384" t="n">
-        <v>125077</v>
+        <v>124032</v>
       </c>
       <c r="C384" t="n">
         <v>0</v>
@@ -9318,18 +9318,18 @@
         <v>0</v>
       </c>
       <c r="F384" t="n">
-        <v>7023</v>
+        <v>6932</v>
       </c>
       <c r="G384" t="inlineStr"/>
     </row>
     <row r="385">
       <c r="A385" t="inlineStr">
         <is>
-          <t>2025-02-20 18:46:45</t>
+          <t>2025-02-21 12:48:34</t>
         </is>
       </c>
       <c r="B385" t="n">
-        <v>125037</v>
+        <v>124902</v>
       </c>
       <c r="C385" t="n">
         <v>0</v>
@@ -9341,9 +9341,285 @@
         <v>0</v>
       </c>
       <c r="F385" t="n">
+        <v>6988</v>
+      </c>
+      <c r="G385" t="inlineStr"/>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>2025-02-21 12:48:34</t>
+        </is>
+      </c>
+      <c r="B386" t="n">
+        <v>125077</v>
+      </c>
+      <c r="C386" t="n">
+        <v>0</v>
+      </c>
+      <c r="D386" t="n">
+        <v>123</v>
+      </c>
+      <c r="E386" t="n">
+        <v>0</v>
+      </c>
+      <c r="F386" t="n">
+        <v>7023</v>
+      </c>
+      <c r="G386" t="inlineStr"/>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>2025-02-21 12:48:34</t>
+        </is>
+      </c>
+      <c r="B387" t="n">
+        <v>125037</v>
+      </c>
+      <c r="C387" t="n">
+        <v>0</v>
+      </c>
+      <c r="D387" t="n">
+        <v>123</v>
+      </c>
+      <c r="E387" t="n">
+        <v>0</v>
+      </c>
+      <c r="F387" t="n">
         <v>7015</v>
       </c>
-      <c r="G385" t="inlineStr"/>
+      <c r="G387" t="inlineStr"/>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>2025-02-28 19:52:54</t>
+        </is>
+      </c>
+      <c r="B388" t="n">
+        <v>128311</v>
+      </c>
+      <c r="C388" t="n">
+        <v>0</v>
+      </c>
+      <c r="D388" t="n">
+        <v>164</v>
+      </c>
+      <c r="E388" t="n">
+        <v>0</v>
+      </c>
+      <c r="F388" t="n">
+        <v>7667</v>
+      </c>
+      <c r="G388" t="inlineStr"/>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>2025-02-28 12:32:07</t>
+        </is>
+      </c>
+      <c r="B389" t="n">
+        <v>17381</v>
+      </c>
+      <c r="C389" t="n">
+        <v>0</v>
+      </c>
+      <c r="D389" t="n">
+        <v>0</v>
+      </c>
+      <c r="E389" t="n">
+        <v>0</v>
+      </c>
+      <c r="F389" t="n">
+        <v>4015</v>
+      </c>
+      <c r="G389" t="inlineStr"/>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>2025-02-28 12:32:07</t>
+        </is>
+      </c>
+      <c r="B390" t="n">
+        <v>123626</v>
+      </c>
+      <c r="C390" t="n">
+        <v>0</v>
+      </c>
+      <c r="D390" t="n">
+        <v>61</v>
+      </c>
+      <c r="E390" t="n">
+        <v>0</v>
+      </c>
+      <c r="F390" t="n">
+        <v>6921</v>
+      </c>
+      <c r="G390" t="inlineStr"/>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>2025-02-21 12:48:34</t>
+        </is>
+      </c>
+      <c r="B391" t="n">
+        <v>122974</v>
+      </c>
+      <c r="C391" t="n">
+        <v>0</v>
+      </c>
+      <c r="D391" t="n">
+        <v>123</v>
+      </c>
+      <c r="E391" t="n">
+        <v>0</v>
+      </c>
+      <c r="F391" t="n">
+        <v>6876</v>
+      </c>
+      <c r="G391" t="inlineStr"/>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>2025-02-21 12:48:34</t>
+        </is>
+      </c>
+      <c r="B392" t="n">
+        <v>123576</v>
+      </c>
+      <c r="C392" t="n">
+        <v>0</v>
+      </c>
+      <c r="D392" t="n">
+        <v>123</v>
+      </c>
+      <c r="E392" t="n">
+        <v>0</v>
+      </c>
+      <c r="F392" t="n">
+        <v>6887</v>
+      </c>
+      <c r="G392" t="inlineStr"/>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>2025-02-21 12:48:34</t>
+        </is>
+      </c>
+      <c r="B393" t="n">
+        <v>124032</v>
+      </c>
+      <c r="C393" t="n">
+        <v>0</v>
+      </c>
+      <c r="D393" t="n">
+        <v>123</v>
+      </c>
+      <c r="E393" t="n">
+        <v>0</v>
+      </c>
+      <c r="F393" t="n">
+        <v>6932</v>
+      </c>
+      <c r="G393" t="inlineStr"/>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>2025-02-21 12:48:34</t>
+        </is>
+      </c>
+      <c r="B394" t="n">
+        <v>124902</v>
+      </c>
+      <c r="C394" t="n">
+        <v>0</v>
+      </c>
+      <c r="D394" t="n">
+        <v>123</v>
+      </c>
+      <c r="E394" t="n">
+        <v>0</v>
+      </c>
+      <c r="F394" t="n">
+        <v>6988</v>
+      </c>
+      <c r="G394" t="inlineStr"/>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>2025-02-21 12:48:34</t>
+        </is>
+      </c>
+      <c r="B395" t="n">
+        <v>125077</v>
+      </c>
+      <c r="C395" t="n">
+        <v>0</v>
+      </c>
+      <c r="D395" t="n">
+        <v>123</v>
+      </c>
+      <c r="E395" t="n">
+        <v>0</v>
+      </c>
+      <c r="F395" t="n">
+        <v>7023</v>
+      </c>
+      <c r="G395" t="inlineStr"/>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>2025-02-21 12:48:34</t>
+        </is>
+      </c>
+      <c r="B396" t="n">
+        <v>125037</v>
+      </c>
+      <c r="C396" t="n">
+        <v>0</v>
+      </c>
+      <c r="D396" t="n">
+        <v>123</v>
+      </c>
+      <c r="E396" t="n">
+        <v>0</v>
+      </c>
+      <c r="F396" t="n">
+        <v>7015</v>
+      </c>
+      <c r="G396" t="inlineStr"/>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>2025-02-28 19:52:54</t>
+        </is>
+      </c>
+      <c r="B397" t="n">
+        <v>128311</v>
+      </c>
+      <c r="C397" t="n">
+        <v>0</v>
+      </c>
+      <c r="D397" t="n">
+        <v>164</v>
+      </c>
+      <c r="E397" t="n">
+        <v>0</v>
+      </c>
+      <c r="F397" t="n">
+        <v>7667</v>
+      </c>
+      <c r="G397" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
just need to rename adducts
</commit_message>
<xml_diff>
--- a/LOC tracking outputs/code_metrics.xlsx
+++ b/LOC tracking outputs/code_metrics.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G407"/>
+  <dimension ref="A1:G416"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9851,6 +9851,213 @@
       </c>
       <c r="G407" t="inlineStr"/>
     </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>2025-02-21 12:48:34</t>
+        </is>
+      </c>
+      <c r="B408" t="n">
+        <v>123576</v>
+      </c>
+      <c r="C408" t="n">
+        <v>0</v>
+      </c>
+      <c r="D408" t="n">
+        <v>123</v>
+      </c>
+      <c r="E408" t="n">
+        <v>0</v>
+      </c>
+      <c r="F408" t="n">
+        <v>6887</v>
+      </c>
+      <c r="G408" t="inlineStr"/>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>2025-02-21 12:48:34</t>
+        </is>
+      </c>
+      <c r="B409" t="n">
+        <v>124032</v>
+      </c>
+      <c r="C409" t="n">
+        <v>0</v>
+      </c>
+      <c r="D409" t="n">
+        <v>123</v>
+      </c>
+      <c r="E409" t="n">
+        <v>0</v>
+      </c>
+      <c r="F409" t="n">
+        <v>6932</v>
+      </c>
+      <c r="G409" t="inlineStr"/>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>2025-02-21 12:48:34</t>
+        </is>
+      </c>
+      <c r="B410" t="n">
+        <v>124902</v>
+      </c>
+      <c r="C410" t="n">
+        <v>0</v>
+      </c>
+      <c r="D410" t="n">
+        <v>123</v>
+      </c>
+      <c r="E410" t="n">
+        <v>0</v>
+      </c>
+      <c r="F410" t="n">
+        <v>6988</v>
+      </c>
+      <c r="G410" t="inlineStr"/>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>2025-02-21 12:48:34</t>
+        </is>
+      </c>
+      <c r="B411" t="n">
+        <v>125077</v>
+      </c>
+      <c r="C411" t="n">
+        <v>0</v>
+      </c>
+      <c r="D411" t="n">
+        <v>123</v>
+      </c>
+      <c r="E411" t="n">
+        <v>0</v>
+      </c>
+      <c r="F411" t="n">
+        <v>7023</v>
+      </c>
+      <c r="G411" t="inlineStr"/>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>2025-02-21 12:48:34</t>
+        </is>
+      </c>
+      <c r="B412" t="n">
+        <v>125037</v>
+      </c>
+      <c r="C412" t="n">
+        <v>0</v>
+      </c>
+      <c r="D412" t="n">
+        <v>123</v>
+      </c>
+      <c r="E412" t="n">
+        <v>0</v>
+      </c>
+      <c r="F412" t="n">
+        <v>7015</v>
+      </c>
+      <c r="G412" t="inlineStr"/>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>2025-02-28 19:52:54</t>
+        </is>
+      </c>
+      <c r="B413" t="n">
+        <v>128311</v>
+      </c>
+      <c r="C413" t="n">
+        <v>0</v>
+      </c>
+      <c r="D413" t="n">
+        <v>164</v>
+      </c>
+      <c r="E413" t="n">
+        <v>0</v>
+      </c>
+      <c r="F413" t="n">
+        <v>7667</v>
+      </c>
+      <c r="G413" t="inlineStr"/>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>2025-03-01 17:52:08</t>
+        </is>
+      </c>
+      <c r="B414" t="n">
+        <v>128327</v>
+      </c>
+      <c r="C414" t="n">
+        <v>0</v>
+      </c>
+      <c r="D414" t="n">
+        <v>164</v>
+      </c>
+      <c r="E414" t="n">
+        <v>0</v>
+      </c>
+      <c r="F414" t="n">
+        <v>7675</v>
+      </c>
+      <c r="G414" t="inlineStr"/>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>2025-03-04 12:57:49</t>
+        </is>
+      </c>
+      <c r="B415" t="n">
+        <v>131661</v>
+      </c>
+      <c r="C415" t="n">
+        <v>0</v>
+      </c>
+      <c r="D415" t="n">
+        <v>164</v>
+      </c>
+      <c r="E415" t="n">
+        <v>0</v>
+      </c>
+      <c r="F415" t="n">
+        <v>8308</v>
+      </c>
+      <c r="G415" t="inlineStr"/>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>2025-03-04 16:45:09</t>
+        </is>
+      </c>
+      <c r="B416" t="n">
+        <v>132486</v>
+      </c>
+      <c r="C416" t="n">
+        <v>0</v>
+      </c>
+      <c r="D416" t="n">
+        <v>164</v>
+      </c>
+      <c r="E416" t="n">
+        <v>0</v>
+      </c>
+      <c r="F416" t="n">
+        <v>8481</v>
+      </c>
+      <c r="G416" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Removed uneeded print statements and checked that the bigger df works
</commit_message>
<xml_diff>
--- a/LOC tracking outputs/code_metrics.xlsx
+++ b/LOC tracking outputs/code_metrics.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G416"/>
+  <dimension ref="A1:G435"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10058,6 +10058,443 @@
       </c>
       <c r="G416" t="inlineStr"/>
     </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>2025-02-21 08:38:45</t>
+        </is>
+      </c>
+      <c r="B417" t="n">
+        <v>123576</v>
+      </c>
+      <c r="C417" t="n">
+        <v>0</v>
+      </c>
+      <c r="D417" t="n">
+        <v>123</v>
+      </c>
+      <c r="E417" t="n">
+        <v>0</v>
+      </c>
+      <c r="F417" t="n">
+        <v>6887</v>
+      </c>
+      <c r="G417" t="inlineStr"/>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>2025-02-21 08:38:45</t>
+        </is>
+      </c>
+      <c r="B418" t="n">
+        <v>124032</v>
+      </c>
+      <c r="C418" t="n">
+        <v>0</v>
+      </c>
+      <c r="D418" t="n">
+        <v>123</v>
+      </c>
+      <c r="E418" t="n">
+        <v>0</v>
+      </c>
+      <c r="F418" t="n">
+        <v>6932</v>
+      </c>
+      <c r="G418" t="inlineStr"/>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>2025-02-21 08:38:45</t>
+        </is>
+      </c>
+      <c r="B419" t="n">
+        <v>124902</v>
+      </c>
+      <c r="C419" t="n">
+        <v>0</v>
+      </c>
+      <c r="D419" t="n">
+        <v>123</v>
+      </c>
+      <c r="E419" t="n">
+        <v>0</v>
+      </c>
+      <c r="F419" t="n">
+        <v>6988</v>
+      </c>
+      <c r="G419" t="inlineStr"/>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>2025-02-21 08:38:45</t>
+        </is>
+      </c>
+      <c r="B420" t="n">
+        <v>125077</v>
+      </c>
+      <c r="C420" t="n">
+        <v>0</v>
+      </c>
+      <c r="D420" t="n">
+        <v>123</v>
+      </c>
+      <c r="E420" t="n">
+        <v>0</v>
+      </c>
+      <c r="F420" t="n">
+        <v>7023</v>
+      </c>
+      <c r="G420" t="inlineStr"/>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>2025-02-21 08:38:45</t>
+        </is>
+      </c>
+      <c r="B421" t="n">
+        <v>125037</v>
+      </c>
+      <c r="C421" t="n">
+        <v>0</v>
+      </c>
+      <c r="D421" t="n">
+        <v>123</v>
+      </c>
+      <c r="E421" t="n">
+        <v>0</v>
+      </c>
+      <c r="F421" t="n">
+        <v>7015</v>
+      </c>
+      <c r="G421" t="inlineStr"/>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>2025-04-01 10:56:06</t>
+        </is>
+      </c>
+      <c r="B422" t="n">
+        <v>128311</v>
+      </c>
+      <c r="C422" t="n">
+        <v>0</v>
+      </c>
+      <c r="D422" t="n">
+        <v>164</v>
+      </c>
+      <c r="E422" t="n">
+        <v>0</v>
+      </c>
+      <c r="F422" t="n">
+        <v>7667</v>
+      </c>
+      <c r="G422" t="inlineStr"/>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>2025-04-01 10:56:06</t>
+        </is>
+      </c>
+      <c r="B423" t="n">
+        <v>128327</v>
+      </c>
+      <c r="C423" t="n">
+        <v>0</v>
+      </c>
+      <c r="D423" t="n">
+        <v>164</v>
+      </c>
+      <c r="E423" t="n">
+        <v>0</v>
+      </c>
+      <c r="F423" t="n">
+        <v>7675</v>
+      </c>
+      <c r="G423" t="inlineStr"/>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>2025-04-01 10:56:06</t>
+        </is>
+      </c>
+      <c r="B424" t="n">
+        <v>131661</v>
+      </c>
+      <c r="C424" t="n">
+        <v>0</v>
+      </c>
+      <c r="D424" t="n">
+        <v>164</v>
+      </c>
+      <c r="E424" t="n">
+        <v>0</v>
+      </c>
+      <c r="F424" t="n">
+        <v>8308</v>
+      </c>
+      <c r="G424" t="inlineStr"/>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>2025-04-01 10:56:06</t>
+        </is>
+      </c>
+      <c r="B425" t="n">
+        <v>132486</v>
+      </c>
+      <c r="C425" t="n">
+        <v>0</v>
+      </c>
+      <c r="D425" t="n">
+        <v>164</v>
+      </c>
+      <c r="E425" t="n">
+        <v>0</v>
+      </c>
+      <c r="F425" t="n">
+        <v>8481</v>
+      </c>
+      <c r="G425" t="inlineStr"/>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>2025-02-21 08:38:45</t>
+        </is>
+      </c>
+      <c r="B426" t="n">
+        <v>123576</v>
+      </c>
+      <c r="C426" t="n">
+        <v>0</v>
+      </c>
+      <c r="D426" t="n">
+        <v>123</v>
+      </c>
+      <c r="E426" t="n">
+        <v>0</v>
+      </c>
+      <c r="F426" t="n">
+        <v>6887</v>
+      </c>
+      <c r="G426" t="inlineStr"/>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>2025-02-21 08:38:45</t>
+        </is>
+      </c>
+      <c r="B427" t="n">
+        <v>124032</v>
+      </c>
+      <c r="C427" t="n">
+        <v>0</v>
+      </c>
+      <c r="D427" t="n">
+        <v>123</v>
+      </c>
+      <c r="E427" t="n">
+        <v>0</v>
+      </c>
+      <c r="F427" t="n">
+        <v>6932</v>
+      </c>
+      <c r="G427" t="inlineStr"/>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>2025-02-21 08:38:45</t>
+        </is>
+      </c>
+      <c r="B428" t="n">
+        <v>124902</v>
+      </c>
+      <c r="C428" t="n">
+        <v>0</v>
+      </c>
+      <c r="D428" t="n">
+        <v>123</v>
+      </c>
+      <c r="E428" t="n">
+        <v>0</v>
+      </c>
+      <c r="F428" t="n">
+        <v>6988</v>
+      </c>
+      <c r="G428" t="inlineStr"/>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>2025-02-21 08:38:45</t>
+        </is>
+      </c>
+      <c r="B429" t="n">
+        <v>125077</v>
+      </c>
+      <c r="C429" t="n">
+        <v>0</v>
+      </c>
+      <c r="D429" t="n">
+        <v>123</v>
+      </c>
+      <c r="E429" t="n">
+        <v>0</v>
+      </c>
+      <c r="F429" t="n">
+        <v>7023</v>
+      </c>
+      <c r="G429" t="inlineStr"/>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>2025-02-21 08:38:45</t>
+        </is>
+      </c>
+      <c r="B430" t="n">
+        <v>125037</v>
+      </c>
+      <c r="C430" t="n">
+        <v>0</v>
+      </c>
+      <c r="D430" t="n">
+        <v>123</v>
+      </c>
+      <c r="E430" t="n">
+        <v>0</v>
+      </c>
+      <c r="F430" t="n">
+        <v>7015</v>
+      </c>
+      <c r="G430" t="inlineStr"/>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>2025-04-01 10:56:06</t>
+        </is>
+      </c>
+      <c r="B431" t="n">
+        <v>128311</v>
+      </c>
+      <c r="C431" t="n">
+        <v>0</v>
+      </c>
+      <c r="D431" t="n">
+        <v>164</v>
+      </c>
+      <c r="E431" t="n">
+        <v>0</v>
+      </c>
+      <c r="F431" t="n">
+        <v>7667</v>
+      </c>
+      <c r="G431" t="inlineStr"/>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>2025-04-01 10:56:06</t>
+        </is>
+      </c>
+      <c r="B432" t="n">
+        <v>128327</v>
+      </c>
+      <c r="C432" t="n">
+        <v>0</v>
+      </c>
+      <c r="D432" t="n">
+        <v>164</v>
+      </c>
+      <c r="E432" t="n">
+        <v>0</v>
+      </c>
+      <c r="F432" t="n">
+        <v>7675</v>
+      </c>
+      <c r="G432" t="inlineStr"/>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>2025-04-01 10:56:06</t>
+        </is>
+      </c>
+      <c r="B433" t="n">
+        <v>131661</v>
+      </c>
+      <c r="C433" t="n">
+        <v>0</v>
+      </c>
+      <c r="D433" t="n">
+        <v>164</v>
+      </c>
+      <c r="E433" t="n">
+        <v>0</v>
+      </c>
+      <c r="F433" t="n">
+        <v>8308</v>
+      </c>
+      <c r="G433" t="inlineStr"/>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>2025-04-01 10:56:06</t>
+        </is>
+      </c>
+      <c r="B434" t="n">
+        <v>132486</v>
+      </c>
+      <c r="C434" t="n">
+        <v>0</v>
+      </c>
+      <c r="D434" t="n">
+        <v>164</v>
+      </c>
+      <c r="E434" t="n">
+        <v>0</v>
+      </c>
+      <c r="F434" t="n">
+        <v>8481</v>
+      </c>
+      <c r="G434" t="inlineStr"/>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>2025-04-17 09:41:50</t>
+        </is>
+      </c>
+      <c r="B435" t="n">
+        <v>375990</v>
+      </c>
+      <c r="C435" t="n">
+        <v>0</v>
+      </c>
+      <c r="D435" t="n">
+        <v>164</v>
+      </c>
+      <c r="E435" t="n">
+        <v>0</v>
+      </c>
+      <c r="F435" t="n">
+        <v>11145</v>
+      </c>
+      <c r="G435" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cleaning head after count
</commit_message>
<xml_diff>
--- a/LOC tracking outputs/code_metrics.xlsx
+++ b/LOC tracking outputs/code_metrics.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G435"/>
+  <dimension ref="A1:G445"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10495,6 +10495,236 @@
       </c>
       <c r="G435" t="inlineStr"/>
     </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>2025-02-21 08:38:45</t>
+        </is>
+      </c>
+      <c r="B436" t="n">
+        <v>124032</v>
+      </c>
+      <c r="C436" t="n">
+        <v>0</v>
+      </c>
+      <c r="D436" t="n">
+        <v>123</v>
+      </c>
+      <c r="E436" t="n">
+        <v>0</v>
+      </c>
+      <c r="F436" t="n">
+        <v>6932</v>
+      </c>
+      <c r="G436" t="inlineStr"/>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>2025-02-21 08:38:45</t>
+        </is>
+      </c>
+      <c r="B437" t="n">
+        <v>124902</v>
+      </c>
+      <c r="C437" t="n">
+        <v>0</v>
+      </c>
+      <c r="D437" t="n">
+        <v>123</v>
+      </c>
+      <c r="E437" t="n">
+        <v>0</v>
+      </c>
+      <c r="F437" t="n">
+        <v>6988</v>
+      </c>
+      <c r="G437" t="inlineStr"/>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>2025-02-21 08:38:45</t>
+        </is>
+      </c>
+      <c r="B438" t="n">
+        <v>125077</v>
+      </c>
+      <c r="C438" t="n">
+        <v>0</v>
+      </c>
+      <c r="D438" t="n">
+        <v>123</v>
+      </c>
+      <c r="E438" t="n">
+        <v>0</v>
+      </c>
+      <c r="F438" t="n">
+        <v>7023</v>
+      </c>
+      <c r="G438" t="inlineStr"/>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>2025-02-21 08:38:45</t>
+        </is>
+      </c>
+      <c r="B439" t="n">
+        <v>125037</v>
+      </c>
+      <c r="C439" t="n">
+        <v>0</v>
+      </c>
+      <c r="D439" t="n">
+        <v>123</v>
+      </c>
+      <c r="E439" t="n">
+        <v>0</v>
+      </c>
+      <c r="F439" t="n">
+        <v>7015</v>
+      </c>
+      <c r="G439" t="inlineStr"/>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>2025-04-01 10:56:06</t>
+        </is>
+      </c>
+      <c r="B440" t="n">
+        <v>128311</v>
+      </c>
+      <c r="C440" t="n">
+        <v>0</v>
+      </c>
+      <c r="D440" t="n">
+        <v>164</v>
+      </c>
+      <c r="E440" t="n">
+        <v>0</v>
+      </c>
+      <c r="F440" t="n">
+        <v>7667</v>
+      </c>
+      <c r="G440" t="inlineStr"/>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>2025-04-01 10:56:06</t>
+        </is>
+      </c>
+      <c r="B441" t="n">
+        <v>128327</v>
+      </c>
+      <c r="C441" t="n">
+        <v>0</v>
+      </c>
+      <c r="D441" t="n">
+        <v>164</v>
+      </c>
+      <c r="E441" t="n">
+        <v>0</v>
+      </c>
+      <c r="F441" t="n">
+        <v>7675</v>
+      </c>
+      <c r="G441" t="inlineStr"/>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>2025-04-01 10:56:06</t>
+        </is>
+      </c>
+      <c r="B442" t="n">
+        <v>131661</v>
+      </c>
+      <c r="C442" t="n">
+        <v>0</v>
+      </c>
+      <c r="D442" t="n">
+        <v>164</v>
+      </c>
+      <c r="E442" t="n">
+        <v>0</v>
+      </c>
+      <c r="F442" t="n">
+        <v>8308</v>
+      </c>
+      <c r="G442" t="inlineStr"/>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>2025-04-01 10:56:06</t>
+        </is>
+      </c>
+      <c r="B443" t="n">
+        <v>132486</v>
+      </c>
+      <c r="C443" t="n">
+        <v>0</v>
+      </c>
+      <c r="D443" t="n">
+        <v>164</v>
+      </c>
+      <c r="E443" t="n">
+        <v>0</v>
+      </c>
+      <c r="F443" t="n">
+        <v>8481</v>
+      </c>
+      <c r="G443" t="inlineStr"/>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>2025-04-17 09:41:50</t>
+        </is>
+      </c>
+      <c r="B444" t="n">
+        <v>375990</v>
+      </c>
+      <c r="C444" t="n">
+        <v>0</v>
+      </c>
+      <c r="D444" t="n">
+        <v>164</v>
+      </c>
+      <c r="E444" t="n">
+        <v>0</v>
+      </c>
+      <c r="F444" t="n">
+        <v>11145</v>
+      </c>
+      <c r="G444" t="inlineStr"/>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>2025-04-17 17:19:29</t>
+        </is>
+      </c>
+      <c r="B445" t="n">
+        <v>380717</v>
+      </c>
+      <c r="C445" t="n">
+        <v>0</v>
+      </c>
+      <c r="D445" t="n">
+        <v>164</v>
+      </c>
+      <c r="E445" t="n">
+        <v>0</v>
+      </c>
+      <c r="F445" t="n">
+        <v>11536</v>
+      </c>
+      <c r="G445" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>